<commit_message>
Atualização automática: pagamentos (09/07/2026 23:47)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -22,16 +22,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -50,21 +47,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -435,57 +423,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>numero_contrato</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>ug_executora</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ug_responsavel</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ug_fiscalizadora</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>valor_total_contrato</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>valor_a_empenhar</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>valor_empenhado</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>valor_liquidado</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>saldo_a_faturar</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>fornecedor</t>
         </is>
@@ -553,92 +541,92 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>modulo</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>referencia</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>numero_recibo</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>numero_nota_fiscal</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>empenho</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>observacao</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>vencimento</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>valor_nfs</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ordem_pagamento</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>faturado</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>tipo_registro</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>empenho_saldo</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>empenho_valor_empenhado</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>empenho_responsavel</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>empenho_justificativa</t>
         </is>
@@ -661,7 +649,7 @@
       <c r="D2" t="n">
         <v>594</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="1" t="n">
         <v>45740</v>
       </c>
       <c r="F2" t="inlineStr">
@@ -670,7 +658,7 @@
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="1" t="n">
         <v>45778</v>
       </c>
       <c r="I2" t="n">
@@ -719,7 +707,7 @@
       <c r="D3" t="n">
         <v>620</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="1" t="n">
         <v>45775</v>
       </c>
       <c r="F3" t="inlineStr">
@@ -728,7 +716,7 @@
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="1" t="n">
         <v>45806</v>
       </c>
       <c r="I3" t="n">
@@ -777,7 +765,7 @@
       <c r="D4" t="n">
         <v>634</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="1" t="n">
         <v>45799</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -786,7 +774,7 @@
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="1" t="n">
         <v>45844</v>
       </c>
       <c r="I4" t="n">
@@ -835,7 +823,7 @@
       <c r="D5" t="n">
         <v>660</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -844,7 +832,7 @@
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="I5" t="n">
@@ -893,7 +881,7 @@
       <c r="D6" t="n">
         <v>661</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -905,7 +893,7 @@
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="I6" t="n">
@@ -956,7 +944,7 @@
       <c r="D7" t="n">
         <v>688</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="1" t="n">
         <v>45901</v>
       </c>
       <c r="F7" t="inlineStr">
@@ -965,7 +953,7 @@
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="1" t="n">
         <v>45938</v>
       </c>
       <c r="I7" t="n">
@@ -1014,7 +1002,7 @@
       <c r="D8" t="n">
         <v>696</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="1" t="n">
         <v>45923</v>
       </c>
       <c r="F8" t="inlineStr">
@@ -1023,7 +1011,7 @@
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="1" t="n">
         <v>45938</v>
       </c>
       <c r="I8" t="n">
@@ -1072,7 +1060,7 @@
       <c r="D9" t="n">
         <v>704</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="1" t="n">
         <v>45957</v>
       </c>
       <c r="F9" t="inlineStr">
@@ -1082,7 +1070,7 @@
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="1" t="n">
         <v>46003</v>
       </c>
       <c r="I9" t="n">
@@ -1127,7 +1115,7 @@
       <c r="D10" t="n">
         <v>705</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="1" t="n">
         <v>45972</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -1136,7 +1124,7 @@
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="1" t="n">
         <v>46016</v>
       </c>
       <c r="I10" t="n">
@@ -1185,7 +1173,7 @@
       <c r="D11" t="n">
         <v>728</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="1" t="n">
         <v>46008</v>
       </c>
       <c r="F11" t="inlineStr">
@@ -1194,7 +1182,7 @@
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="1" t="n">
         <v>46040</v>
       </c>
       <c r="I11" t="n">
@@ -1243,7 +1231,7 @@
       <c r="D12" t="n">
         <v>278</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="1" t="n">
         <v>46042</v>
       </c>
       <c r="F12" t="inlineStr">
@@ -1252,7 +1240,7 @@
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" s="2" t="n">
+      <c r="H12" s="1" t="n">
         <v>46074</v>
       </c>
       <c r="I12" t="n">
@@ -1299,7 +1287,7 @@
       <c r="D13" t="n">
         <v>10</v>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="1" t="n">
         <v>46078</v>
       </c>
       <c r="F13" t="inlineStr">
@@ -1308,7 +1296,7 @@
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" s="2" t="n">
+      <c r="H13" s="1" t="n">
         <v>46106</v>
       </c>
       <c r="I13" t="n">
@@ -1353,7 +1341,7 @@
       <c r="D14" t="n">
         <v>15</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="1" t="n">
         <v>46094</v>
       </c>
       <c r="F14" t="inlineStr">
@@ -1362,7 +1350,7 @@
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" s="2" t="n">
+      <c r="H14" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="I14" t="n">
@@ -1409,7 +1397,7 @@
       <c r="D15" t="n">
         <v>28</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="F15" t="inlineStr">
@@ -1418,7 +1406,7 @@
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" s="2" t="n">
+      <c r="H15" s="1" t="n">
         <v>46164</v>
       </c>
       <c r="I15" t="n">
@@ -1465,7 +1453,7 @@
       <c r="D16" t="n">
         <v>33</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="1" t="n">
         <v>46156</v>
       </c>
       <c r="F16" t="inlineStr">
@@ -1474,7 +1462,7 @@
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" s="2" t="n">
+      <c r="H16" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="I16" t="n">
@@ -1521,7 +1509,7 @@
       <c r="D17" t="n">
         <v>29</v>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E17" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="F17" t="inlineStr">
@@ -1530,7 +1518,7 @@
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" s="2" t="n">
+      <c r="H17" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="I17" t="n">
@@ -1577,7 +1565,7 @@
       <c r="D18" t="n">
         <v>40</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="1" t="n">
         <v>46156</v>
       </c>
       <c r="F18" t="inlineStr">
@@ -1586,7 +1574,7 @@
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" s="2" t="n">
+      <c r="H18" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="I18" t="n">
@@ -1633,7 +1621,7 @@
       <c r="D19" t="n">
         <v>402</v>
       </c>
-      <c r="E19" s="2" t="n">
+      <c r="E19" s="1" t="n">
         <v>45791</v>
       </c>
       <c r="F19" t="inlineStr">
@@ -1642,7 +1630,7 @@
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="2" t="n">
+      <c r="H19" s="1" t="n">
         <v>45834</v>
       </c>
       <c r="I19" t="n">
@@ -1689,7 +1677,7 @@
       <c r="D20" t="n">
         <v>447</v>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="1" t="n">
         <v>45814</v>
       </c>
       <c r="F20" t="inlineStr">
@@ -1698,7 +1686,7 @@
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" s="2" t="n">
+      <c r="H20" s="1" t="n">
         <v>45955</v>
       </c>
       <c r="I20" t="n">
@@ -1749,7 +1737,7 @@
       <c r="D21" t="n">
         <v>529</v>
       </c>
-      <c r="E21" s="2" t="n">
+      <c r="E21" s="1" t="n">
         <v>45853</v>
       </c>
       <c r="F21" t="inlineStr">
@@ -1758,7 +1746,7 @@
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" s="2" t="n">
+      <c r="H21" s="1" t="n">
         <v>45939</v>
       </c>
       <c r="I21" t="n">
@@ -1809,7 +1797,7 @@
       <c r="D22" t="n">
         <v>691</v>
       </c>
-      <c r="E22" s="2" t="n">
+      <c r="E22" s="1" t="n">
         <v>45910</v>
       </c>
       <c r="F22" t="inlineStr">
@@ -1818,7 +1806,7 @@
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" s="2" t="n">
+      <c r="H22" s="1" t="n">
         <v>45941</v>
       </c>
       <c r="I22" t="n">
@@ -1867,7 +1855,7 @@
       <c r="D23" t="n">
         <v>677</v>
       </c>
-      <c r="E23" s="2" t="n">
+      <c r="E23" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="F23" t="inlineStr">
@@ -1876,7 +1864,7 @@
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" s="2" t="n">
+      <c r="H23" s="1" t="n">
         <v>45935</v>
       </c>
       <c r="I23" t="n">
@@ -1923,7 +1911,7 @@
       <c r="D24" t="n">
         <v>278</v>
       </c>
-      <c r="E24" s="2" t="n">
+      <c r="E24" s="1" t="n">
         <v>46008</v>
       </c>
       <c r="F24" t="inlineStr">
@@ -1932,7 +1920,7 @@
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" s="2" t="n">
+      <c r="H24" s="1" t="n">
         <v>46066</v>
       </c>
       <c r="I24" t="n">
@@ -1981,7 +1969,7 @@
       <c r="D25" t="n">
         <v>748</v>
       </c>
-      <c r="E25" s="2" t="n">
+      <c r="E25" s="1" t="n">
         <v>45930</v>
       </c>
       <c r="F25" t="inlineStr">
@@ -1990,7 +1978,7 @@
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" s="2" t="n">
+      <c r="H25" s="1" t="n">
         <v>45935</v>
       </c>
       <c r="I25" t="n">
@@ -2037,7 +2025,7 @@
       <c r="D26" t="n">
         <v>822</v>
       </c>
-      <c r="E26" s="2" t="n">
+      <c r="E26" s="1" t="n">
         <v>45968</v>
       </c>
       <c r="F26" t="inlineStr">
@@ -2046,7 +2034,7 @@
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" s="2" t="n">
+      <c r="H26" s="1" t="n">
         <v>45935</v>
       </c>
       <c r="I26" t="n">
@@ -2093,7 +2081,7 @@
       <c r="D27" t="n">
         <v>360</v>
       </c>
-      <c r="E27" s="2" t="n">
+      <c r="E27" s="1" t="n">
         <v>46043</v>
       </c>
       <c r="F27" t="inlineStr">
@@ -2102,7 +2090,7 @@
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" s="2" t="n">
+      <c r="H27" s="1" t="n">
         <v>46075</v>
       </c>
       <c r="I27" t="n">
@@ -2223,7 +2211,7 @@
       <c r="D30" t="n">
         <v>1465</v>
       </c>
-      <c r="E30" s="2" t="n">
+      <c r="E30" s="1" t="n">
         <v>46104</v>
       </c>
       <c r="F30" t="inlineStr">
@@ -2232,7 +2220,7 @@
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" s="2" t="n">
+      <c r="H30" s="1" t="n">
         <v>46106</v>
       </c>
       <c r="I30" t="n">
@@ -2275,27 +2263,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>numero_empenho</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>valor_empenhado</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>saldo</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>responsavel</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>justificativa</t>
         </is>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (10/07/2026 10:10)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -22,13 +22,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +42,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,12 +50,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -423,57 +435,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>numero_contrato</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ug_executora</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>ug_responsavel</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ug_fiscalizadora</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>valor_total_contrato</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>valor_a_empenhar</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>valor_empenhado</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>valor_liquidado</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>saldo_a_faturar</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>fornecedor</t>
         </is>
@@ -541,92 +553,92 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>modulo</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>referencia</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>numero_recibo</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>numero_nota_fiscal</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>empenho</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>observacao</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>vencimento</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>valor_nfs</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>ordem_pagamento</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>faturado</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>tipo_registro</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>empenho_saldo</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>empenho_valor_empenhado</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>empenho_responsavel</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>empenho_justificativa</t>
         </is>
@@ -649,7 +661,7 @@
       <c r="D2" t="n">
         <v>594</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="2" t="n">
         <v>45740</v>
       </c>
       <c r="F2" t="inlineStr">
@@ -658,7 +670,7 @@
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="1" t="n">
+      <c r="H2" s="2" t="n">
         <v>45778</v>
       </c>
       <c r="I2" t="n">
@@ -707,7 +719,7 @@
       <c r="D3" t="n">
         <v>620</v>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="2" t="n">
         <v>45775</v>
       </c>
       <c r="F3" t="inlineStr">
@@ -716,7 +728,7 @@
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="1" t="n">
+      <c r="H3" s="2" t="n">
         <v>45806</v>
       </c>
       <c r="I3" t="n">
@@ -765,7 +777,7 @@
       <c r="D4" t="n">
         <v>634</v>
       </c>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="2" t="n">
         <v>45799</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -774,7 +786,7 @@
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" s="1" t="n">
+      <c r="H4" s="2" t="n">
         <v>45844</v>
       </c>
       <c r="I4" t="n">
@@ -823,7 +835,7 @@
       <c r="D5" t="n">
         <v>660</v>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E5" s="2" t="n">
         <v>45856</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -832,7 +844,7 @@
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" s="1" t="n">
+      <c r="H5" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="I5" t="n">
@@ -881,7 +893,7 @@
       <c r="D6" t="n">
         <v>661</v>
       </c>
-      <c r="E6" s="1" t="n">
+      <c r="E6" s="2" t="n">
         <v>45856</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -893,7 +905,7 @@
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" s="1" t="n">
+      <c r="H6" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="I6" t="n">
@@ -944,7 +956,7 @@
       <c r="D7" t="n">
         <v>688</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>45901</v>
       </c>
       <c r="F7" t="inlineStr">
@@ -953,7 +965,7 @@
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" s="1" t="n">
+      <c r="H7" s="2" t="n">
         <v>45938</v>
       </c>
       <c r="I7" t="n">
@@ -1002,7 +1014,7 @@
       <c r="D8" t="n">
         <v>696</v>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="2" t="n">
         <v>45923</v>
       </c>
       <c r="F8" t="inlineStr">
@@ -1011,7 +1023,7 @@
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" s="1" t="n">
+      <c r="H8" s="2" t="n">
         <v>45938</v>
       </c>
       <c r="I8" t="n">
@@ -1060,7 +1072,7 @@
       <c r="D9" t="n">
         <v>704</v>
       </c>
-      <c r="E9" s="1" t="n">
+      <c r="E9" s="2" t="n">
         <v>45957</v>
       </c>
       <c r="F9" t="inlineStr">
@@ -1070,7 +1082,7 @@
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" s="1" t="n">
+      <c r="H9" s="2" t="n">
         <v>46003</v>
       </c>
       <c r="I9" t="n">
@@ -1115,7 +1127,7 @@
       <c r="D10" t="n">
         <v>705</v>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="2" t="n">
         <v>45972</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -1124,7 +1136,7 @@
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" s="1" t="n">
+      <c r="H10" s="2" t="n">
         <v>46016</v>
       </c>
       <c r="I10" t="n">
@@ -1173,7 +1185,7 @@
       <c r="D11" t="n">
         <v>728</v>
       </c>
-      <c r="E11" s="1" t="n">
+      <c r="E11" s="2" t="n">
         <v>46008</v>
       </c>
       <c r="F11" t="inlineStr">
@@ -1182,7 +1194,7 @@
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" s="1" t="n">
+      <c r="H11" s="2" t="n">
         <v>46040</v>
       </c>
       <c r="I11" t="n">
@@ -1231,7 +1243,7 @@
       <c r="D12" t="n">
         <v>278</v>
       </c>
-      <c r="E12" s="1" t="n">
+      <c r="E12" s="2" t="n">
         <v>46042</v>
       </c>
       <c r="F12" t="inlineStr">
@@ -1240,7 +1252,7 @@
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" s="1" t="n">
+      <c r="H12" s="2" t="n">
         <v>46074</v>
       </c>
       <c r="I12" t="n">
@@ -1287,7 +1299,7 @@
       <c r="D13" t="n">
         <v>10</v>
       </c>
-      <c r="E13" s="1" t="n">
+      <c r="E13" s="2" t="n">
         <v>46078</v>
       </c>
       <c r="F13" t="inlineStr">
@@ -1296,7 +1308,7 @@
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" s="1" t="n">
+      <c r="H13" s="2" t="n">
         <v>46106</v>
       </c>
       <c r="I13" t="n">
@@ -1341,7 +1353,7 @@
       <c r="D14" t="n">
         <v>15</v>
       </c>
-      <c r="E14" s="1" t="n">
+      <c r="E14" s="2" t="n">
         <v>46094</v>
       </c>
       <c r="F14" t="inlineStr">
@@ -1350,7 +1362,7 @@
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" s="1" t="n">
+      <c r="H14" s="2" t="n">
         <v>46128</v>
       </c>
       <c r="I14" t="n">
@@ -1397,7 +1409,7 @@
       <c r="D15" t="n">
         <v>28</v>
       </c>
-      <c r="E15" s="1" t="n">
+      <c r="E15" s="2" t="n">
         <v>46128</v>
       </c>
       <c r="F15" t="inlineStr">
@@ -1406,7 +1418,7 @@
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" s="1" t="n">
+      <c r="H15" s="2" t="n">
         <v>46164</v>
       </c>
       <c r="I15" t="n">
@@ -1453,7 +1465,7 @@
       <c r="D16" t="n">
         <v>33</v>
       </c>
-      <c r="E16" s="1" t="n">
+      <c r="E16" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="F16" t="inlineStr">
@@ -1462,7 +1474,7 @@
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" s="1" t="n">
+      <c r="H16" s="2" t="n">
         <v>46191</v>
       </c>
       <c r="I16" t="n">
@@ -1509,7 +1521,7 @@
       <c r="D17" t="n">
         <v>29</v>
       </c>
-      <c r="E17" s="1" t="n">
+      <c r="E17" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="F17" t="inlineStr">
@@ -1518,7 +1530,7 @@
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" s="1" t="n">
+      <c r="H17" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="I17" t="n">
@@ -1565,7 +1577,7 @@
       <c r="D18" t="n">
         <v>40</v>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="F18" t="inlineStr">
@@ -1574,7 +1586,7 @@
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" s="1" t="n">
+      <c r="H18" s="2" t="n">
         <v>46191</v>
       </c>
       <c r="I18" t="n">
@@ -1621,7 +1633,7 @@
       <c r="D19" t="n">
         <v>402</v>
       </c>
-      <c r="E19" s="1" t="n">
+      <c r="E19" s="2" t="n">
         <v>45791</v>
       </c>
       <c r="F19" t="inlineStr">
@@ -1630,7 +1642,7 @@
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="1" t="n">
+      <c r="H19" s="2" t="n">
         <v>45834</v>
       </c>
       <c r="I19" t="n">
@@ -1677,7 +1689,7 @@
       <c r="D20" t="n">
         <v>447</v>
       </c>
-      <c r="E20" s="1" t="n">
+      <c r="E20" s="2" t="n">
         <v>45814</v>
       </c>
       <c r="F20" t="inlineStr">
@@ -1686,7 +1698,7 @@
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" s="1" t="n">
+      <c r="H20" s="2" t="n">
         <v>45955</v>
       </c>
       <c r="I20" t="n">
@@ -1737,7 +1749,7 @@
       <c r="D21" t="n">
         <v>529</v>
       </c>
-      <c r="E21" s="1" t="n">
+      <c r="E21" s="2" t="n">
         <v>45853</v>
       </c>
       <c r="F21" t="inlineStr">
@@ -1746,7 +1758,7 @@
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" s="1" t="n">
+      <c r="H21" s="2" t="n">
         <v>45939</v>
       </c>
       <c r="I21" t="n">
@@ -1797,7 +1809,7 @@
       <c r="D22" t="n">
         <v>691</v>
       </c>
-      <c r="E22" s="1" t="n">
+      <c r="E22" s="2" t="n">
         <v>45910</v>
       </c>
       <c r="F22" t="inlineStr">
@@ -1806,7 +1818,7 @@
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" s="1" t="n">
+      <c r="H22" s="2" t="n">
         <v>45941</v>
       </c>
       <c r="I22" t="n">
@@ -1855,7 +1867,7 @@
       <c r="D23" t="n">
         <v>677</v>
       </c>
-      <c r="E23" s="1" t="n">
+      <c r="E23" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="F23" t="inlineStr">
@@ -1864,7 +1876,7 @@
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" s="1" t="n">
+      <c r="H23" s="2" t="n">
         <v>45935</v>
       </c>
       <c r="I23" t="n">
@@ -1911,7 +1923,7 @@
       <c r="D24" t="n">
         <v>278</v>
       </c>
-      <c r="E24" s="1" t="n">
+      <c r="E24" s="2" t="n">
         <v>46008</v>
       </c>
       <c r="F24" t="inlineStr">
@@ -1920,7 +1932,7 @@
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" s="1" t="n">
+      <c r="H24" s="2" t="n">
         <v>46066</v>
       </c>
       <c r="I24" t="n">
@@ -1969,7 +1981,7 @@
       <c r="D25" t="n">
         <v>748</v>
       </c>
-      <c r="E25" s="1" t="n">
+      <c r="E25" s="2" t="n">
         <v>45930</v>
       </c>
       <c r="F25" t="inlineStr">
@@ -1978,7 +1990,7 @@
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" s="1" t="n">
+      <c r="H25" s="2" t="n">
         <v>45935</v>
       </c>
       <c r="I25" t="n">
@@ -2025,7 +2037,7 @@
       <c r="D26" t="n">
         <v>822</v>
       </c>
-      <c r="E26" s="1" t="n">
+      <c r="E26" s="2" t="n">
         <v>45968</v>
       </c>
       <c r="F26" t="inlineStr">
@@ -2034,7 +2046,7 @@
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" s="1" t="n">
+      <c r="H26" s="2" t="n">
         <v>45935</v>
       </c>
       <c r="I26" t="n">
@@ -2081,7 +2093,7 @@
       <c r="D27" t="n">
         <v>360</v>
       </c>
-      <c r="E27" s="1" t="n">
+      <c r="E27" s="2" t="n">
         <v>46043</v>
       </c>
       <c r="F27" t="inlineStr">
@@ -2090,7 +2102,7 @@
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" s="1" t="n">
+      <c r="H27" s="2" t="n">
         <v>46075</v>
       </c>
       <c r="I27" t="n">
@@ -2211,7 +2223,7 @@
       <c r="D30" t="n">
         <v>1465</v>
       </c>
-      <c r="E30" s="1" t="n">
+      <c r="E30" s="2" t="n">
         <v>46104</v>
       </c>
       <c r="F30" t="inlineStr">
@@ -2220,7 +2232,7 @@
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" s="1" t="n">
+      <c r="H30" s="2" t="n">
         <v>46106</v>
       </c>
       <c r="I30" t="n">
@@ -2263,27 +2275,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>numero_empenho</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>valor_empenhado</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>saldo</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>responsavel</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>justificativa</t>
         </is>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (10/07/2026 17:31)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -22,16 +22,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -50,21 +47,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -435,57 +423,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>numero_contrato</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>ug_executora</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ug_responsavel</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ug_fiscalizadora</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>valor_total_contrato</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>valor_a_empenhar</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>valor_empenhado</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>valor_liquidado</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>saldo_a_faturar</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>fornecedor</t>
         </is>
@@ -553,92 +541,92 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>modulo</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>referencia</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>numero_recibo</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>numero_nota_fiscal</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>empenho</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>observacao</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>vencimento</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>valor_nfs</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ordem_pagamento</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>faturado</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>tipo_registro</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>empenho_saldo</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>empenho_valor_empenhado</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>empenho_responsavel</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>empenho_justificativa</t>
         </is>
@@ -661,7 +649,7 @@
       <c r="D2" t="n">
         <v>594</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="1" t="n">
         <v>45740</v>
       </c>
       <c r="F2" t="inlineStr">
@@ -670,7 +658,7 @@
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="1" t="n">
         <v>45778</v>
       </c>
       <c r="I2" t="n">
@@ -719,7 +707,7 @@
       <c r="D3" t="n">
         <v>620</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="1" t="n">
         <v>45775</v>
       </c>
       <c r="F3" t="inlineStr">
@@ -728,7 +716,7 @@
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="1" t="n">
         <v>45806</v>
       </c>
       <c r="I3" t="n">
@@ -777,7 +765,7 @@
       <c r="D4" t="n">
         <v>634</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="1" t="n">
         <v>45799</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -786,7 +774,7 @@
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="1" t="n">
         <v>45844</v>
       </c>
       <c r="I4" t="n">
@@ -835,7 +823,7 @@
       <c r="D5" t="n">
         <v>660</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -844,7 +832,7 @@
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="I5" t="n">
@@ -893,7 +881,7 @@
       <c r="D6" t="n">
         <v>661</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -905,7 +893,7 @@
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="I6" t="n">
@@ -956,7 +944,7 @@
       <c r="D7" t="n">
         <v>688</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="1" t="n">
         <v>45901</v>
       </c>
       <c r="F7" t="inlineStr">
@@ -965,7 +953,7 @@
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="1" t="n">
         <v>45938</v>
       </c>
       <c r="I7" t="n">
@@ -1014,7 +1002,7 @@
       <c r="D8" t="n">
         <v>696</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="1" t="n">
         <v>45923</v>
       </c>
       <c r="F8" t="inlineStr">
@@ -1023,7 +1011,7 @@
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="1" t="n">
         <v>45938</v>
       </c>
       <c r="I8" t="n">
@@ -1072,7 +1060,7 @@
       <c r="D9" t="n">
         <v>704</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="1" t="n">
         <v>45957</v>
       </c>
       <c r="F9" t="inlineStr">
@@ -1082,7 +1070,7 @@
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="1" t="n">
         <v>46003</v>
       </c>
       <c r="I9" t="n">
@@ -1127,7 +1115,7 @@
       <c r="D10" t="n">
         <v>705</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="1" t="n">
         <v>45972</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -1136,7 +1124,7 @@
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="1" t="n">
         <v>46016</v>
       </c>
       <c r="I10" t="n">
@@ -1185,7 +1173,7 @@
       <c r="D11" t="n">
         <v>728</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="1" t="n">
         <v>46008</v>
       </c>
       <c r="F11" t="inlineStr">
@@ -1194,7 +1182,7 @@
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="1" t="n">
         <v>46040</v>
       </c>
       <c r="I11" t="n">
@@ -1243,7 +1231,7 @@
       <c r="D12" t="n">
         <v>278</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="1" t="n">
         <v>46042</v>
       </c>
       <c r="F12" t="inlineStr">
@@ -1252,7 +1240,7 @@
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" s="2" t="n">
+      <c r="H12" s="1" t="n">
         <v>46074</v>
       </c>
       <c r="I12" t="n">
@@ -1299,7 +1287,7 @@
       <c r="D13" t="n">
         <v>10</v>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="1" t="n">
         <v>46078</v>
       </c>
       <c r="F13" t="inlineStr">
@@ -1308,7 +1296,7 @@
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" s="2" t="n">
+      <c r="H13" s="1" t="n">
         <v>46106</v>
       </c>
       <c r="I13" t="n">
@@ -1353,7 +1341,7 @@
       <c r="D14" t="n">
         <v>15</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="1" t="n">
         <v>46094</v>
       </c>
       <c r="F14" t="inlineStr">
@@ -1362,7 +1350,7 @@
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" s="2" t="n">
+      <c r="H14" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="I14" t="n">
@@ -1409,7 +1397,7 @@
       <c r="D15" t="n">
         <v>28</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="F15" t="inlineStr">
@@ -1418,7 +1406,7 @@
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" s="2" t="n">
+      <c r="H15" s="1" t="n">
         <v>46164</v>
       </c>
       <c r="I15" t="n">
@@ -1465,7 +1453,7 @@
       <c r="D16" t="n">
         <v>33</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="1" t="n">
         <v>46156</v>
       </c>
       <c r="F16" t="inlineStr">
@@ -1474,7 +1462,7 @@
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" s="2" t="n">
+      <c r="H16" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="I16" t="n">
@@ -1521,7 +1509,7 @@
       <c r="D17" t="n">
         <v>29</v>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E17" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="F17" t="inlineStr">
@@ -1530,7 +1518,7 @@
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" s="2" t="n">
+      <c r="H17" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="I17" t="n">
@@ -1577,7 +1565,7 @@
       <c r="D18" t="n">
         <v>40</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="1" t="n">
         <v>46156</v>
       </c>
       <c r="F18" t="inlineStr">
@@ -1586,7 +1574,7 @@
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" s="2" t="n">
+      <c r="H18" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="I18" t="n">
@@ -1633,7 +1621,7 @@
       <c r="D19" t="n">
         <v>402</v>
       </c>
-      <c r="E19" s="2" t="n">
+      <c r="E19" s="1" t="n">
         <v>45791</v>
       </c>
       <c r="F19" t="inlineStr">
@@ -1642,7 +1630,7 @@
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="2" t="n">
+      <c r="H19" s="1" t="n">
         <v>45834</v>
       </c>
       <c r="I19" t="n">
@@ -1689,7 +1677,7 @@
       <c r="D20" t="n">
         <v>447</v>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="1" t="n">
         <v>45814</v>
       </c>
       <c r="F20" t="inlineStr">
@@ -1698,7 +1686,7 @@
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" s="2" t="n">
+      <c r="H20" s="1" t="n">
         <v>45955</v>
       </c>
       <c r="I20" t="n">
@@ -1749,7 +1737,7 @@
       <c r="D21" t="n">
         <v>529</v>
       </c>
-      <c r="E21" s="2" t="n">
+      <c r="E21" s="1" t="n">
         <v>45853</v>
       </c>
       <c r="F21" t="inlineStr">
@@ -1758,7 +1746,7 @@
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" s="2" t="n">
+      <c r="H21" s="1" t="n">
         <v>45939</v>
       </c>
       <c r="I21" t="n">
@@ -1809,7 +1797,7 @@
       <c r="D22" t="n">
         <v>691</v>
       </c>
-      <c r="E22" s="2" t="n">
+      <c r="E22" s="1" t="n">
         <v>45910</v>
       </c>
       <c r="F22" t="inlineStr">
@@ -1818,7 +1806,7 @@
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" s="2" t="n">
+      <c r="H22" s="1" t="n">
         <v>45941</v>
       </c>
       <c r="I22" t="n">
@@ -1867,7 +1855,7 @@
       <c r="D23" t="n">
         <v>677</v>
       </c>
-      <c r="E23" s="2" t="n">
+      <c r="E23" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="F23" t="inlineStr">
@@ -1876,7 +1864,7 @@
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" s="2" t="n">
+      <c r="H23" s="1" t="n">
         <v>45935</v>
       </c>
       <c r="I23" t="n">
@@ -1923,7 +1911,7 @@
       <c r="D24" t="n">
         <v>278</v>
       </c>
-      <c r="E24" s="2" t="n">
+      <c r="E24" s="1" t="n">
         <v>46008</v>
       </c>
       <c r="F24" t="inlineStr">
@@ -1932,7 +1920,7 @@
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" s="2" t="n">
+      <c r="H24" s="1" t="n">
         <v>46066</v>
       </c>
       <c r="I24" t="n">
@@ -1981,7 +1969,7 @@
       <c r="D25" t="n">
         <v>748</v>
       </c>
-      <c r="E25" s="2" t="n">
+      <c r="E25" s="1" t="n">
         <v>45930</v>
       </c>
       <c r="F25" t="inlineStr">
@@ -1990,7 +1978,7 @@
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" s="2" t="n">
+      <c r="H25" s="1" t="n">
         <v>45935</v>
       </c>
       <c r="I25" t="n">
@@ -2037,7 +2025,7 @@
       <c r="D26" t="n">
         <v>822</v>
       </c>
-      <c r="E26" s="2" t="n">
+      <c r="E26" s="1" t="n">
         <v>45968</v>
       </c>
       <c r="F26" t="inlineStr">
@@ -2046,7 +2034,7 @@
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" s="2" t="n">
+      <c r="H26" s="1" t="n">
         <v>45935</v>
       </c>
       <c r="I26" t="n">
@@ -2093,7 +2081,7 @@
       <c r="D27" t="n">
         <v>360</v>
       </c>
-      <c r="E27" s="2" t="n">
+      <c r="E27" s="1" t="n">
         <v>46043</v>
       </c>
       <c r="F27" t="inlineStr">
@@ -2102,7 +2090,7 @@
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" s="2" t="n">
+      <c r="H27" s="1" t="n">
         <v>46075</v>
       </c>
       <c r="I27" t="n">
@@ -2223,7 +2211,7 @@
       <c r="D30" t="n">
         <v>1465</v>
       </c>
-      <c r="E30" s="2" t="n">
+      <c r="E30" s="1" t="n">
         <v>46104</v>
       </c>
       <c r="F30" t="inlineStr">
@@ -2232,7 +2220,7 @@
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" s="2" t="n">
+      <c r="H30" s="1" t="n">
         <v>46106</v>
       </c>
       <c r="I30" t="n">
@@ -2275,27 +2263,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>numero_empenho</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>valor_empenhado</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>saldo</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>responsavel</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>justificativa</t>
         </is>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (10/07/2026 16:00)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -22,13 +22,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +42,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,12 +50,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -423,57 +435,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>numero_contrato</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ug_executora</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>ug_responsavel</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ug_fiscalizadora</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>valor_total_contrato</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>valor_a_empenhar</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>valor_empenhado</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>valor_liquidado</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>saldo_a_faturar</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>fornecedor</t>
         </is>
@@ -541,92 +553,92 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>modulo</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>referencia</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>numero_recibo</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>numero_nota_fiscal</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>empenho</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>observacao</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>vencimento</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>valor_nfs</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>ordem_pagamento</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>faturado</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>tipo_registro</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>empenho_saldo</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>empenho_valor_empenhado</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>empenho_responsavel</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>empenho_justificativa</t>
         </is>
@@ -649,7 +661,7 @@
       <c r="D2" t="n">
         <v>594</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="2" t="n">
         <v>45740</v>
       </c>
       <c r="F2" t="inlineStr">
@@ -658,7 +670,7 @@
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="1" t="n">
+      <c r="H2" s="2" t="n">
         <v>45778</v>
       </c>
       <c r="I2" t="n">
@@ -707,7 +719,7 @@
       <c r="D3" t="n">
         <v>620</v>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="2" t="n">
         <v>45775</v>
       </c>
       <c r="F3" t="inlineStr">
@@ -716,7 +728,7 @@
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="1" t="n">
+      <c r="H3" s="2" t="n">
         <v>45806</v>
       </c>
       <c r="I3" t="n">
@@ -765,7 +777,7 @@
       <c r="D4" t="n">
         <v>634</v>
       </c>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="2" t="n">
         <v>45799</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -774,7 +786,7 @@
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" s="1" t="n">
+      <c r="H4" s="2" t="n">
         <v>45844</v>
       </c>
       <c r="I4" t="n">
@@ -823,7 +835,7 @@
       <c r="D5" t="n">
         <v>660</v>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E5" s="2" t="n">
         <v>45856</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -832,7 +844,7 @@
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" s="1" t="n">
+      <c r="H5" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="I5" t="n">
@@ -881,7 +893,7 @@
       <c r="D6" t="n">
         <v>661</v>
       </c>
-      <c r="E6" s="1" t="n">
+      <c r="E6" s="2" t="n">
         <v>45856</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -893,7 +905,7 @@
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" s="1" t="n">
+      <c r="H6" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="I6" t="n">
@@ -944,7 +956,7 @@
       <c r="D7" t="n">
         <v>688</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>45901</v>
       </c>
       <c r="F7" t="inlineStr">
@@ -953,7 +965,7 @@
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" s="1" t="n">
+      <c r="H7" s="2" t="n">
         <v>45938</v>
       </c>
       <c r="I7" t="n">
@@ -1002,7 +1014,7 @@
       <c r="D8" t="n">
         <v>696</v>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="2" t="n">
         <v>45923</v>
       </c>
       <c r="F8" t="inlineStr">
@@ -1011,7 +1023,7 @@
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" s="1" t="n">
+      <c r="H8" s="2" t="n">
         <v>45938</v>
       </c>
       <c r="I8" t="n">
@@ -1060,7 +1072,7 @@
       <c r="D9" t="n">
         <v>704</v>
       </c>
-      <c r="E9" s="1" t="n">
+      <c r="E9" s="2" t="n">
         <v>45957</v>
       </c>
       <c r="F9" t="inlineStr">
@@ -1070,7 +1082,7 @@
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" s="1" t="n">
+      <c r="H9" s="2" t="n">
         <v>46003</v>
       </c>
       <c r="I9" t="n">
@@ -1115,7 +1127,7 @@
       <c r="D10" t="n">
         <v>705</v>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="2" t="n">
         <v>45972</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -1124,7 +1136,7 @@
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" s="1" t="n">
+      <c r="H10" s="2" t="n">
         <v>46016</v>
       </c>
       <c r="I10" t="n">
@@ -1173,7 +1185,7 @@
       <c r="D11" t="n">
         <v>728</v>
       </c>
-      <c r="E11" s="1" t="n">
+      <c r="E11" s="2" t="n">
         <v>46008</v>
       </c>
       <c r="F11" t="inlineStr">
@@ -1182,7 +1194,7 @@
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" s="1" t="n">
+      <c r="H11" s="2" t="n">
         <v>46040</v>
       </c>
       <c r="I11" t="n">
@@ -1231,7 +1243,7 @@
       <c r="D12" t="n">
         <v>278</v>
       </c>
-      <c r="E12" s="1" t="n">
+      <c r="E12" s="2" t="n">
         <v>46042</v>
       </c>
       <c r="F12" t="inlineStr">
@@ -1240,7 +1252,7 @@
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" s="1" t="n">
+      <c r="H12" s="2" t="n">
         <v>46074</v>
       </c>
       <c r="I12" t="n">
@@ -1287,7 +1299,7 @@
       <c r="D13" t="n">
         <v>10</v>
       </c>
-      <c r="E13" s="1" t="n">
+      <c r="E13" s="2" t="n">
         <v>46078</v>
       </c>
       <c r="F13" t="inlineStr">
@@ -1296,7 +1308,7 @@
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" s="1" t="n">
+      <c r="H13" s="2" t="n">
         <v>46106</v>
       </c>
       <c r="I13" t="n">
@@ -1341,7 +1353,7 @@
       <c r="D14" t="n">
         <v>15</v>
       </c>
-      <c r="E14" s="1" t="n">
+      <c r="E14" s="2" t="n">
         <v>46094</v>
       </c>
       <c r="F14" t="inlineStr">
@@ -1350,7 +1362,7 @@
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" s="1" t="n">
+      <c r="H14" s="2" t="n">
         <v>46128</v>
       </c>
       <c r="I14" t="n">
@@ -1397,7 +1409,7 @@
       <c r="D15" t="n">
         <v>28</v>
       </c>
-      <c r="E15" s="1" t="n">
+      <c r="E15" s="2" t="n">
         <v>46128</v>
       </c>
       <c r="F15" t="inlineStr">
@@ -1406,7 +1418,7 @@
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" s="1" t="n">
+      <c r="H15" s="2" t="n">
         <v>46164</v>
       </c>
       <c r="I15" t="n">
@@ -1453,7 +1465,7 @@
       <c r="D16" t="n">
         <v>33</v>
       </c>
-      <c r="E16" s="1" t="n">
+      <c r="E16" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="F16" t="inlineStr">
@@ -1462,7 +1474,7 @@
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" s="1" t="n">
+      <c r="H16" s="2" t="n">
         <v>46191</v>
       </c>
       <c r="I16" t="n">
@@ -1509,7 +1521,7 @@
       <c r="D17" t="n">
         <v>29</v>
       </c>
-      <c r="E17" s="1" t="n">
+      <c r="E17" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="F17" t="inlineStr">
@@ -1518,7 +1530,7 @@
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" s="1" t="n">
+      <c r="H17" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="I17" t="n">
@@ -1565,7 +1577,7 @@
       <c r="D18" t="n">
         <v>40</v>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="F18" t="inlineStr">
@@ -1574,7 +1586,7 @@
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" s="1" t="n">
+      <c r="H18" s="2" t="n">
         <v>46191</v>
       </c>
       <c r="I18" t="n">
@@ -1621,7 +1633,7 @@
       <c r="D19" t="n">
         <v>402</v>
       </c>
-      <c r="E19" s="1" t="n">
+      <c r="E19" s="2" t="n">
         <v>45791</v>
       </c>
       <c r="F19" t="inlineStr">
@@ -1630,7 +1642,7 @@
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="1" t="n">
+      <c r="H19" s="2" t="n">
         <v>45834</v>
       </c>
       <c r="I19" t="n">
@@ -1677,7 +1689,7 @@
       <c r="D20" t="n">
         <v>447</v>
       </c>
-      <c r="E20" s="1" t="n">
+      <c r="E20" s="2" t="n">
         <v>45814</v>
       </c>
       <c r="F20" t="inlineStr">
@@ -1686,7 +1698,7 @@
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" s="1" t="n">
+      <c r="H20" s="2" t="n">
         <v>45955</v>
       </c>
       <c r="I20" t="n">
@@ -1737,7 +1749,7 @@
       <c r="D21" t="n">
         <v>529</v>
       </c>
-      <c r="E21" s="1" t="n">
+      <c r="E21" s="2" t="n">
         <v>45853</v>
       </c>
       <c r="F21" t="inlineStr">
@@ -1746,7 +1758,7 @@
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" s="1" t="n">
+      <c r="H21" s="2" t="n">
         <v>45939</v>
       </c>
       <c r="I21" t="n">
@@ -1797,7 +1809,7 @@
       <c r="D22" t="n">
         <v>691</v>
       </c>
-      <c r="E22" s="1" t="n">
+      <c r="E22" s="2" t="n">
         <v>45910</v>
       </c>
       <c r="F22" t="inlineStr">
@@ -1806,7 +1818,7 @@
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" s="1" t="n">
+      <c r="H22" s="2" t="n">
         <v>45941</v>
       </c>
       <c r="I22" t="n">
@@ -1855,7 +1867,7 @@
       <c r="D23" t="n">
         <v>677</v>
       </c>
-      <c r="E23" s="1" t="n">
+      <c r="E23" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="F23" t="inlineStr">
@@ -1864,7 +1876,7 @@
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" s="1" t="n">
+      <c r="H23" s="2" t="n">
         <v>45935</v>
       </c>
       <c r="I23" t="n">
@@ -1911,7 +1923,7 @@
       <c r="D24" t="n">
         <v>278</v>
       </c>
-      <c r="E24" s="1" t="n">
+      <c r="E24" s="2" t="n">
         <v>46008</v>
       </c>
       <c r="F24" t="inlineStr">
@@ -1920,7 +1932,7 @@
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" s="1" t="n">
+      <c r="H24" s="2" t="n">
         <v>46066</v>
       </c>
       <c r="I24" t="n">
@@ -1969,7 +1981,7 @@
       <c r="D25" t="n">
         <v>748</v>
       </c>
-      <c r="E25" s="1" t="n">
+      <c r="E25" s="2" t="n">
         <v>45930</v>
       </c>
       <c r="F25" t="inlineStr">
@@ -1978,7 +1990,7 @@
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" s="1" t="n">
+      <c r="H25" s="2" t="n">
         <v>45935</v>
       </c>
       <c r="I25" t="n">
@@ -2025,7 +2037,7 @@
       <c r="D26" t="n">
         <v>822</v>
       </c>
-      <c r="E26" s="1" t="n">
+      <c r="E26" s="2" t="n">
         <v>45968</v>
       </c>
       <c r="F26" t="inlineStr">
@@ -2034,7 +2046,7 @@
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" s="1" t="n">
+      <c r="H26" s="2" t="n">
         <v>45935</v>
       </c>
       <c r="I26" t="n">
@@ -2081,7 +2093,7 @@
       <c r="D27" t="n">
         <v>360</v>
       </c>
-      <c r="E27" s="1" t="n">
+      <c r="E27" s="2" t="n">
         <v>46043</v>
       </c>
       <c r="F27" t="inlineStr">
@@ -2090,7 +2102,7 @@
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" s="1" t="n">
+      <c r="H27" s="2" t="n">
         <v>46075</v>
       </c>
       <c r="I27" t="n">
@@ -2211,7 +2223,7 @@
       <c r="D30" t="n">
         <v>1465</v>
       </c>
-      <c r="E30" s="1" t="n">
+      <c r="E30" s="2" t="n">
         <v>46104</v>
       </c>
       <c r="F30" t="inlineStr">
@@ -2220,7 +2232,7 @@
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" s="1" t="n">
+      <c r="H30" s="2" t="n">
         <v>46106</v>
       </c>
       <c r="I30" t="n">
@@ -2263,27 +2275,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>numero_empenho</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>valor_empenhado</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>saldo</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>responsavel</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>justificativa</t>
         </is>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (10/07/2026 22:38)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -22,16 +22,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -50,21 +47,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -435,57 +423,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>numero_contrato</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>ug_executora</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ug_responsavel</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ug_fiscalizadora</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>valor_total_contrato</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>valor_a_empenhar</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>valor_empenhado</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>valor_liquidado</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>saldo_a_faturar</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>fornecedor</t>
         </is>
@@ -553,92 +541,92 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>modulo</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>referencia</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>numero_recibo</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>numero_nota_fiscal</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>empenho</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>observacao</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>vencimento</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>valor_nfs</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ordem_pagamento</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>faturado</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>tipo_registro</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>empenho_saldo</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>empenho_valor_empenhado</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>empenho_responsavel</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>empenho_justificativa</t>
         </is>
@@ -661,7 +649,7 @@
       <c r="D2" t="n">
         <v>594</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="1" t="n">
         <v>45740</v>
       </c>
       <c r="F2" t="inlineStr">
@@ -670,7 +658,7 @@
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="1" t="n">
         <v>45778</v>
       </c>
       <c r="I2" t="n">
@@ -719,7 +707,7 @@
       <c r="D3" t="n">
         <v>620</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="1" t="n">
         <v>45775</v>
       </c>
       <c r="F3" t="inlineStr">
@@ -728,7 +716,7 @@
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="1" t="n">
         <v>45806</v>
       </c>
       <c r="I3" t="n">
@@ -777,7 +765,7 @@
       <c r="D4" t="n">
         <v>634</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="1" t="n">
         <v>45799</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -786,7 +774,7 @@
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="1" t="n">
         <v>45844</v>
       </c>
       <c r="I4" t="n">
@@ -835,7 +823,7 @@
       <c r="D5" t="n">
         <v>660</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -844,7 +832,7 @@
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="I5" t="n">
@@ -893,7 +881,7 @@
       <c r="D6" t="n">
         <v>661</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -905,7 +893,7 @@
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="I6" t="n">
@@ -956,7 +944,7 @@
       <c r="D7" t="n">
         <v>688</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="1" t="n">
         <v>45901</v>
       </c>
       <c r="F7" t="inlineStr">
@@ -965,7 +953,7 @@
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="1" t="n">
         <v>45938</v>
       </c>
       <c r="I7" t="n">
@@ -1014,7 +1002,7 @@
       <c r="D8" t="n">
         <v>696</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="1" t="n">
         <v>45923</v>
       </c>
       <c r="F8" t="inlineStr">
@@ -1023,7 +1011,7 @@
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="1" t="n">
         <v>45938</v>
       </c>
       <c r="I8" t="n">
@@ -1072,7 +1060,7 @@
       <c r="D9" t="n">
         <v>704</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="1" t="n">
         <v>45957</v>
       </c>
       <c r="F9" t="inlineStr">
@@ -1082,7 +1070,7 @@
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="1" t="n">
         <v>46003</v>
       </c>
       <c r="I9" t="n">
@@ -1127,7 +1115,7 @@
       <c r="D10" t="n">
         <v>705</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="1" t="n">
         <v>45972</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -1136,7 +1124,7 @@
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="1" t="n">
         <v>46016</v>
       </c>
       <c r="I10" t="n">
@@ -1185,7 +1173,7 @@
       <c r="D11" t="n">
         <v>728</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="1" t="n">
         <v>46008</v>
       </c>
       <c r="F11" t="inlineStr">
@@ -1194,7 +1182,7 @@
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="1" t="n">
         <v>46040</v>
       </c>
       <c r="I11" t="n">
@@ -1243,7 +1231,7 @@
       <c r="D12" t="n">
         <v>278</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="1" t="n">
         <v>46042</v>
       </c>
       <c r="F12" t="inlineStr">
@@ -1252,7 +1240,7 @@
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" s="2" t="n">
+      <c r="H12" s="1" t="n">
         <v>46074</v>
       </c>
       <c r="I12" t="n">
@@ -1299,7 +1287,7 @@
       <c r="D13" t="n">
         <v>10</v>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="1" t="n">
         <v>46078</v>
       </c>
       <c r="F13" t="inlineStr">
@@ -1308,7 +1296,7 @@
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" s="2" t="n">
+      <c r="H13" s="1" t="n">
         <v>46106</v>
       </c>
       <c r="I13" t="n">
@@ -1353,7 +1341,7 @@
       <c r="D14" t="n">
         <v>15</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="1" t="n">
         <v>46094</v>
       </c>
       <c r="F14" t="inlineStr">
@@ -1362,7 +1350,7 @@
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" s="2" t="n">
+      <c r="H14" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="I14" t="n">
@@ -1409,7 +1397,7 @@
       <c r="D15" t="n">
         <v>28</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="F15" t="inlineStr">
@@ -1418,7 +1406,7 @@
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" s="2" t="n">
+      <c r="H15" s="1" t="n">
         <v>46164</v>
       </c>
       <c r="I15" t="n">
@@ -1465,7 +1453,7 @@
       <c r="D16" t="n">
         <v>33</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="1" t="n">
         <v>46156</v>
       </c>
       <c r="F16" t="inlineStr">
@@ -1474,7 +1462,7 @@
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" s="2" t="n">
+      <c r="H16" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="I16" t="n">
@@ -1521,7 +1509,7 @@
       <c r="D17" t="n">
         <v>29</v>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E17" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="F17" t="inlineStr">
@@ -1530,7 +1518,7 @@
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" s="2" t="n">
+      <c r="H17" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="I17" t="n">
@@ -1577,7 +1565,7 @@
       <c r="D18" t="n">
         <v>40</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="1" t="n">
         <v>46156</v>
       </c>
       <c r="F18" t="inlineStr">
@@ -1586,7 +1574,7 @@
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" s="2" t="n">
+      <c r="H18" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="I18" t="n">
@@ -1633,7 +1621,7 @@
       <c r="D19" t="n">
         <v>402</v>
       </c>
-      <c r="E19" s="2" t="n">
+      <c r="E19" s="1" t="n">
         <v>45791</v>
       </c>
       <c r="F19" t="inlineStr">
@@ -1642,7 +1630,7 @@
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="2" t="n">
+      <c r="H19" s="1" t="n">
         <v>45834</v>
       </c>
       <c r="I19" t="n">
@@ -1689,7 +1677,7 @@
       <c r="D20" t="n">
         <v>447</v>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="1" t="n">
         <v>45814</v>
       </c>
       <c r="F20" t="inlineStr">
@@ -1698,7 +1686,7 @@
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" s="2" t="n">
+      <c r="H20" s="1" t="n">
         <v>45955</v>
       </c>
       <c r="I20" t="n">
@@ -1749,7 +1737,7 @@
       <c r="D21" t="n">
         <v>529</v>
       </c>
-      <c r="E21" s="2" t="n">
+      <c r="E21" s="1" t="n">
         <v>45853</v>
       </c>
       <c r="F21" t="inlineStr">
@@ -1758,7 +1746,7 @@
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" s="2" t="n">
+      <c r="H21" s="1" t="n">
         <v>45939</v>
       </c>
       <c r="I21" t="n">
@@ -1809,7 +1797,7 @@
       <c r="D22" t="n">
         <v>691</v>
       </c>
-      <c r="E22" s="2" t="n">
+      <c r="E22" s="1" t="n">
         <v>45910</v>
       </c>
       <c r="F22" t="inlineStr">
@@ -1818,7 +1806,7 @@
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" s="2" t="n">
+      <c r="H22" s="1" t="n">
         <v>45941</v>
       </c>
       <c r="I22" t="n">
@@ -1867,7 +1855,7 @@
       <c r="D23" t="n">
         <v>677</v>
       </c>
-      <c r="E23" s="2" t="n">
+      <c r="E23" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="F23" t="inlineStr">
@@ -1876,7 +1864,7 @@
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" s="2" t="n">
+      <c r="H23" s="1" t="n">
         <v>45935</v>
       </c>
       <c r="I23" t="n">
@@ -1923,7 +1911,7 @@
       <c r="D24" t="n">
         <v>278</v>
       </c>
-      <c r="E24" s="2" t="n">
+      <c r="E24" s="1" t="n">
         <v>46008</v>
       </c>
       <c r="F24" t="inlineStr">
@@ -1932,7 +1920,7 @@
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" s="2" t="n">
+      <c r="H24" s="1" t="n">
         <v>46066</v>
       </c>
       <c r="I24" t="n">
@@ -1981,7 +1969,7 @@
       <c r="D25" t="n">
         <v>748</v>
       </c>
-      <c r="E25" s="2" t="n">
+      <c r="E25" s="1" t="n">
         <v>45930</v>
       </c>
       <c r="F25" t="inlineStr">
@@ -1990,7 +1978,7 @@
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" s="2" t="n">
+      <c r="H25" s="1" t="n">
         <v>45935</v>
       </c>
       <c r="I25" t="n">
@@ -2037,7 +2025,7 @@
       <c r="D26" t="n">
         <v>822</v>
       </c>
-      <c r="E26" s="2" t="n">
+      <c r="E26" s="1" t="n">
         <v>45968</v>
       </c>
       <c r="F26" t="inlineStr">
@@ -2046,7 +2034,7 @@
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" s="2" t="n">
+      <c r="H26" s="1" t="n">
         <v>45935</v>
       </c>
       <c r="I26" t="n">
@@ -2093,7 +2081,7 @@
       <c r="D27" t="n">
         <v>360</v>
       </c>
-      <c r="E27" s="2" t="n">
+      <c r="E27" s="1" t="n">
         <v>46043</v>
       </c>
       <c r="F27" t="inlineStr">
@@ -2102,7 +2090,7 @@
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" s="2" t="n">
+      <c r="H27" s="1" t="n">
         <v>46075</v>
       </c>
       <c r="I27" t="n">
@@ -2223,7 +2211,7 @@
       <c r="D30" t="n">
         <v>1465</v>
       </c>
-      <c r="E30" s="2" t="n">
+      <c r="E30" s="1" t="n">
         <v>46104</v>
       </c>
       <c r="F30" t="inlineStr">
@@ -2232,7 +2220,7 @@
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" s="2" t="n">
+      <c r="H30" s="1" t="n">
         <v>46106</v>
       </c>
       <c r="I30" t="n">
@@ -2275,27 +2263,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>numero_empenho</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>valor_empenhado</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>saldo</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>responsavel</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>justificativa</t>
         </is>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (10/07/2026 20:00)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -22,13 +22,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +42,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,12 +50,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -423,57 +435,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>numero_contrato</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>ug_executora</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>ug_responsavel</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ug_fiscalizadora</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>valor_total_contrato</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>valor_a_empenhar</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>valor_empenhado</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>valor_liquidado</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>saldo_a_faturar</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>fornecedor</t>
         </is>
@@ -541,92 +553,92 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>modulo</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>referencia</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>numero_recibo</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>numero_nota_fiscal</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>empenho</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>observacao</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>vencimento</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>valor_nfs</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>ordem_pagamento</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>faturado</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>tipo_registro</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>empenho_saldo</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>empenho_valor_empenhado</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>empenho_responsavel</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>empenho_justificativa</t>
         </is>
@@ -649,7 +661,7 @@
       <c r="D2" t="n">
         <v>594</v>
       </c>
-      <c r="E2" s="1" t="n">
+      <c r="E2" s="2" t="n">
         <v>45740</v>
       </c>
       <c r="F2" t="inlineStr">
@@ -658,7 +670,7 @@
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="1" t="n">
+      <c r="H2" s="2" t="n">
         <v>45778</v>
       </c>
       <c r="I2" t="n">
@@ -707,7 +719,7 @@
       <c r="D3" t="n">
         <v>620</v>
       </c>
-      <c r="E3" s="1" t="n">
+      <c r="E3" s="2" t="n">
         <v>45775</v>
       </c>
       <c r="F3" t="inlineStr">
@@ -716,7 +728,7 @@
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="1" t="n">
+      <c r="H3" s="2" t="n">
         <v>45806</v>
       </c>
       <c r="I3" t="n">
@@ -765,7 +777,7 @@
       <c r="D4" t="n">
         <v>634</v>
       </c>
-      <c r="E4" s="1" t="n">
+      <c r="E4" s="2" t="n">
         <v>45799</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -774,7 +786,7 @@
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" s="1" t="n">
+      <c r="H4" s="2" t="n">
         <v>45844</v>
       </c>
       <c r="I4" t="n">
@@ -823,7 +835,7 @@
       <c r="D5" t="n">
         <v>660</v>
       </c>
-      <c r="E5" s="1" t="n">
+      <c r="E5" s="2" t="n">
         <v>45856</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -832,7 +844,7 @@
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" s="1" t="n">
+      <c r="H5" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="I5" t="n">
@@ -881,7 +893,7 @@
       <c r="D6" t="n">
         <v>661</v>
       </c>
-      <c r="E6" s="1" t="n">
+      <c r="E6" s="2" t="n">
         <v>45856</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -893,7 +905,7 @@
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" s="1" t="n">
+      <c r="H6" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="I6" t="n">
@@ -944,7 +956,7 @@
       <c r="D7" t="n">
         <v>688</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E7" s="2" t="n">
         <v>45901</v>
       </c>
       <c r="F7" t="inlineStr">
@@ -953,7 +965,7 @@
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" s="1" t="n">
+      <c r="H7" s="2" t="n">
         <v>45938</v>
       </c>
       <c r="I7" t="n">
@@ -1002,7 +1014,7 @@
       <c r="D8" t="n">
         <v>696</v>
       </c>
-      <c r="E8" s="1" t="n">
+      <c r="E8" s="2" t="n">
         <v>45923</v>
       </c>
       <c r="F8" t="inlineStr">
@@ -1011,7 +1023,7 @@
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" s="1" t="n">
+      <c r="H8" s="2" t="n">
         <v>45938</v>
       </c>
       <c r="I8" t="n">
@@ -1060,7 +1072,7 @@
       <c r="D9" t="n">
         <v>704</v>
       </c>
-      <c r="E9" s="1" t="n">
+      <c r="E9" s="2" t="n">
         <v>45957</v>
       </c>
       <c r="F9" t="inlineStr">
@@ -1070,7 +1082,7 @@
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" s="1" t="n">
+      <c r="H9" s="2" t="n">
         <v>46003</v>
       </c>
       <c r="I9" t="n">
@@ -1115,7 +1127,7 @@
       <c r="D10" t="n">
         <v>705</v>
       </c>
-      <c r="E10" s="1" t="n">
+      <c r="E10" s="2" t="n">
         <v>45972</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -1124,7 +1136,7 @@
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" s="1" t="n">
+      <c r="H10" s="2" t="n">
         <v>46016</v>
       </c>
       <c r="I10" t="n">
@@ -1173,7 +1185,7 @@
       <c r="D11" t="n">
         <v>728</v>
       </c>
-      <c r="E11" s="1" t="n">
+      <c r="E11" s="2" t="n">
         <v>46008</v>
       </c>
       <c r="F11" t="inlineStr">
@@ -1182,7 +1194,7 @@
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" s="1" t="n">
+      <c r="H11" s="2" t="n">
         <v>46040</v>
       </c>
       <c r="I11" t="n">
@@ -1231,7 +1243,7 @@
       <c r="D12" t="n">
         <v>278</v>
       </c>
-      <c r="E12" s="1" t="n">
+      <c r="E12" s="2" t="n">
         <v>46042</v>
       </c>
       <c r="F12" t="inlineStr">
@@ -1240,7 +1252,7 @@
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" s="1" t="n">
+      <c r="H12" s="2" t="n">
         <v>46074</v>
       </c>
       <c r="I12" t="n">
@@ -1287,7 +1299,7 @@
       <c r="D13" t="n">
         <v>10</v>
       </c>
-      <c r="E13" s="1" t="n">
+      <c r="E13" s="2" t="n">
         <v>46078</v>
       </c>
       <c r="F13" t="inlineStr">
@@ -1296,7 +1308,7 @@
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" s="1" t="n">
+      <c r="H13" s="2" t="n">
         <v>46106</v>
       </c>
       <c r="I13" t="n">
@@ -1341,7 +1353,7 @@
       <c r="D14" t="n">
         <v>15</v>
       </c>
-      <c r="E14" s="1" t="n">
+      <c r="E14" s="2" t="n">
         <v>46094</v>
       </c>
       <c r="F14" t="inlineStr">
@@ -1350,7 +1362,7 @@
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" s="1" t="n">
+      <c r="H14" s="2" t="n">
         <v>46128</v>
       </c>
       <c r="I14" t="n">
@@ -1397,7 +1409,7 @@
       <c r="D15" t="n">
         <v>28</v>
       </c>
-      <c r="E15" s="1" t="n">
+      <c r="E15" s="2" t="n">
         <v>46128</v>
       </c>
       <c r="F15" t="inlineStr">
@@ -1406,7 +1418,7 @@
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" s="1" t="n">
+      <c r="H15" s="2" t="n">
         <v>46164</v>
       </c>
       <c r="I15" t="n">
@@ -1453,7 +1465,7 @@
       <c r="D16" t="n">
         <v>33</v>
       </c>
-      <c r="E16" s="1" t="n">
+      <c r="E16" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="F16" t="inlineStr">
@@ -1462,7 +1474,7 @@
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" s="1" t="n">
+      <c r="H16" s="2" t="n">
         <v>46191</v>
       </c>
       <c r="I16" t="n">
@@ -1509,7 +1521,7 @@
       <c r="D17" t="n">
         <v>29</v>
       </c>
-      <c r="E17" s="1" t="n">
+      <c r="E17" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="F17" t="inlineStr">
@@ -1518,7 +1530,7 @@
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" s="1" t="n">
+      <c r="H17" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="I17" t="n">
@@ -1565,7 +1577,7 @@
       <c r="D18" t="n">
         <v>40</v>
       </c>
-      <c r="E18" s="1" t="n">
+      <c r="E18" s="2" t="n">
         <v>46156</v>
       </c>
       <c r="F18" t="inlineStr">
@@ -1574,7 +1586,7 @@
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" s="1" t="n">
+      <c r="H18" s="2" t="n">
         <v>46191</v>
       </c>
       <c r="I18" t="n">
@@ -1621,7 +1633,7 @@
       <c r="D19" t="n">
         <v>402</v>
       </c>
-      <c r="E19" s="1" t="n">
+      <c r="E19" s="2" t="n">
         <v>45791</v>
       </c>
       <c r="F19" t="inlineStr">
@@ -1630,7 +1642,7 @@
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="1" t="n">
+      <c r="H19" s="2" t="n">
         <v>45834</v>
       </c>
       <c r="I19" t="n">
@@ -1677,7 +1689,7 @@
       <c r="D20" t="n">
         <v>447</v>
       </c>
-      <c r="E20" s="1" t="n">
+      <c r="E20" s="2" t="n">
         <v>45814</v>
       </c>
       <c r="F20" t="inlineStr">
@@ -1686,7 +1698,7 @@
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" s="1" t="n">
+      <c r="H20" s="2" t="n">
         <v>45955</v>
       </c>
       <c r="I20" t="n">
@@ -1737,7 +1749,7 @@
       <c r="D21" t="n">
         <v>529</v>
       </c>
-      <c r="E21" s="1" t="n">
+      <c r="E21" s="2" t="n">
         <v>45853</v>
       </c>
       <c r="F21" t="inlineStr">
@@ -1746,7 +1758,7 @@
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" s="1" t="n">
+      <c r="H21" s="2" t="n">
         <v>45939</v>
       </c>
       <c r="I21" t="n">
@@ -1797,7 +1809,7 @@
       <c r="D22" t="n">
         <v>691</v>
       </c>
-      <c r="E22" s="1" t="n">
+      <c r="E22" s="2" t="n">
         <v>45910</v>
       </c>
       <c r="F22" t="inlineStr">
@@ -1806,7 +1818,7 @@
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" s="1" t="n">
+      <c r="H22" s="2" t="n">
         <v>45941</v>
       </c>
       <c r="I22" t="n">
@@ -1855,7 +1867,7 @@
       <c r="D23" t="n">
         <v>677</v>
       </c>
-      <c r="E23" s="1" t="n">
+      <c r="E23" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="F23" t="inlineStr">
@@ -1864,7 +1876,7 @@
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" s="1" t="n">
+      <c r="H23" s="2" t="n">
         <v>45935</v>
       </c>
       <c r="I23" t="n">
@@ -1911,7 +1923,7 @@
       <c r="D24" t="n">
         <v>278</v>
       </c>
-      <c r="E24" s="1" t="n">
+      <c r="E24" s="2" t="n">
         <v>46008</v>
       </c>
       <c r="F24" t="inlineStr">
@@ -1920,7 +1932,7 @@
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" s="1" t="n">
+      <c r="H24" s="2" t="n">
         <v>46066</v>
       </c>
       <c r="I24" t="n">
@@ -1969,7 +1981,7 @@
       <c r="D25" t="n">
         <v>748</v>
       </c>
-      <c r="E25" s="1" t="n">
+      <c r="E25" s="2" t="n">
         <v>45930</v>
       </c>
       <c r="F25" t="inlineStr">
@@ -1978,7 +1990,7 @@
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" s="1" t="n">
+      <c r="H25" s="2" t="n">
         <v>45935</v>
       </c>
       <c r="I25" t="n">
@@ -2025,7 +2037,7 @@
       <c r="D26" t="n">
         <v>822</v>
       </c>
-      <c r="E26" s="1" t="n">
+      <c r="E26" s="2" t="n">
         <v>45968</v>
       </c>
       <c r="F26" t="inlineStr">
@@ -2034,7 +2046,7 @@
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" s="1" t="n">
+      <c r="H26" s="2" t="n">
         <v>45935</v>
       </c>
       <c r="I26" t="n">
@@ -2081,7 +2093,7 @@
       <c r="D27" t="n">
         <v>360</v>
       </c>
-      <c r="E27" s="1" t="n">
+      <c r="E27" s="2" t="n">
         <v>46043</v>
       </c>
       <c r="F27" t="inlineStr">
@@ -2090,7 +2102,7 @@
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" s="1" t="n">
+      <c r="H27" s="2" t="n">
         <v>46075</v>
       </c>
       <c r="I27" t="n">
@@ -2211,7 +2223,7 @@
       <c r="D30" t="n">
         <v>1465</v>
       </c>
-      <c r="E30" s="1" t="n">
+      <c r="E30" s="2" t="n">
         <v>46104</v>
       </c>
       <c r="F30" t="inlineStr">
@@ -2220,7 +2232,7 @@
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" s="1" t="n">
+      <c r="H30" s="2" t="n">
         <v>46106</v>
       </c>
       <c r="I30" t="n">
@@ -2263,27 +2275,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>numero_empenho</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>valor_empenhado</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>saldo</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>responsavel</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>justificativa</t>
         </is>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (11/07/2026 07:19)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -22,16 +22,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -50,21 +47,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -435,57 +423,57 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>numero_contrato</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>ug_executora</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>ug_responsavel</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>ug_fiscalizadora</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>valor_total_contrato</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>valor_a_empenhar</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>valor_empenhado</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>valor_liquidado</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>saldo_a_faturar</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>fornecedor</t>
         </is>
@@ -553,92 +541,92 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>modulo</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>referencia</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>numero_recibo</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>numero_nota_fiscal</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>data</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>empenho</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>observacao</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>vencimento</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>valor_nfs</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>ordem_pagamento</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>faturado</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>pendente</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>tipo_registro</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>situacao</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>empenho_saldo</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>empenho_valor_empenhado</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>empenho_responsavel</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>empenho_justificativa</t>
         </is>
@@ -661,7 +649,7 @@
       <c r="D2" t="n">
         <v>594</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="1" t="n">
         <v>45740</v>
       </c>
       <c r="F2" t="inlineStr">
@@ -670,7 +658,7 @@
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="1" t="n">
         <v>45778</v>
       </c>
       <c r="I2" t="n">
@@ -719,7 +707,7 @@
       <c r="D3" t="n">
         <v>620</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="1" t="n">
         <v>45775</v>
       </c>
       <c r="F3" t="inlineStr">
@@ -728,7 +716,7 @@
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="1" t="n">
         <v>45806</v>
       </c>
       <c r="I3" t="n">
@@ -777,7 +765,7 @@
       <c r="D4" t="n">
         <v>634</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="1" t="n">
         <v>45799</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -786,7 +774,7 @@
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="1" t="n">
         <v>45844</v>
       </c>
       <c r="I4" t="n">
@@ -835,7 +823,7 @@
       <c r="D5" t="n">
         <v>660</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -844,7 +832,7 @@
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="I5" t="n">
@@ -893,7 +881,7 @@
       <c r="D6" t="n">
         <v>661</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -905,7 +893,7 @@
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="1" t="n">
         <v>45891</v>
       </c>
       <c r="I6" t="n">
@@ -956,7 +944,7 @@
       <c r="D7" t="n">
         <v>688</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="1" t="n">
         <v>45901</v>
       </c>
       <c r="F7" t="inlineStr">
@@ -965,7 +953,7 @@
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="1" t="n">
         <v>45938</v>
       </c>
       <c r="I7" t="n">
@@ -1014,7 +1002,7 @@
       <c r="D8" t="n">
         <v>696</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="1" t="n">
         <v>45923</v>
       </c>
       <c r="F8" t="inlineStr">
@@ -1023,7 +1011,7 @@
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="1" t="n">
         <v>45938</v>
       </c>
       <c r="I8" t="n">
@@ -1072,7 +1060,7 @@
       <c r="D9" t="n">
         <v>704</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="1" t="n">
         <v>45957</v>
       </c>
       <c r="F9" t="inlineStr">
@@ -1082,7 +1070,7 @@
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="1" t="n">
         <v>46003</v>
       </c>
       <c r="I9" t="n">
@@ -1127,7 +1115,7 @@
       <c r="D10" t="n">
         <v>705</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="1" t="n">
         <v>45972</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -1136,7 +1124,7 @@
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="1" t="n">
         <v>46016</v>
       </c>
       <c r="I10" t="n">
@@ -1185,7 +1173,7 @@
       <c r="D11" t="n">
         <v>728</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="1" t="n">
         <v>46008</v>
       </c>
       <c r="F11" t="inlineStr">
@@ -1194,7 +1182,7 @@
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="1" t="n">
         <v>46040</v>
       </c>
       <c r="I11" t="n">
@@ -1243,7 +1231,7 @@
       <c r="D12" t="n">
         <v>278</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="1" t="n">
         <v>46042</v>
       </c>
       <c r="F12" t="inlineStr">
@@ -1252,7 +1240,7 @@
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" s="2" t="n">
+      <c r="H12" s="1" t="n">
         <v>46074</v>
       </c>
       <c r="I12" t="n">
@@ -1299,7 +1287,7 @@
       <c r="D13" t="n">
         <v>10</v>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="E13" s="1" t="n">
         <v>46078</v>
       </c>
       <c r="F13" t="inlineStr">
@@ -1308,7 +1296,7 @@
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" s="2" t="n">
+      <c r="H13" s="1" t="n">
         <v>46106</v>
       </c>
       <c r="I13" t="n">
@@ -1353,7 +1341,7 @@
       <c r="D14" t="n">
         <v>15</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="1" t="n">
         <v>46094</v>
       </c>
       <c r="F14" t="inlineStr">
@@ -1362,7 +1350,7 @@
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" s="2" t="n">
+      <c r="H14" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="I14" t="n">
@@ -1409,7 +1397,7 @@
       <c r="D15" t="n">
         <v>28</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E15" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="F15" t="inlineStr">
@@ -1418,7 +1406,7 @@
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" s="2" t="n">
+      <c r="H15" s="1" t="n">
         <v>46164</v>
       </c>
       <c r="I15" t="n">
@@ -1465,7 +1453,7 @@
       <c r="D16" t="n">
         <v>33</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="1" t="n">
         <v>46156</v>
       </c>
       <c r="F16" t="inlineStr">
@@ -1474,7 +1462,7 @@
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" s="2" t="n">
+      <c r="H16" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="I16" t="n">
@@ -1521,7 +1509,7 @@
       <c r="D17" t="n">
         <v>29</v>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E17" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="F17" t="inlineStr">
@@ -1530,7 +1518,7 @@
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" s="2" t="n">
+      <c r="H17" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="I17" t="n">
@@ -1577,7 +1565,7 @@
       <c r="D18" t="n">
         <v>40</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="1" t="n">
         <v>46156</v>
       </c>
       <c r="F18" t="inlineStr">
@@ -1586,7 +1574,7 @@
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" s="2" t="n">
+      <c r="H18" s="1" t="n">
         <v>46191</v>
       </c>
       <c r="I18" t="n">
@@ -1633,7 +1621,7 @@
       <c r="D19" t="n">
         <v>402</v>
       </c>
-      <c r="E19" s="2" t="n">
+      <c r="E19" s="1" t="n">
         <v>45791</v>
       </c>
       <c r="F19" t="inlineStr">
@@ -1642,7 +1630,7 @@
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" s="2" t="n">
+      <c r="H19" s="1" t="n">
         <v>45834</v>
       </c>
       <c r="I19" t="n">
@@ -1689,7 +1677,7 @@
       <c r="D20" t="n">
         <v>447</v>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="1" t="n">
         <v>45814</v>
       </c>
       <c r="F20" t="inlineStr">
@@ -1698,7 +1686,7 @@
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" s="2" t="n">
+      <c r="H20" s="1" t="n">
         <v>45955</v>
       </c>
       <c r="I20" t="n">
@@ -1749,7 +1737,7 @@
       <c r="D21" t="n">
         <v>529</v>
       </c>
-      <c r="E21" s="2" t="n">
+      <c r="E21" s="1" t="n">
         <v>45853</v>
       </c>
       <c r="F21" t="inlineStr">
@@ -1758,7 +1746,7 @@
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" s="2" t="n">
+      <c r="H21" s="1" t="n">
         <v>45939</v>
       </c>
       <c r="I21" t="n">
@@ -1809,7 +1797,7 @@
       <c r="D22" t="n">
         <v>691</v>
       </c>
-      <c r="E22" s="2" t="n">
+      <c r="E22" s="1" t="n">
         <v>45910</v>
       </c>
       <c r="F22" t="inlineStr">
@@ -1818,7 +1806,7 @@
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" s="2" t="n">
+      <c r="H22" s="1" t="n">
         <v>45941</v>
       </c>
       <c r="I22" t="n">
@@ -1867,7 +1855,7 @@
       <c r="D23" t="n">
         <v>677</v>
       </c>
-      <c r="E23" s="2" t="n">
+      <c r="E23" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="F23" t="inlineStr">
@@ -1876,7 +1864,7 @@
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" s="2" t="n">
+      <c r="H23" s="1" t="n">
         <v>45935</v>
       </c>
       <c r="I23" t="n">
@@ -1923,7 +1911,7 @@
       <c r="D24" t="n">
         <v>278</v>
       </c>
-      <c r="E24" s="2" t="n">
+      <c r="E24" s="1" t="n">
         <v>46008</v>
       </c>
       <c r="F24" t="inlineStr">
@@ -1932,7 +1920,7 @@
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" s="2" t="n">
+      <c r="H24" s="1" t="n">
         <v>46066</v>
       </c>
       <c r="I24" t="n">
@@ -1981,7 +1969,7 @@
       <c r="D25" t="n">
         <v>748</v>
       </c>
-      <c r="E25" s="2" t="n">
+      <c r="E25" s="1" t="n">
         <v>45930</v>
       </c>
       <c r="F25" t="inlineStr">
@@ -1990,7 +1978,7 @@
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" s="2" t="n">
+      <c r="H25" s="1" t="n">
         <v>45935</v>
       </c>
       <c r="I25" t="n">
@@ -2037,7 +2025,7 @@
       <c r="D26" t="n">
         <v>822</v>
       </c>
-      <c r="E26" s="2" t="n">
+      <c r="E26" s="1" t="n">
         <v>45968</v>
       </c>
       <c r="F26" t="inlineStr">
@@ -2046,7 +2034,7 @@
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" s="2" t="n">
+      <c r="H26" s="1" t="n">
         <v>45935</v>
       </c>
       <c r="I26" t="n">
@@ -2093,7 +2081,7 @@
       <c r="D27" t="n">
         <v>360</v>
       </c>
-      <c r="E27" s="2" t="n">
+      <c r="E27" s="1" t="n">
         <v>46043</v>
       </c>
       <c r="F27" t="inlineStr">
@@ -2102,7 +2090,7 @@
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
-      <c r="H27" s="2" t="n">
+      <c r="H27" s="1" t="n">
         <v>46075</v>
       </c>
       <c r="I27" t="n">
@@ -2223,7 +2211,7 @@
       <c r="D30" t="n">
         <v>1465</v>
       </c>
-      <c r="E30" s="2" t="n">
+      <c r="E30" s="1" t="n">
         <v>46104</v>
       </c>
       <c r="F30" t="inlineStr">
@@ -2232,7 +2220,7 @@
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" s="2" t="n">
+      <c r="H30" s="1" t="n">
         <v>46106</v>
       </c>
       <c r="I30" t="n">
@@ -2275,27 +2263,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>numero_empenho</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>valor_empenhado</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>saldo</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>responsavel</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>justificativa</t>
         </is>

</xml_diff>

<commit_message>
Atualização manual: Pagamentos (18/07/2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="145">
   <si>
     <t>numero_contrato</t>
   </si>
@@ -169,6 +169,9 @@
   </si>
   <si>
     <t>MAIO/26</t>
+  </si>
+  <si>
+    <t>JUNHO/26</t>
   </si>
   <si>
     <t>Módulo II – Parcial Orçamento 10 (FAB 2728)</t>
@@ -334,6 +337,9 @@
     <t>2026NP402373</t>
   </si>
   <si>
+    <t>Faturado</t>
+  </si>
+  <si>
     <t>2025NP002620</t>
   </si>
   <si>
@@ -361,6 +367,9 @@
     <t>2026NP400445</t>
   </si>
   <si>
+    <t>2026NP401058</t>
+  </si>
+  <si>
     <t>mensal</t>
   </si>
   <si>
@@ -371,9 +380,6 @@
   </si>
   <si>
     <t>Pendente</t>
-  </si>
-  <si>
-    <t>Faturado, aguardando pagamento</t>
   </si>
   <si>
     <t>numero_empenho</t>
@@ -458,8 +464,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -475,7 +489,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -483,12 +497,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -788,37 +820,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -864,62 +896,62 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R30"/>
+  <dimension ref="A1:R31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -931,34 +963,34 @@
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
-        <v>66</v>
-      </c>
-      <c r="H2" s="1">
+        <v>67</v>
+      </c>
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
         <v>748504.24</v>
       </c>
       <c r="J2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K2">
         <v>748504.24</v>
       </c>
       <c r="M2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="P2">
         <v>881914.1800000001</v>
@@ -972,34 +1004,34 @@
         <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
-        <v>67</v>
-      </c>
-      <c r="H3" s="1">
+        <v>68</v>
+      </c>
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
         <v>1110378.24</v>
       </c>
       <c r="J3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K3">
         <v>1110378.24</v>
       </c>
       <c r="M3" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="P3">
         <v>2634000</v>
@@ -1013,34 +1045,34 @@
         <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
-        <v>68</v>
-      </c>
-      <c r="H4" s="1">
+        <v>69</v>
+      </c>
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
         <v>974557.12</v>
       </c>
       <c r="J4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K4">
         <v>974557.12</v>
       </c>
       <c r="M4" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="P4">
         <v>1686034.96</v>
@@ -1054,34 +1086,34 @@
         <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
-        <v>69</v>
-      </c>
-      <c r="H5" s="1">
+        <v>70</v>
+      </c>
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
         <v>1402001.34</v>
       </c>
       <c r="J5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K5">
         <v>1402001.34</v>
       </c>
       <c r="M5" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N5" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="P5">
         <v>1600334.09</v>
@@ -1095,34 +1127,34 @@
         <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
-        <v>70</v>
-      </c>
-      <c r="H6" s="1">
+        <v>71</v>
+      </c>
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
         <v>1223702.3</v>
       </c>
       <c r="J6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K6">
         <v>1223702.3</v>
       </c>
       <c r="M6" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N6" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="O6">
         <v>0.02</v>
@@ -1139,34 +1171,34 @@
         <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
-        <v>71</v>
-      </c>
-      <c r="H7" s="1">
+        <v>72</v>
+      </c>
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
         <v>1011677.95</v>
       </c>
       <c r="J7" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="K7">
         <v>1011677.95</v>
       </c>
       <c r="M7" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N7" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="P7">
         <v>2568571.48</v>
@@ -1180,34 +1212,34 @@
         <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
-        <v>72</v>
-      </c>
-      <c r="H8" s="1">
+        <v>73</v>
+      </c>
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
         <v>896744.0600000001</v>
       </c>
       <c r="J8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="K8">
         <v>896744.0600000001</v>
       </c>
       <c r="M8" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N8" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="P8">
         <v>968237.39</v>
@@ -1221,34 +1253,34 @@
         <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H9" s="1">
+        <v>74</v>
+      </c>
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
         <v>919329.0600000001</v>
       </c>
       <c r="J9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K9">
         <v>919329.0600000001</v>
       </c>
       <c r="M9" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N9" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="P9">
         <v>1947932.74</v>
@@ -1264,29 +1296,29 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
-        <v>74</v>
-      </c>
-      <c r="H10" s="1">
+        <v>75</v>
+      </c>
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
         <v>1157009.26</v>
       </c>
       <c r="J10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K10">
         <v>1157009.26</v>
       </c>
       <c r="M10" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="P10">
         <v>3105605.8</v>
@@ -1300,34 +1332,34 @@
         <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
-        <v>75</v>
-      </c>
-      <c r="H11" s="1">
+        <v>76</v>
+      </c>
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
         <v>1214597.952</v>
       </c>
       <c r="J11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K11">
         <v>1214597.952</v>
       </c>
       <c r="M11" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N11" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="P11">
         <v>2096487.74</v>
@@ -1341,34 +1373,34 @@
         <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
-        <v>76</v>
-      </c>
-      <c r="H12" s="1">
+        <v>77</v>
+      </c>
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
         <v>967082.09</v>
       </c>
       <c r="J12" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K12">
         <v>967082.09</v>
       </c>
       <c r="M12" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N12" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="O12">
         <v>497601.53</v>
@@ -1387,29 +1419,29 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
-        <v>77</v>
-      </c>
-      <c r="H13" s="1">
+        <v>78</v>
+      </c>
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
         <v>719561.08</v>
       </c>
       <c r="J13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K13">
         <v>719561.08</v>
       </c>
       <c r="M13" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N13" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="P13">
         <v>1500000</v>
@@ -1425,29 +1457,29 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
-        <v>78</v>
-      </c>
-      <c r="H14" s="1">
+        <v>79</v>
+      </c>
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
         <v>885881.08</v>
       </c>
       <c r="J14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K14">
         <v>885881.08</v>
       </c>
       <c r="M14" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N14" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="O14">
         <v>34065.36</v>
@@ -1466,29 +1498,29 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
-        <v>79</v>
-      </c>
-      <c r="H15" s="1">
+        <v>80</v>
+      </c>
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
         <v>1350542.52</v>
       </c>
       <c r="J15" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K15">
         <v>1350542.52</v>
       </c>
       <c r="M15" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N15" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="O15">
         <v>0.01</v>
@@ -1507,29 +1539,29 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
-        <v>80</v>
-      </c>
-      <c r="H16" s="1">
+        <v>81</v>
+      </c>
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
         <v>1108954.435833333</v>
       </c>
       <c r="J16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K16">
         <v>1108954.435833333</v>
       </c>
       <c r="M16" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N16" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="O16">
         <v>497601.54</v>
@@ -1548,29 +1580,29 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
-        <v>80</v>
-      </c>
-      <c r="H17" s="1">
+        <v>81</v>
+      </c>
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
         <v>218206.1</v>
       </c>
       <c r="J17" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K17">
         <v>218206.1</v>
       </c>
       <c r="M17" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N17" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="O17">
         <v>497601.54</v>
@@ -1589,29 +1621,29 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
-        <v>80</v>
-      </c>
-      <c r="H18" s="1">
+        <v>81</v>
+      </c>
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
         <v>1549250.84</v>
       </c>
       <c r="J18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K18">
         <v>1549250.84</v>
       </c>
       <c r="M18" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="N18" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="O18">
         <v>497601.54</v>
@@ -1622,40 +1654,22 @@
     </row>
     <row r="19" spans="1:16">
       <c r="A19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B19" t="s">
         <v>51</v>
       </c>
-      <c r="D19">
-        <v>402</v>
-      </c>
-      <c r="E19" s="1">
-        <v>45791</v>
-      </c>
-      <c r="F19" t="s">
-        <v>81</v>
-      </c>
-      <c r="H19" s="1">
-        <v>45834</v>
-      </c>
-      <c r="I19">
-        <v>188246.17</v>
-      </c>
       <c r="J19" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K19">
-        <v>188246.17</v>
+        <v>1340865.98</v>
       </c>
       <c r="M19" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="N19" t="s">
-        <v>115</v>
-      </c>
-      <c r="P19">
-        <v>211614.23</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" spans="1:16">
@@ -1665,41 +1679,35 @@
       <c r="B20" t="s">
         <v>52</v>
       </c>
-      <c r="C20">
-        <v>46</v>
-      </c>
       <c r="D20">
-        <v>447</v>
-      </c>
-      <c r="E20" s="1">
-        <v>45814</v>
+        <v>402</v>
+      </c>
+      <c r="E20" s="2">
+        <v>45791</v>
       </c>
       <c r="F20" t="s">
         <v>82</v>
       </c>
-      <c r="H20" s="1">
-        <v>45955</v>
+      <c r="H20" s="2">
+        <v>45834</v>
       </c>
       <c r="I20">
-        <v>112720.77</v>
+        <v>188246.17</v>
       </c>
       <c r="J20" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K20">
-        <v>112720.77</v>
+        <v>188246.17</v>
       </c>
       <c r="M20" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="N20" t="s">
-        <v>115</v>
-      </c>
-      <c r="O20">
-        <v>0.01</v>
+        <v>118</v>
       </c>
       <c r="P20">
-        <v>3359394.8</v>
+        <v>211614.23</v>
       </c>
     </row>
     <row r="21" spans="1:16">
@@ -1709,41 +1717,41 @@
       <c r="B21" t="s">
         <v>53</v>
       </c>
-      <c r="C21" t="s">
-        <v>64</v>
+      <c r="C21">
+        <v>46</v>
       </c>
       <c r="D21">
-        <v>529</v>
-      </c>
-      <c r="E21" s="1">
-        <v>45853</v>
+        <v>447</v>
+      </c>
+      <c r="E21" s="2">
+        <v>45814</v>
       </c>
       <c r="F21" t="s">
         <v>83</v>
       </c>
-      <c r="H21" s="1">
-        <v>45939</v>
+      <c r="H21" s="2">
+        <v>45955</v>
       </c>
       <c r="I21">
-        <v>378307.61</v>
+        <v>112720.77</v>
       </c>
       <c r="J21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K21">
-        <v>378307.61</v>
+        <v>112720.77</v>
       </c>
       <c r="M21" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="N21" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="O21">
         <v>0.01</v>
       </c>
       <c r="P21">
-        <v>2391157.41</v>
+        <v>3359394.8</v>
       </c>
     </row>
     <row r="22" spans="1:16">
@@ -1754,34 +1762,34 @@
         <v>54</v>
       </c>
       <c r="C22" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D22">
-        <v>691</v>
-      </c>
-      <c r="E22" s="1">
-        <v>45910</v>
+        <v>529</v>
+      </c>
+      <c r="E22" s="2">
+        <v>45853</v>
       </c>
       <c r="F22" t="s">
-        <v>83</v>
-      </c>
-      <c r="H22" s="1">
-        <v>45941</v>
+        <v>84</v>
+      </c>
+      <c r="H22" s="2">
+        <v>45939</v>
       </c>
       <c r="I22">
-        <v>3315.047100000025</v>
+        <v>378307.61</v>
       </c>
       <c r="J22" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K22">
-        <v>3315.04710000003</v>
+        <v>378307.61</v>
       </c>
       <c r="M22" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="N22" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="O22">
         <v>0.01</v>
@@ -1797,38 +1805,41 @@
       <c r="B23" t="s">
         <v>55</v>
       </c>
-      <c r="C23">
-        <v>135</v>
+      <c r="C23" t="s">
+        <v>65</v>
       </c>
       <c r="D23">
-        <v>677</v>
-      </c>
-      <c r="E23" s="1">
-        <v>45904</v>
+        <v>691</v>
+      </c>
+      <c r="E23" s="2">
+        <v>45910</v>
       </c>
       <c r="F23" t="s">
-        <v>69</v>
-      </c>
-      <c r="H23" s="1">
-        <v>45935</v>
+        <v>84</v>
+      </c>
+      <c r="H23" s="2">
+        <v>45941</v>
       </c>
       <c r="I23">
-        <v>198332.75</v>
+        <v>3315.047100000025</v>
       </c>
       <c r="J23" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K23">
-        <v>198332.75</v>
+        <v>3315.04710000003</v>
       </c>
       <c r="M23" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="N23" t="s">
-        <v>115</v>
+        <v>118</v>
+      </c>
+      <c r="O23">
+        <v>0.01</v>
       </c>
       <c r="P23">
-        <v>1600334.09</v>
+        <v>2391157.41</v>
       </c>
     </row>
     <row r="24" spans="1:16">
@@ -1839,37 +1850,37 @@
         <v>56</v>
       </c>
       <c r="C24">
-        <v>40</v>
+        <v>135</v>
       </c>
       <c r="D24">
-        <v>278</v>
-      </c>
-      <c r="E24" s="1">
-        <v>46008</v>
+        <v>677</v>
+      </c>
+      <c r="E24" s="2">
+        <v>45904</v>
       </c>
       <c r="F24" t="s">
-        <v>84</v>
-      </c>
-      <c r="H24" s="1">
-        <v>46066</v>
+        <v>70</v>
+      </c>
+      <c r="H24" s="2">
+        <v>45935</v>
       </c>
       <c r="I24">
-        <v>1528.62</v>
+        <v>198332.75</v>
       </c>
       <c r="J24" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="K24">
-        <v>1528.62</v>
+        <v>198332.75</v>
       </c>
       <c r="M24" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="N24" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="P24">
-        <v>1157673.06</v>
+        <v>1600334.09</v>
       </c>
     </row>
     <row r="25" spans="1:16">
@@ -1879,38 +1890,38 @@
       <c r="B25" t="s">
         <v>57</v>
       </c>
-      <c r="C25" t="s">
-        <v>65</v>
+      <c r="C25">
+        <v>40</v>
       </c>
       <c r="D25">
-        <v>748</v>
-      </c>
-      <c r="E25" s="1">
-        <v>45930</v>
+        <v>278</v>
+      </c>
+      <c r="E25" s="2">
+        <v>46008</v>
       </c>
       <c r="F25" t="s">
         <v>85</v>
       </c>
-      <c r="H25" s="1">
-        <v>45935</v>
+      <c r="H25" s="2">
+        <v>46066</v>
       </c>
       <c r="I25">
-        <v>38718.58</v>
+        <v>1528.62</v>
       </c>
       <c r="J25" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K25">
-        <v>38718.58</v>
+        <v>1528.62</v>
       </c>
       <c r="M25" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="N25" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="P25">
-        <v>63746.85</v>
+        <v>1157673.06</v>
       </c>
     </row>
     <row r="26" spans="1:16">
@@ -1920,38 +1931,38 @@
       <c r="B26" t="s">
         <v>58</v>
       </c>
-      <c r="C26">
-        <v>154</v>
+      <c r="C26" t="s">
+        <v>66</v>
       </c>
       <c r="D26">
-        <v>822</v>
-      </c>
-      <c r="E26" s="1">
-        <v>45968</v>
+        <v>748</v>
+      </c>
+      <c r="E26" s="2">
+        <v>45930</v>
       </c>
       <c r="F26" t="s">
         <v>86</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45935</v>
       </c>
       <c r="I26">
-        <v>133124.11</v>
+        <v>38718.58</v>
       </c>
       <c r="J26" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="K26">
-        <v>133124.11</v>
+        <v>38718.58</v>
       </c>
       <c r="M26" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="N26" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="P26">
-        <v>1000001.64</v>
+        <v>63746.85</v>
       </c>
     </row>
     <row r="27" spans="1:16">
@@ -1962,37 +1973,37 @@
         <v>59</v>
       </c>
       <c r="C27">
-        <v>252</v>
+        <v>154</v>
       </c>
       <c r="D27">
-        <v>360</v>
-      </c>
-      <c r="E27" s="1">
-        <v>46043</v>
+        <v>822</v>
+      </c>
+      <c r="E27" s="2">
+        <v>45968</v>
       </c>
       <c r="F27" t="s">
-        <v>77</v>
-      </c>
-      <c r="H27" s="1">
-        <v>46075</v>
+        <v>87</v>
+      </c>
+      <c r="H27" s="2">
+        <v>45935</v>
       </c>
       <c r="I27">
-        <v>11372.9</v>
+        <v>133124.11</v>
       </c>
       <c r="J27" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K27">
-        <v>11372.9</v>
+        <v>133124.11</v>
       </c>
       <c r="M27" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="N27" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="P27">
-        <v>1500000</v>
+        <v>1000001.64</v>
       </c>
     </row>
     <row r="28" spans="1:16">
@@ -2002,17 +2013,38 @@
       <c r="B28" t="s">
         <v>60</v>
       </c>
-      <c r="G28" t="s">
-        <v>87</v>
-      </c>
-      <c r="L28">
-        <v>15854.78</v>
+      <c r="C28">
+        <v>252</v>
+      </c>
+      <c r="D28">
+        <v>360</v>
+      </c>
+      <c r="E28" s="2">
+        <v>46043</v>
+      </c>
+      <c r="F28" t="s">
+        <v>78</v>
+      </c>
+      <c r="H28" s="2">
+        <v>46075</v>
+      </c>
+      <c r="I28">
+        <v>11372.9</v>
+      </c>
+      <c r="J28" t="s">
+        <v>114</v>
+      </c>
+      <c r="K28">
+        <v>11372.9</v>
       </c>
       <c r="M28" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="N28" t="s">
-        <v>116</v>
+        <v>118</v>
+      </c>
+      <c r="P28">
+        <v>1500000</v>
       </c>
     </row>
     <row r="29" spans="1:16">
@@ -2022,48 +2054,74 @@
       <c r="B29" t="s">
         <v>61</v>
       </c>
+      <c r="G29" t="s">
+        <v>88</v>
+      </c>
       <c r="L29">
-        <v>24962.38</v>
+        <v>15854.78</v>
       </c>
       <c r="M29" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="N29" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="30" spans="1:16">
       <c r="A30">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B30" t="s">
         <v>62</v>
       </c>
-      <c r="D30">
+      <c r="G30" t="s">
+        <v>88</v>
+      </c>
+      <c r="L30">
+        <v>24962.38</v>
+      </c>
+      <c r="M30" t="s">
+        <v>117</v>
+      </c>
+      <c r="N30" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16">
+      <c r="A31">
+        <v>3</v>
+      </c>
+      <c r="B31" t="s">
+        <v>63</v>
+      </c>
+      <c r="D31">
         <v>1465</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E31" s="2">
         <v>46104</v>
       </c>
-      <c r="F30" t="s">
-        <v>77</v>
-      </c>
-      <c r="H30" s="1">
+      <c r="F31" t="s">
+        <v>78</v>
+      </c>
+      <c r="H31" s="2">
         <v>46106</v>
       </c>
-      <c r="I30">
+      <c r="I31">
         <v>27801.11</v>
       </c>
-      <c r="K30">
+      <c r="J31" t="s">
+        <v>115</v>
+      </c>
+      <c r="K31">
         <v>27801.11</v>
       </c>
-      <c r="M30" t="s">
-        <v>114</v>
-      </c>
-      <c r="N30" t="s">
+      <c r="M31" t="s">
         <v>117</v>
       </c>
-      <c r="P30">
+      <c r="N31" t="s">
+        <v>118</v>
+      </c>
+      <c r="P31">
         <v>1500000</v>
       </c>
     </row>
@@ -2078,25 +2136,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
-        <v>118</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
-        <v>119</v>
-      </c>
-      <c r="D1" t="s">
-        <v>120</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="C1" s="1" t="s">
         <v>121</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B2">
         <v>52250.04</v>
@@ -2107,7 +2165,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B3">
         <v>881914.1800000001</v>
@@ -2118,7 +2176,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B4">
         <v>750000</v>
@@ -2129,7 +2187,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B5">
         <v>949835.78</v>
@@ -2140,7 +2198,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B6">
         <v>524584.95</v>
@@ -2151,7 +2209,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B7">
         <v>211614.23</v>
@@ -2162,7 +2220,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B8">
         <v>2391157.41</v>
@@ -2173,7 +2231,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B9">
         <v>618154.38</v>
@@ -2184,7 +2242,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B10">
         <v>1600334.09</v>
@@ -2195,7 +2253,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B11">
         <v>1867169.54</v>
@@ -2206,7 +2264,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B12">
         <v>968237.39</v>
@@ -2217,7 +2275,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B13">
         <v>1011677.95</v>
@@ -2228,7 +2286,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B14">
         <v>1580293.02</v>
@@ -2239,7 +2297,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -2250,7 +2308,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B16">
         <v>63746.85</v>
@@ -2261,7 +2319,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B17">
         <v>947931.1</v>
@@ -2272,7 +2330,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B18">
         <v>259790.57</v>
@@ -2283,7 +2341,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B19">
         <v>170479.3</v>
@@ -2294,7 +2352,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B20">
         <v>1500000</v>
@@ -2305,7 +2363,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B21">
         <v>1000001.64</v>
@@ -2316,7 +2374,7 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B22">
         <v>68405.66</v>
@@ -2327,7 +2385,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B23">
         <v>1157673.06</v>
@@ -2338,7 +2396,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B24">
         <v>34065.36</v>
@@ -2349,7 +2407,7 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -2360,7 +2418,7 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -2371,7 +2429,7 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -2382,7 +2440,7 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B28">
         <v>0</v>
@@ -2393,7 +2451,7 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -2404,7 +2462,7 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B30">
         <v>0</v>

</xml_diff>

<commit_message>
Corrige lançamento de pagamento que não aparecia (limites de bloco fixos)
"Módulo III – Orçamento 19 GPS" (NF 1882, empenho 2025NE001065) tinha sido
acrescentado como linha nova na planilha original, mas a extração parava
num número de linha fixo que não incluía essa linha. Blocos agora são
descobertos dinamicamente (procura os cabeçalhos "Referência" + fim por
sequência em branco), sobrevivendo a linhas novas no futuro sem precisar
mexer no código.

De quebra, corrige a classificação de "situação": um valor tipo "Faturado"
(texto, sem número de ordem) na coluna "Ordem de Pagamento" caía como
"Pago" por engano — agora só conta como Pago quando bate o padrão real de
ordem (AAAANPnnnnnn). Afetava também o lançamento "JUNHO/26".

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="147">
   <si>
     <t>numero_contrato</t>
   </si>
@@ -208,6 +208,9 @@
   </si>
   <si>
     <t>Módulo III – Orçamento 17 Manuais</t>
+  </si>
+  <si>
+    <t>Módulo III – Orçamento 19 GPS</t>
   </si>
   <si>
     <t>-</t>
@@ -286,6 +289,9 @@
     <t>2025NE001828</t>
   </si>
   <si>
+    <t>2025NE001065</t>
+  </si>
+  <si>
     <t>Aprovado e aguardando itens</t>
   </si>
   <si>
@@ -379,6 +385,9 @@
     <t>Pago</t>
   </si>
   <si>
+    <t>Faturado, aguardando pagamento</t>
+  </si>
+  <si>
     <t>Pendente</t>
   </si>
   <si>
@@ -410,9 +419,6 @@
   </si>
   <si>
     <t>2025NE000774</t>
-  </si>
-  <si>
-    <t>2025NE001065</t>
   </si>
   <si>
     <t>2025NE001598</t>
@@ -896,7 +902,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R31"/>
+  <dimension ref="A1:R32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
@@ -963,7 +969,7 @@
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D2">
         <v>594</v>
@@ -972,7 +978,7 @@
         <v>45740</v>
       </c>
       <c r="F2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H2" s="2">
         <v>45778</v>
@@ -981,16 +987,16 @@
         <v>748504.24</v>
       </c>
       <c r="J2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="K2">
         <v>748504.24</v>
       </c>
       <c r="M2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P2">
         <v>881914.1800000001</v>
@@ -1004,7 +1010,7 @@
         <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D3">
         <v>620</v>
@@ -1013,7 +1019,7 @@
         <v>45775</v>
       </c>
       <c r="F3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H3" s="2">
         <v>45806</v>
@@ -1022,16 +1028,16 @@
         <v>1110378.24</v>
       </c>
       <c r="J3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="K3">
         <v>1110378.24</v>
       </c>
       <c r="M3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P3">
         <v>2634000</v>
@@ -1045,7 +1051,7 @@
         <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D4">
         <v>634</v>
@@ -1054,7 +1060,7 @@
         <v>45799</v>
       </c>
       <c r="F4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H4" s="2">
         <v>45844</v>
@@ -1063,16 +1069,16 @@
         <v>974557.12</v>
       </c>
       <c r="J4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="K4">
         <v>974557.12</v>
       </c>
       <c r="M4" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N4" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P4">
         <v>1686034.96</v>
@@ -1086,7 +1092,7 @@
         <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D5">
         <v>660</v>
@@ -1095,7 +1101,7 @@
         <v>45856</v>
       </c>
       <c r="F5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H5" s="2">
         <v>45891</v>
@@ -1104,16 +1110,16 @@
         <v>1402001.34</v>
       </c>
       <c r="J5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="K5">
         <v>1402001.34</v>
       </c>
       <c r="M5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P5">
         <v>1600334.09</v>
@@ -1127,7 +1133,7 @@
         <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D6">
         <v>661</v>
@@ -1136,7 +1142,7 @@
         <v>45856</v>
       </c>
       <c r="F6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H6" s="2">
         <v>45891</v>
@@ -1145,16 +1151,16 @@
         <v>1223702.3</v>
       </c>
       <c r="J6" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="K6">
         <v>1223702.3</v>
       </c>
       <c r="M6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="O6">
         <v>0.02</v>
@@ -1171,7 +1177,7 @@
         <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D7">
         <v>688</v>
@@ -1180,7 +1186,7 @@
         <v>45901</v>
       </c>
       <c r="F7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H7" s="2">
         <v>45938</v>
@@ -1189,16 +1195,16 @@
         <v>1011677.95</v>
       </c>
       <c r="J7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="K7">
         <v>1011677.95</v>
       </c>
       <c r="M7" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N7" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P7">
         <v>2568571.48</v>
@@ -1212,7 +1218,7 @@
         <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D8">
         <v>696</v>
@@ -1221,7 +1227,7 @@
         <v>45923</v>
       </c>
       <c r="F8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H8" s="2">
         <v>45938</v>
@@ -1230,16 +1236,16 @@
         <v>896744.0600000001</v>
       </c>
       <c r="J8" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="K8">
         <v>896744.0600000001</v>
       </c>
       <c r="M8" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P8">
         <v>968237.39</v>
@@ -1253,7 +1259,7 @@
         <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D9">
         <v>704</v>
@@ -1262,7 +1268,7 @@
         <v>45957</v>
       </c>
       <c r="F9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H9" s="2">
         <v>46003</v>
@@ -1271,16 +1277,16 @@
         <v>919329.0600000001</v>
       </c>
       <c r="J9" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="K9">
         <v>919329.0600000001</v>
       </c>
       <c r="M9" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N9" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P9">
         <v>1947932.74</v>
@@ -1300,7 +1306,7 @@
         <v>45972</v>
       </c>
       <c r="F10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H10" s="2">
         <v>46016</v>
@@ -1309,16 +1315,16 @@
         <v>1157009.26</v>
       </c>
       <c r="J10" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="K10">
         <v>1157009.26</v>
       </c>
       <c r="M10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P10">
         <v>3105605.8</v>
@@ -1332,7 +1338,7 @@
         <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D11">
         <v>728</v>
@@ -1341,7 +1347,7 @@
         <v>46008</v>
       </c>
       <c r="F11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H11" s="2">
         <v>46040</v>
@@ -1350,16 +1356,16 @@
         <v>1214597.952</v>
       </c>
       <c r="J11" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="K11">
         <v>1214597.952</v>
       </c>
       <c r="M11" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N11" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P11">
         <v>2096487.74</v>
@@ -1373,7 +1379,7 @@
         <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D12">
         <v>278</v>
@@ -1382,7 +1388,7 @@
         <v>46042</v>
       </c>
       <c r="F12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H12" s="2">
         <v>46074</v>
@@ -1391,16 +1397,16 @@
         <v>967082.09</v>
       </c>
       <c r="J12" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="K12">
         <v>967082.09</v>
       </c>
       <c r="M12" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N12" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="O12">
         <v>497601.53</v>
@@ -1423,7 +1429,7 @@
         <v>46078</v>
       </c>
       <c r="F13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H13" s="2">
         <v>46106</v>
@@ -1432,16 +1438,16 @@
         <v>719561.08</v>
       </c>
       <c r="J13" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="K13">
         <v>719561.08</v>
       </c>
       <c r="M13" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P13">
         <v>1500000</v>
@@ -1461,7 +1467,7 @@
         <v>46094</v>
       </c>
       <c r="F14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H14" s="2">
         <v>46128</v>
@@ -1470,16 +1476,16 @@
         <v>885881.08</v>
       </c>
       <c r="J14" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="K14">
         <v>885881.08</v>
       </c>
       <c r="M14" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N14" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="O14">
         <v>34065.36</v>
@@ -1502,7 +1508,7 @@
         <v>46128</v>
       </c>
       <c r="F15" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H15" s="2">
         <v>46164</v>
@@ -1511,16 +1517,16 @@
         <v>1350542.52</v>
       </c>
       <c r="J15" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="K15">
         <v>1350542.52</v>
       </c>
       <c r="M15" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N15" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="O15">
         <v>0.01</v>
@@ -1543,7 +1549,7 @@
         <v>46156</v>
       </c>
       <c r="F16" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H16" s="2">
         <v>46191</v>
@@ -1552,16 +1558,16 @@
         <v>1108954.435833333</v>
       </c>
       <c r="J16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="K16">
         <v>1108954.435833333</v>
       </c>
       <c r="M16" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N16" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="O16">
         <v>497601.54</v>
@@ -1584,7 +1590,7 @@
         <v>46149</v>
       </c>
       <c r="F17" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H17" s="2">
         <v>46185</v>
@@ -1593,16 +1599,16 @@
         <v>218206.1</v>
       </c>
       <c r="J17" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="K17">
         <v>218206.1</v>
       </c>
       <c r="M17" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N17" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="O17">
         <v>497601.54</v>
@@ -1625,7 +1631,7 @@
         <v>46156</v>
       </c>
       <c r="F18" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H18" s="2">
         <v>46191</v>
@@ -1634,16 +1640,16 @@
         <v>1549250.84</v>
       </c>
       <c r="J18" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K18">
         <v>1549250.84</v>
       </c>
       <c r="M18" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N18" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="O18">
         <v>497601.54</v>
@@ -1660,16 +1666,16 @@
         <v>51</v>
       </c>
       <c r="J19" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="K19">
         <v>1340865.98</v>
       </c>
       <c r="M19" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="N19" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="20" spans="1:16">
@@ -1686,7 +1692,7 @@
         <v>45791</v>
       </c>
       <c r="F20" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H20" s="2">
         <v>45834</v>
@@ -1695,16 +1701,16 @@
         <v>188246.17</v>
       </c>
       <c r="J20" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="K20">
         <v>188246.17</v>
       </c>
       <c r="M20" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="N20" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P20">
         <v>211614.23</v>
@@ -1727,7 +1733,7 @@
         <v>45814</v>
       </c>
       <c r="F21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H21" s="2">
         <v>45955</v>
@@ -1736,16 +1742,16 @@
         <v>112720.77</v>
       </c>
       <c r="J21" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="K21">
         <v>112720.77</v>
       </c>
       <c r="M21" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="N21" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="O21">
         <v>0.01</v>
@@ -1762,7 +1768,7 @@
         <v>54</v>
       </c>
       <c r="C22" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D22">
         <v>529</v>
@@ -1771,7 +1777,7 @@
         <v>45853</v>
       </c>
       <c r="F22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H22" s="2">
         <v>45939</v>
@@ -1780,16 +1786,16 @@
         <v>378307.61</v>
       </c>
       <c r="J22" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K22">
         <v>378307.61</v>
       </c>
       <c r="M22" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="N22" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="O22">
         <v>0.01</v>
@@ -1806,7 +1812,7 @@
         <v>55</v>
       </c>
       <c r="C23" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D23">
         <v>691</v>
@@ -1815,7 +1821,7 @@
         <v>45910</v>
       </c>
       <c r="F23" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H23" s="2">
         <v>45941</v>
@@ -1824,16 +1830,16 @@
         <v>3315.047100000025</v>
       </c>
       <c r="J23" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="K23">
         <v>3315.04710000003</v>
       </c>
       <c r="M23" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="N23" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="O23">
         <v>0.01</v>
@@ -1859,7 +1865,7 @@
         <v>45904</v>
       </c>
       <c r="F24" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H24" s="2">
         <v>45935</v>
@@ -1868,16 +1874,16 @@
         <v>198332.75</v>
       </c>
       <c r="J24" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="K24">
         <v>198332.75</v>
       </c>
       <c r="M24" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="N24" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P24">
         <v>1600334.09</v>
@@ -1900,7 +1906,7 @@
         <v>46008</v>
       </c>
       <c r="F25" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H25" s="2">
         <v>46066</v>
@@ -1909,16 +1915,16 @@
         <v>1528.62</v>
       </c>
       <c r="J25" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="K25">
         <v>1528.62</v>
       </c>
       <c r="M25" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="N25" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P25">
         <v>1157673.06</v>
@@ -1932,7 +1938,7 @@
         <v>58</v>
       </c>
       <c r="C26" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D26">
         <v>748</v>
@@ -1941,7 +1947,7 @@
         <v>45930</v>
       </c>
       <c r="F26" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H26" s="2">
         <v>45935</v>
@@ -1950,16 +1956,16 @@
         <v>38718.58</v>
       </c>
       <c r="J26" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="K26">
         <v>38718.58</v>
       </c>
       <c r="M26" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="N26" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P26">
         <v>63746.85</v>
@@ -1982,7 +1988,7 @@
         <v>45968</v>
       </c>
       <c r="F27" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H27" s="2">
         <v>45935</v>
@@ -1991,16 +1997,16 @@
         <v>133124.11</v>
       </c>
       <c r="J27" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="K27">
         <v>133124.11</v>
       </c>
       <c r="M27" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="N27" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P27">
         <v>1000001.64</v>
@@ -2023,7 +2029,7 @@
         <v>46043</v>
       </c>
       <c r="F28" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H28" s="2">
         <v>46075</v>
@@ -2032,16 +2038,16 @@
         <v>11372.9</v>
       </c>
       <c r="J28" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="K28">
         <v>11372.9</v>
       </c>
       <c r="M28" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="N28" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P28">
         <v>1500000</v>
@@ -2055,16 +2061,16 @@
         <v>61</v>
       </c>
       <c r="G29" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="L29">
         <v>15854.78</v>
       </c>
       <c r="M29" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="N29" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -2075,16 +2081,16 @@
         <v>62</v>
       </c>
       <c r="G30" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="L30">
         <v>24962.38</v>
       </c>
       <c r="M30" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="N30" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -2101,7 +2107,7 @@
         <v>46104</v>
       </c>
       <c r="F31" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H31" s="2">
         <v>46106</v>
@@ -2110,19 +2116,60 @@
         <v>27801.11</v>
       </c>
       <c r="J31" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="K31">
         <v>27801.11</v>
       </c>
       <c r="M31" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="N31" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P31">
         <v>1500000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16">
+      <c r="A32">
+        <v>3</v>
+      </c>
+      <c r="B32" t="s">
+        <v>64</v>
+      </c>
+      <c r="D32">
+        <v>1882</v>
+      </c>
+      <c r="E32" s="2">
+        <v>46199</v>
+      </c>
+      <c r="F32" t="s">
+        <v>89</v>
+      </c>
+      <c r="H32" s="2">
+        <v>46233</v>
+      </c>
+      <c r="I32">
+        <v>58868.35</v>
+      </c>
+      <c r="J32" t="s">
+        <v>107</v>
+      </c>
+      <c r="K32">
+        <v>58868.35</v>
+      </c>
+      <c r="M32" t="s">
+        <v>119</v>
+      </c>
+      <c r="N32" t="s">
+        <v>121</v>
+      </c>
+      <c r="O32">
+        <v>497601.53</v>
+      </c>
+      <c r="P32">
+        <v>1867169.54</v>
       </c>
     </row>
   </sheetData>
@@ -2137,24 +2184,24 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B2">
         <v>52250.04</v>
@@ -2165,7 +2212,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B3">
         <v>881914.1800000001</v>
@@ -2176,7 +2223,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B4">
         <v>750000</v>
@@ -2187,7 +2234,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B5">
         <v>949835.78</v>
@@ -2198,7 +2245,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B6">
         <v>524584.95</v>
@@ -2209,7 +2256,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B7">
         <v>211614.23</v>
@@ -2220,7 +2267,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B8">
         <v>2391157.41</v>
@@ -2231,7 +2278,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B9">
         <v>618154.38</v>
@@ -2242,7 +2289,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B10">
         <v>1600334.09</v>
@@ -2253,7 +2300,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>130</v>
+        <v>89</v>
       </c>
       <c r="B11">
         <v>1867169.54</v>
@@ -2264,7 +2311,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B12">
         <v>968237.39</v>
@@ -2275,7 +2322,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B13">
         <v>1011677.95</v>
@@ -2286,7 +2333,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B14">
         <v>1580293.02</v>
@@ -2297,7 +2344,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -2308,7 +2355,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B16">
         <v>63746.85</v>
@@ -2319,7 +2366,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B17">
         <v>947931.1</v>
@@ -2330,7 +2377,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B18">
         <v>259790.57</v>
@@ -2341,7 +2388,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B19">
         <v>170479.3</v>
@@ -2352,7 +2399,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B20">
         <v>1500000</v>
@@ -2363,7 +2410,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B21">
         <v>1000001.64</v>
@@ -2374,7 +2421,7 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B22">
         <v>68405.66</v>
@@ -2385,7 +2432,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B23">
         <v>1157673.06</v>
@@ -2396,7 +2443,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B24">
         <v>34065.36</v>
@@ -2407,7 +2454,7 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -2418,7 +2465,7 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -2429,7 +2476,7 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -2440,7 +2487,7 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B28">
         <v>0</v>
@@ -2451,7 +2498,7 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -2462,7 +2509,7 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B30">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (20/07/2026 16:19)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -470,16 +470,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -495,7 +487,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -503,30 +495,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -826,37 +800,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -906,58 +880,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -974,13 +948,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>68</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1015,13 +989,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>69</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1056,13 +1030,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>70</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1097,13 +1071,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>71</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1138,13 +1112,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>72</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1182,13 +1156,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>73</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1223,13 +1197,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>74</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1264,13 +1238,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>75</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1302,13 +1276,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>76</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1343,13 +1317,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>77</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1384,13 +1358,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>78</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1425,13 +1399,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>79</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1463,13 +1437,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>80</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1504,13 +1478,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>81</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1545,13 +1519,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>82</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1586,13 +1560,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>82</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1627,13 +1601,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>82</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1688,13 +1662,13 @@
       <c r="D20">
         <v>402</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>45791</v>
       </c>
       <c r="F20" t="s">
         <v>83</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>45834</v>
       </c>
       <c r="I20">
@@ -1729,13 +1703,13 @@
       <c r="D21">
         <v>447</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45814</v>
       </c>
       <c r="F21" t="s">
         <v>84</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45955</v>
       </c>
       <c r="I21">
@@ -1773,13 +1747,13 @@
       <c r="D22">
         <v>529</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45853</v>
       </c>
       <c r="F22" t="s">
         <v>85</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45939</v>
       </c>
       <c r="I22">
@@ -1817,13 +1791,13 @@
       <c r="D23">
         <v>691</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45910</v>
       </c>
       <c r="F23" t="s">
         <v>85</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45941</v>
       </c>
       <c r="I23">
@@ -1861,13 +1835,13 @@
       <c r="D24">
         <v>677</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45904</v>
       </c>
       <c r="F24" t="s">
         <v>71</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45935</v>
       </c>
       <c r="I24">
@@ -1902,13 +1876,13 @@
       <c r="D25">
         <v>278</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>46008</v>
       </c>
       <c r="F25" t="s">
         <v>86</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46066</v>
       </c>
       <c r="I25">
@@ -1943,13 +1917,13 @@
       <c r="D26">
         <v>748</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45930</v>
       </c>
       <c r="F26" t="s">
         <v>87</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -1984,13 +1958,13 @@
       <c r="D27">
         <v>822</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45968</v>
       </c>
       <c r="F27" t="s">
         <v>88</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2025,13 +1999,13 @@
       <c r="D28">
         <v>360</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>46043</v>
       </c>
       <c r="F28" t="s">
         <v>79</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46075</v>
       </c>
       <c r="I28">
@@ -2103,13 +2077,13 @@
       <c r="D31">
         <v>1465</v>
       </c>
-      <c r="E31" s="2">
+      <c r="E31" s="1">
         <v>46104</v>
       </c>
       <c r="F31" t="s">
         <v>79</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46106</v>
       </c>
       <c r="I31">
@@ -2141,13 +2115,13 @@
       <c r="D32">
         <v>1882</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>46199</v>
       </c>
       <c r="F32" t="s">
         <v>89</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46233</v>
       </c>
       <c r="I32">
@@ -2183,19 +2157,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>123</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>124</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>125</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>126</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (22/07/2026 12:02)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -470,8 +470,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -487,7 +495,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -495,12 +503,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -800,37 +826,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -880,58 +906,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -948,13 +974,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>68</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -989,13 +1015,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>69</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1030,13 +1056,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>70</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1071,13 +1097,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>71</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1112,13 +1138,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>72</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1156,13 +1182,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>73</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1197,13 +1223,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>74</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1238,13 +1264,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>75</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1276,13 +1302,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>76</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1317,13 +1343,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>77</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1358,13 +1384,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>78</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1399,13 +1425,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>79</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1437,13 +1463,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>80</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1478,13 +1504,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>81</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1519,13 +1545,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>82</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1560,13 +1586,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>82</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1601,13 +1627,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>82</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1662,13 +1688,13 @@
       <c r="D20">
         <v>402</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>45791</v>
       </c>
       <c r="F20" t="s">
         <v>83</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>45834</v>
       </c>
       <c r="I20">
@@ -1703,13 +1729,13 @@
       <c r="D21">
         <v>447</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45814</v>
       </c>
       <c r="F21" t="s">
         <v>84</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45955</v>
       </c>
       <c r="I21">
@@ -1747,13 +1773,13 @@
       <c r="D22">
         <v>529</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45853</v>
       </c>
       <c r="F22" t="s">
         <v>85</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45939</v>
       </c>
       <c r="I22">
@@ -1791,13 +1817,13 @@
       <c r="D23">
         <v>691</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45910</v>
       </c>
       <c r="F23" t="s">
         <v>85</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45941</v>
       </c>
       <c r="I23">
@@ -1835,13 +1861,13 @@
       <c r="D24">
         <v>677</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45904</v>
       </c>
       <c r="F24" t="s">
         <v>71</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45935</v>
       </c>
       <c r="I24">
@@ -1876,13 +1902,13 @@
       <c r="D25">
         <v>278</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>46008</v>
       </c>
       <c r="F25" t="s">
         <v>86</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46066</v>
       </c>
       <c r="I25">
@@ -1917,13 +1943,13 @@
       <c r="D26">
         <v>748</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45930</v>
       </c>
       <c r="F26" t="s">
         <v>87</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -1958,13 +1984,13 @@
       <c r="D27">
         <v>822</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45968</v>
       </c>
       <c r="F27" t="s">
         <v>88</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -1999,13 +2025,13 @@
       <c r="D28">
         <v>360</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>46043</v>
       </c>
       <c r="F28" t="s">
         <v>79</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46075</v>
       </c>
       <c r="I28">
@@ -2077,13 +2103,13 @@
       <c r="D31">
         <v>1465</v>
       </c>
-      <c r="E31" s="1">
+      <c r="E31" s="2">
         <v>46104</v>
       </c>
       <c r="F31" t="s">
         <v>79</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46106</v>
       </c>
       <c r="I31">
@@ -2115,13 +2141,13 @@
       <c r="D32">
         <v>1882</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E32" s="2">
         <v>46199</v>
       </c>
       <c r="F32" t="s">
         <v>89</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46233</v>
       </c>
       <c r="I32">
@@ -2157,19 +2183,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>126</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (22/07/2026 16:09)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -470,16 +470,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -495,7 +487,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -503,30 +495,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -826,37 +800,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -906,58 +880,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -974,13 +948,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>68</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1015,13 +989,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>69</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1056,13 +1030,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>70</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1097,13 +1071,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>71</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1138,13 +1112,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>72</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1182,13 +1156,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>73</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1223,13 +1197,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>74</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1264,13 +1238,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>75</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1302,13 +1276,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>76</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1343,13 +1317,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>77</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1384,13 +1358,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>78</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1425,13 +1399,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>79</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1463,13 +1437,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>80</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1504,13 +1478,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>81</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1545,13 +1519,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>82</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1586,13 +1560,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>82</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1627,13 +1601,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>82</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1688,13 +1662,13 @@
       <c r="D20">
         <v>402</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>45791</v>
       </c>
       <c r="F20" t="s">
         <v>83</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>45834</v>
       </c>
       <c r="I20">
@@ -1729,13 +1703,13 @@
       <c r="D21">
         <v>447</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45814</v>
       </c>
       <c r="F21" t="s">
         <v>84</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45955</v>
       </c>
       <c r="I21">
@@ -1773,13 +1747,13 @@
       <c r="D22">
         <v>529</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45853</v>
       </c>
       <c r="F22" t="s">
         <v>85</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45939</v>
       </c>
       <c r="I22">
@@ -1817,13 +1791,13 @@
       <c r="D23">
         <v>691</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45910</v>
       </c>
       <c r="F23" t="s">
         <v>85</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45941</v>
       </c>
       <c r="I23">
@@ -1861,13 +1835,13 @@
       <c r="D24">
         <v>677</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45904</v>
       </c>
       <c r="F24" t="s">
         <v>71</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45935</v>
       </c>
       <c r="I24">
@@ -1902,13 +1876,13 @@
       <c r="D25">
         <v>278</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>46008</v>
       </c>
       <c r="F25" t="s">
         <v>86</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46066</v>
       </c>
       <c r="I25">
@@ -1943,13 +1917,13 @@
       <c r="D26">
         <v>748</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45930</v>
       </c>
       <c r="F26" t="s">
         <v>87</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -1984,13 +1958,13 @@
       <c r="D27">
         <v>822</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45968</v>
       </c>
       <c r="F27" t="s">
         <v>88</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2025,13 +1999,13 @@
       <c r="D28">
         <v>360</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>46043</v>
       </c>
       <c r="F28" t="s">
         <v>79</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46075</v>
       </c>
       <c r="I28">
@@ -2103,13 +2077,13 @@
       <c r="D31">
         <v>1465</v>
       </c>
-      <c r="E31" s="2">
+      <c r="E31" s="1">
         <v>46104</v>
       </c>
       <c r="F31" t="s">
         <v>79</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46106</v>
       </c>
       <c r="I31">
@@ -2141,13 +2115,13 @@
       <c r="D32">
         <v>1882</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>46199</v>
       </c>
       <c r="F32" t="s">
         <v>89</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46233</v>
       </c>
       <c r="I32">
@@ -2183,19 +2157,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>123</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>124</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>125</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>126</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (23/07/2026 11:41)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -470,8 +470,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -487,7 +495,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -495,12 +503,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -800,37 +826,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -880,58 +906,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -948,13 +974,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>68</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -989,13 +1015,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>69</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1030,13 +1056,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>70</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1071,13 +1097,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>71</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1112,13 +1138,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>72</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1156,13 +1182,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>73</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1197,13 +1223,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>74</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1238,13 +1264,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>75</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1276,13 +1302,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>76</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1317,13 +1343,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>77</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1358,13 +1384,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>78</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1399,13 +1425,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>79</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1437,13 +1463,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>80</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1478,13 +1504,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>81</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1519,13 +1545,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>82</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1560,13 +1586,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>82</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1601,13 +1627,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>82</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1662,13 +1688,13 @@
       <c r="D20">
         <v>402</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>45791</v>
       </c>
       <c r="F20" t="s">
         <v>83</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>45834</v>
       </c>
       <c r="I20">
@@ -1703,13 +1729,13 @@
       <c r="D21">
         <v>447</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45814</v>
       </c>
       <c r="F21" t="s">
         <v>84</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45955</v>
       </c>
       <c r="I21">
@@ -1747,13 +1773,13 @@
       <c r="D22">
         <v>529</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45853</v>
       </c>
       <c r="F22" t="s">
         <v>85</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45939</v>
       </c>
       <c r="I22">
@@ -1791,13 +1817,13 @@
       <c r="D23">
         <v>691</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45910</v>
       </c>
       <c r="F23" t="s">
         <v>85</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45941</v>
       </c>
       <c r="I23">
@@ -1835,13 +1861,13 @@
       <c r="D24">
         <v>677</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45904</v>
       </c>
       <c r="F24" t="s">
         <v>71</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45935</v>
       </c>
       <c r="I24">
@@ -1876,13 +1902,13 @@
       <c r="D25">
         <v>278</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>46008</v>
       </c>
       <c r="F25" t="s">
         <v>86</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46066</v>
       </c>
       <c r="I25">
@@ -1917,13 +1943,13 @@
       <c r="D26">
         <v>748</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45930</v>
       </c>
       <c r="F26" t="s">
         <v>87</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -1958,13 +1984,13 @@
       <c r="D27">
         <v>822</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45968</v>
       </c>
       <c r="F27" t="s">
         <v>88</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -1999,13 +2025,13 @@
       <c r="D28">
         <v>360</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>46043</v>
       </c>
       <c r="F28" t="s">
         <v>79</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46075</v>
       </c>
       <c r="I28">
@@ -2077,13 +2103,13 @@
       <c r="D31">
         <v>1465</v>
       </c>
-      <c r="E31" s="1">
+      <c r="E31" s="2">
         <v>46104</v>
       </c>
       <c r="F31" t="s">
         <v>79</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46106</v>
       </c>
       <c r="I31">
@@ -2115,13 +2141,13 @@
       <c r="D32">
         <v>1882</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E32" s="2">
         <v>46199</v>
       </c>
       <c r="F32" t="s">
         <v>89</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46233</v>
       </c>
       <c r="I32">
@@ -2157,19 +2183,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>126</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (23/07/2026 16:17)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -470,16 +470,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -495,7 +487,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -503,30 +495,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -826,37 +800,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -906,58 +880,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -974,13 +948,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>68</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1015,13 +989,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>69</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1056,13 +1030,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>70</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1097,13 +1071,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>71</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1138,13 +1112,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>72</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1182,13 +1156,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>73</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1223,13 +1197,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>74</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1264,13 +1238,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>75</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1302,13 +1276,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>76</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1343,13 +1317,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>77</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1384,13 +1358,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>78</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1425,13 +1399,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>79</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1463,13 +1437,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>80</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1504,13 +1478,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>81</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1545,13 +1519,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>82</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1586,13 +1560,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>82</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1627,13 +1601,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>82</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1688,13 +1662,13 @@
       <c r="D20">
         <v>402</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>45791</v>
       </c>
       <c r="F20" t="s">
         <v>83</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>45834</v>
       </c>
       <c r="I20">
@@ -1729,13 +1703,13 @@
       <c r="D21">
         <v>447</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45814</v>
       </c>
       <c r="F21" t="s">
         <v>84</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45955</v>
       </c>
       <c r="I21">
@@ -1773,13 +1747,13 @@
       <c r="D22">
         <v>529</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45853</v>
       </c>
       <c r="F22" t="s">
         <v>85</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45939</v>
       </c>
       <c r="I22">
@@ -1817,13 +1791,13 @@
       <c r="D23">
         <v>691</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45910</v>
       </c>
       <c r="F23" t="s">
         <v>85</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45941</v>
       </c>
       <c r="I23">
@@ -1861,13 +1835,13 @@
       <c r="D24">
         <v>677</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45904</v>
       </c>
       <c r="F24" t="s">
         <v>71</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45935</v>
       </c>
       <c r="I24">
@@ -1902,13 +1876,13 @@
       <c r="D25">
         <v>278</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>46008</v>
       </c>
       <c r="F25" t="s">
         <v>86</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46066</v>
       </c>
       <c r="I25">
@@ -1943,13 +1917,13 @@
       <c r="D26">
         <v>748</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45930</v>
       </c>
       <c r="F26" t="s">
         <v>87</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -1984,13 +1958,13 @@
       <c r="D27">
         <v>822</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45968</v>
       </c>
       <c r="F27" t="s">
         <v>88</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2025,13 +1999,13 @@
       <c r="D28">
         <v>360</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>46043</v>
       </c>
       <c r="F28" t="s">
         <v>79</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46075</v>
       </c>
       <c r="I28">
@@ -2103,13 +2077,13 @@
       <c r="D31">
         <v>1465</v>
       </c>
-      <c r="E31" s="2">
+      <c r="E31" s="1">
         <v>46104</v>
       </c>
       <c r="F31" t="s">
         <v>79</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46106</v>
       </c>
       <c r="I31">
@@ -2141,13 +2115,13 @@
       <c r="D32">
         <v>1882</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>46199</v>
       </c>
       <c r="F32" t="s">
         <v>89</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46233</v>
       </c>
       <c r="I32">
@@ -2183,19 +2157,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>123</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>124</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>125</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>126</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Histórico diário dos Empenhos (Contrato 005) + consumo de Hora de Voo pela hora real
Wallace: "quando for atendido e depois for para o saldo la nos
empenhos pode ter um dalay, entao cria o historico para o dinheiro
nunca sumir" — extrair_pagamentos.py grava snapshot diário da aba
EMPENHOS (historico_empenhos.csv), exibido como "Evolução" na aba
Empenhos (Contrato 005) do MTA.

"media de gasto nao é do cronograma é o real, quantas horas falta no
ano? divide por quantos meses nao paguei e multiplica pela hora de voo
(valor)" — substitui a média baseada no valor R$ da fila por: horas de
Hora de Voo ainda não atendidas (extraídas do texto da tarefa, ex.
"1000 HV") ÷ meses não pagos (a partir do mês seguinte ao último
realmente empenhado, não do mês corrente) × valor real da hora de voo
(Reajuste, pós 2° Reajuste).

Também sincroniza com a atualização que o Wallace fez na planilha
005_CELOG-PAMALS_2025 (novo empenho, 30 NEs agora).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="148">
   <si>
     <t>numero_contrato</t>
   </si>
@@ -461,6 +461,9 @@
   </si>
   <si>
     <t>2026NE000842</t>
+  </si>
+  <si>
+    <t>2026NE000944</t>
   </si>
 </sst>
 </file>
@@ -470,8 +473,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -487,7 +498,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -495,12 +506,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -800,37 +829,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -880,58 +909,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -948,13 +977,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>68</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -989,13 +1018,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>69</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1030,13 +1059,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>70</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1071,13 +1100,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>71</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1112,13 +1141,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>72</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1156,13 +1185,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>73</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1197,13 +1226,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>74</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1238,13 +1267,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>75</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1276,13 +1305,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>76</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1317,13 +1346,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>77</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1358,13 +1387,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>78</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1382,11 +1411,8 @@
       <c r="N12" t="s">
         <v>120</v>
       </c>
-      <c r="O12">
-        <v>497601.53</v>
-      </c>
       <c r="P12">
-        <v>3024842.6</v>
+        <v>3522444.13</v>
       </c>
     </row>
     <row r="13" spans="1:18">
@@ -1399,13 +1425,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>79</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1437,13 +1463,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>80</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1478,13 +1504,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>81</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1519,13 +1545,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>82</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1544,10 +1570,10 @@
         <v>120</v>
       </c>
       <c r="O16">
-        <v>497601.54</v>
+        <v>0.01</v>
       </c>
       <c r="P16">
-        <v>5838619.970000001</v>
+        <v>6336221.5</v>
       </c>
     </row>
     <row r="17" spans="1:16">
@@ -1560,13 +1586,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>82</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1585,10 +1611,10 @@
         <v>120</v>
       </c>
       <c r="O17">
-        <v>497601.54</v>
+        <v>0.01</v>
       </c>
       <c r="P17">
-        <v>5838619.970000001</v>
+        <v>6336221.5</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -1601,13 +1627,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>82</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1626,10 +1652,10 @@
         <v>120</v>
       </c>
       <c r="O18">
-        <v>497601.54</v>
+        <v>0.01</v>
       </c>
       <c r="P18">
-        <v>5838619.970000001</v>
+        <v>6336221.5</v>
       </c>
     </row>
     <row r="19" spans="1:16">
@@ -1662,13 +1688,13 @@
       <c r="D20">
         <v>402</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>45791</v>
       </c>
       <c r="F20" t="s">
         <v>83</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>45834</v>
       </c>
       <c r="I20">
@@ -1703,13 +1729,13 @@
       <c r="D21">
         <v>447</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45814</v>
       </c>
       <c r="F21" t="s">
         <v>84</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45955</v>
       </c>
       <c r="I21">
@@ -1747,13 +1773,13 @@
       <c r="D22">
         <v>529</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45853</v>
       </c>
       <c r="F22" t="s">
         <v>85</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45939</v>
       </c>
       <c r="I22">
@@ -1791,13 +1817,13 @@
       <c r="D23">
         <v>691</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45910</v>
       </c>
       <c r="F23" t="s">
         <v>85</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45941</v>
       </c>
       <c r="I23">
@@ -1835,13 +1861,13 @@
       <c r="D24">
         <v>677</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45904</v>
       </c>
       <c r="F24" t="s">
         <v>71</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45935</v>
       </c>
       <c r="I24">
@@ -1876,13 +1902,13 @@
       <c r="D25">
         <v>278</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>46008</v>
       </c>
       <c r="F25" t="s">
         <v>86</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46066</v>
       </c>
       <c r="I25">
@@ -1917,13 +1943,13 @@
       <c r="D26">
         <v>748</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45930</v>
       </c>
       <c r="F26" t="s">
         <v>87</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -1958,13 +1984,13 @@
       <c r="D27">
         <v>822</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45968</v>
       </c>
       <c r="F27" t="s">
         <v>88</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -1999,13 +2025,13 @@
       <c r="D28">
         <v>360</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>46043</v>
       </c>
       <c r="F28" t="s">
         <v>79</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46075</v>
       </c>
       <c r="I28">
@@ -2077,13 +2103,13 @@
       <c r="D31">
         <v>1465</v>
       </c>
-      <c r="E31" s="1">
+      <c r="E31" s="2">
         <v>46104</v>
       </c>
       <c r="F31" t="s">
         <v>79</v>
       </c>
-      <c r="H31" s="1">
+      <c r="H31" s="2">
         <v>46106</v>
       </c>
       <c r="I31">
@@ -2115,13 +2141,13 @@
       <c r="D32">
         <v>1882</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E32" s="2">
         <v>46199</v>
       </c>
       <c r="F32" t="s">
         <v>89</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46233</v>
       </c>
       <c r="I32">
@@ -2139,11 +2165,8 @@
       <c r="N32" t="s">
         <v>121</v>
       </c>
-      <c r="O32">
-        <v>497601.53</v>
-      </c>
       <c r="P32">
-        <v>1867169.54</v>
+        <v>2364771.07</v>
       </c>
     </row>
   </sheetData>
@@ -2153,23 +2176,23 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>126</v>
       </c>
     </row>
@@ -2277,10 +2300,10 @@
         <v>89</v>
       </c>
       <c r="B11">
-        <v>1867169.54</v>
+        <v>2364771.07</v>
       </c>
       <c r="C11">
-        <v>497601.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -2431,10 +2454,10 @@
         <v>141</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>843261.89</v>
       </c>
       <c r="C25">
-        <v>1770880.5</v>
+        <v>927618.61</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -2490,6 +2513,17 @@
       </c>
       <c r="C30">
         <v>1530656.62</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
+        <v>147</v>
+      </c>
+      <c r="B31">
+        <v>0</v>
+      </c>
+      <c r="C31">
+        <v>173846.38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (29/07/2026 13:12)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -473,16 +473,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -498,7 +490,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -506,30 +498,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -829,37 +803,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -909,58 +883,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -977,13 +951,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>68</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1018,13 +992,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>69</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1059,13 +1033,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>70</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1100,13 +1074,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>71</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1141,13 +1115,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>72</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1185,13 +1159,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>73</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1226,13 +1200,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>74</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1267,13 +1241,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>75</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1305,13 +1279,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>76</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1346,13 +1320,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>77</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1387,13 +1361,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>78</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1425,13 +1399,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>79</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1463,13 +1437,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>80</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1504,13 +1478,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>81</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1545,13 +1519,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>82</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1586,13 +1560,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>82</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1627,13 +1601,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>82</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1688,13 +1662,13 @@
       <c r="D20">
         <v>402</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>45791</v>
       </c>
       <c r="F20" t="s">
         <v>83</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>45834</v>
       </c>
       <c r="I20">
@@ -1729,13 +1703,13 @@
       <c r="D21">
         <v>447</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45814</v>
       </c>
       <c r="F21" t="s">
         <v>84</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45955</v>
       </c>
       <c r="I21">
@@ -1773,13 +1747,13 @@
       <c r="D22">
         <v>529</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45853</v>
       </c>
       <c r="F22" t="s">
         <v>85</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45939</v>
       </c>
       <c r="I22">
@@ -1817,13 +1791,13 @@
       <c r="D23">
         <v>691</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45910</v>
       </c>
       <c r="F23" t="s">
         <v>85</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45941</v>
       </c>
       <c r="I23">
@@ -1861,13 +1835,13 @@
       <c r="D24">
         <v>677</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45904</v>
       </c>
       <c r="F24" t="s">
         <v>71</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45935</v>
       </c>
       <c r="I24">
@@ -1902,13 +1876,13 @@
       <c r="D25">
         <v>278</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>46008</v>
       </c>
       <c r="F25" t="s">
         <v>86</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46066</v>
       </c>
       <c r="I25">
@@ -1943,13 +1917,13 @@
       <c r="D26">
         <v>748</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45930</v>
       </c>
       <c r="F26" t="s">
         <v>87</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -1984,13 +1958,13 @@
       <c r="D27">
         <v>822</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45968</v>
       </c>
       <c r="F27" t="s">
         <v>88</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2025,13 +1999,13 @@
       <c r="D28">
         <v>360</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>46043</v>
       </c>
       <c r="F28" t="s">
         <v>79</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46075</v>
       </c>
       <c r="I28">
@@ -2103,13 +2077,13 @@
       <c r="D31">
         <v>1465</v>
       </c>
-      <c r="E31" s="2">
+      <c r="E31" s="1">
         <v>46104</v>
       </c>
       <c r="F31" t="s">
         <v>79</v>
       </c>
-      <c r="H31" s="2">
+      <c r="H31" s="1">
         <v>46106</v>
       </c>
       <c r="I31">
@@ -2141,13 +2115,13 @@
       <c r="D32">
         <v>1882</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>46199</v>
       </c>
       <c r="F32" t="s">
         <v>89</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46233</v>
       </c>
       <c r="I32">
@@ -2180,19 +2154,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>123</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>124</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>125</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>126</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização manual: pagamentos (06/08/2026)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="151">
   <si>
     <t>numero_contrato</t>
   </si>
@@ -205,6 +205,9 @@
   </si>
   <si>
     <t>Módulo II – Orçamento 03/26</t>
+  </si>
+  <si>
+    <t>Módulo II – Orçamento 04/26</t>
   </si>
   <si>
     <t>Módulo III – Orçamento 17 Manuais</t>
@@ -479,8 +482,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -496,7 +507,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -504,12 +515,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -809,37 +838,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -885,62 +914,62 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R32"/>
+  <dimension ref="A1:R33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -952,34 +981,34 @@
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
-        <v>68</v>
-      </c>
-      <c r="H2" s="1">
+        <v>69</v>
+      </c>
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
         <v>748504.24</v>
       </c>
       <c r="J2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K2">
         <v>748504.24</v>
       </c>
       <c r="M2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P2">
         <v>881914.1800000001</v>
@@ -993,34 +1022,34 @@
         <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
-        <v>69</v>
-      </c>
-      <c r="H3" s="1">
+        <v>70</v>
+      </c>
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
         <v>1110378.24</v>
       </c>
       <c r="J3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="K3">
         <v>1110378.24</v>
       </c>
       <c r="M3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P3">
         <v>2634000</v>
@@ -1034,34 +1063,34 @@
         <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
-        <v>70</v>
-      </c>
-      <c r="H4" s="1">
+        <v>71</v>
+      </c>
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
         <v>974557.12</v>
       </c>
       <c r="J4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="K4">
         <v>974557.12</v>
       </c>
       <c r="M4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P4">
         <v>1686034.96</v>
@@ -1075,34 +1104,34 @@
         <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
-        <v>71</v>
-      </c>
-      <c r="H5" s="1">
+        <v>72</v>
+      </c>
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
         <v>1402001.34</v>
       </c>
       <c r="J5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K5">
         <v>1402001.34</v>
       </c>
       <c r="M5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P5">
         <v>1600334.09</v>
@@ -1116,34 +1145,34 @@
         <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
-        <v>72</v>
-      </c>
-      <c r="H6" s="1">
+        <v>73</v>
+      </c>
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
         <v>1223702.3</v>
       </c>
       <c r="J6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K6">
         <v>1223702.3</v>
       </c>
       <c r="M6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="O6">
         <v>0.02</v>
@@ -1160,34 +1189,34 @@
         <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
-        <v>73</v>
-      </c>
-      <c r="H7" s="1">
+        <v>74</v>
+      </c>
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
         <v>1011677.95</v>
       </c>
       <c r="J7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K7">
         <v>1011677.95</v>
       </c>
       <c r="M7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P7">
         <v>2568571.48</v>
@@ -1201,34 +1230,34 @@
         <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
-        <v>74</v>
-      </c>
-      <c r="H8" s="1">
+        <v>75</v>
+      </c>
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
         <v>896744.0600000001</v>
       </c>
       <c r="J8" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K8">
         <v>896744.0600000001</v>
       </c>
       <c r="M8" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P8">
         <v>968237.39</v>
@@ -1242,34 +1271,34 @@
         <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
-        <v>75</v>
-      </c>
-      <c r="H9" s="1">
+        <v>76</v>
+      </c>
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
         <v>919329.0600000001</v>
       </c>
       <c r="J9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K9">
         <v>919329.0600000001</v>
       </c>
       <c r="M9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P9">
         <v>1947932.74</v>
@@ -1285,29 +1314,29 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
-        <v>76</v>
-      </c>
-      <c r="H10" s="1">
+        <v>77</v>
+      </c>
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
         <v>1157009.26</v>
       </c>
       <c r="J10" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K10">
         <v>1157009.26</v>
       </c>
       <c r="M10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P10">
         <v>3105605.8</v>
@@ -1321,34 +1350,34 @@
         <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
-        <v>77</v>
-      </c>
-      <c r="H11" s="1">
+        <v>78</v>
+      </c>
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
         <v>1214597.952</v>
       </c>
       <c r="J11" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K11">
         <v>1214597.952</v>
       </c>
       <c r="M11" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P11">
         <v>2096487.74</v>
@@ -1362,34 +1391,34 @@
         <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
-        <v>78</v>
-      </c>
-      <c r="H12" s="1">
+        <v>79</v>
+      </c>
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
         <v>967082.09</v>
       </c>
       <c r="J12" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K12">
         <v>967082.09</v>
       </c>
       <c r="M12" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N12" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P12">
         <v>3522444.13</v>
@@ -1405,29 +1434,29 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
-        <v>79</v>
-      </c>
-      <c r="H13" s="1">
+        <v>80</v>
+      </c>
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
         <v>719561.08</v>
       </c>
       <c r="J13" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K13">
         <v>719561.08</v>
       </c>
       <c r="M13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N13" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P13">
         <v>1500000</v>
@@ -1443,29 +1472,29 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
-        <v>80</v>
-      </c>
-      <c r="H14" s="1">
+        <v>81</v>
+      </c>
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
         <v>885881.08</v>
       </c>
       <c r="J14" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K14">
         <v>885881.08</v>
       </c>
       <c r="M14" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N14" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="O14">
         <v>34065.36</v>
@@ -1484,29 +1513,29 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
-        <v>81</v>
-      </c>
-      <c r="H15" s="1">
+        <v>82</v>
+      </c>
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
         <v>1350542.52</v>
       </c>
       <c r="J15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K15">
         <v>1350542.52</v>
       </c>
       <c r="M15" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N15" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="O15">
         <v>0.01</v>
@@ -1525,29 +1554,29 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
-        <v>82</v>
-      </c>
-      <c r="H16" s="1">
+        <v>83</v>
+      </c>
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
         <v>1108954.435833333</v>
       </c>
       <c r="J16" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K16">
         <v>1108954.435833333</v>
       </c>
       <c r="M16" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N16" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="O16">
         <v>0.01</v>
@@ -1566,29 +1595,29 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
-        <v>82</v>
-      </c>
-      <c r="H17" s="1">
+        <v>83</v>
+      </c>
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
         <v>218206.1</v>
       </c>
       <c r="J17" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K17">
         <v>218206.1</v>
       </c>
       <c r="M17" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N17" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="O17">
         <v>0.01</v>
@@ -1607,29 +1636,29 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
-        <v>82</v>
-      </c>
-      <c r="H18" s="1">
+        <v>83</v>
+      </c>
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
         <v>1549250.84</v>
       </c>
       <c r="J18" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K18">
         <v>1549250.84</v>
       </c>
       <c r="M18" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N18" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="O18">
         <v>0.01</v>
@@ -1648,29 +1677,29 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
-        <v>83</v>
-      </c>
-      <c r="H19" s="1">
+        <v>84</v>
+      </c>
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
         <v>1340865.98</v>
       </c>
       <c r="J19" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K19">
         <v>1340865.98</v>
       </c>
       <c r="M19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N19" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="O19">
         <v>927618.61</v>
@@ -1689,29 +1718,29 @@
       <c r="D20">
         <v>402</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>45791</v>
       </c>
       <c r="F20" t="s">
-        <v>84</v>
-      </c>
-      <c r="H20" s="1">
+        <v>85</v>
+      </c>
+      <c r="H20" s="2">
         <v>45834</v>
       </c>
       <c r="I20">
         <v>188246.17</v>
       </c>
       <c r="J20" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="K20">
         <v>188246.17</v>
       </c>
       <c r="M20" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P20">
         <v>211614.23</v>
@@ -1730,29 +1759,29 @@
       <c r="D21">
         <v>447</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45814</v>
       </c>
       <c r="F21" t="s">
-        <v>85</v>
-      </c>
-      <c r="H21" s="1">
+        <v>86</v>
+      </c>
+      <c r="H21" s="2">
         <v>45955</v>
       </c>
       <c r="I21">
         <v>112720.77</v>
       </c>
       <c r="J21" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K21">
         <v>112720.77</v>
       </c>
       <c r="M21" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N21" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="O21">
         <v>0.01</v>
@@ -1769,34 +1798,34 @@
         <v>54</v>
       </c>
       <c r="C22" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D22">
         <v>529</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45853</v>
       </c>
       <c r="F22" t="s">
-        <v>86</v>
-      </c>
-      <c r="H22" s="1">
+        <v>87</v>
+      </c>
+      <c r="H22" s="2">
         <v>45939</v>
       </c>
       <c r="I22">
         <v>378307.61</v>
       </c>
       <c r="J22" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="K22">
         <v>378307.61</v>
       </c>
       <c r="M22" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N22" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="O22">
         <v>0.01</v>
@@ -1813,34 +1842,34 @@
         <v>55</v>
       </c>
       <c r="C23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D23">
         <v>691</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45910</v>
       </c>
       <c r="F23" t="s">
-        <v>86</v>
-      </c>
-      <c r="H23" s="1">
+        <v>87</v>
+      </c>
+      <c r="H23" s="2">
         <v>45941</v>
       </c>
       <c r="I23">
         <v>3315.047100000025</v>
       </c>
       <c r="J23" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K23">
         <v>3315.04710000003</v>
       </c>
       <c r="M23" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N23" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="O23">
         <v>0.01</v>
@@ -1862,29 +1891,29 @@
       <c r="D24">
         <v>677</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45904</v>
       </c>
       <c r="F24" t="s">
-        <v>71</v>
-      </c>
-      <c r="H24" s="1">
+        <v>72</v>
+      </c>
+      <c r="H24" s="2">
         <v>45935</v>
       </c>
       <c r="I24">
         <v>198332.75</v>
       </c>
       <c r="J24" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K24">
         <v>198332.75</v>
       </c>
       <c r="M24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N24" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P24">
         <v>1600334.09</v>
@@ -1903,29 +1932,29 @@
       <c r="D25">
         <v>278</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>46008</v>
       </c>
       <c r="F25" t="s">
-        <v>87</v>
-      </c>
-      <c r="H25" s="1">
+        <v>88</v>
+      </c>
+      <c r="H25" s="2">
         <v>46066</v>
       </c>
       <c r="I25">
         <v>1528.62</v>
       </c>
       <c r="J25" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K25">
         <v>1528.62</v>
       </c>
       <c r="M25" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P25">
         <v>1157673.06</v>
@@ -1939,34 +1968,34 @@
         <v>58</v>
       </c>
       <c r="C26" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D26">
         <v>748</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45930</v>
       </c>
       <c r="F26" t="s">
-        <v>88</v>
-      </c>
-      <c r="H26" s="1">
+        <v>89</v>
+      </c>
+      <c r="H26" s="2">
         <v>45935</v>
       </c>
       <c r="I26">
         <v>38718.58</v>
       </c>
       <c r="J26" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K26">
         <v>38718.58</v>
       </c>
       <c r="M26" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P26">
         <v>63746.85</v>
@@ -1985,29 +2014,29 @@
       <c r="D27">
         <v>822</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45968</v>
       </c>
       <c r="F27" t="s">
-        <v>89</v>
-      </c>
-      <c r="H27" s="1">
+        <v>90</v>
+      </c>
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
         <v>133124.11</v>
       </c>
       <c r="J27" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K27">
         <v>133124.11</v>
       </c>
       <c r="M27" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N27" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P27">
         <v>1000001.64</v>
@@ -2026,29 +2055,29 @@
       <c r="D28">
         <v>360</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>46043</v>
       </c>
       <c r="F28" t="s">
-        <v>79</v>
-      </c>
-      <c r="H28" s="1">
+        <v>80</v>
+      </c>
+      <c r="H28" s="2">
         <v>46075</v>
       </c>
       <c r="I28">
         <v>11372.9</v>
       </c>
       <c r="J28" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K28">
         <v>11372.9</v>
       </c>
       <c r="M28" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N28" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P28">
         <v>1500000</v>
@@ -2062,16 +2091,16 @@
         <v>61</v>
       </c>
       <c r="G29" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L29">
         <v>15854.78</v>
       </c>
       <c r="M29" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N29" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -2082,54 +2111,36 @@
         <v>62</v>
       </c>
       <c r="G30" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L30">
-        <v>30940.19</v>
+        <v>42229.72325</v>
       </c>
       <c r="M30" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N30" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="31" spans="1:16">
       <c r="A31">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B31" t="s">
         <v>63</v>
       </c>
-      <c r="D31">
-        <v>1465</v>
-      </c>
-      <c r="E31" s="1">
-        <v>46104</v>
-      </c>
-      <c r="F31" t="s">
-        <v>79</v>
-      </c>
-      <c r="H31" s="1">
-        <v>46106</v>
-      </c>
-      <c r="I31">
-        <v>27801.11</v>
-      </c>
-      <c r="J31" t="s">
-        <v>118</v>
-      </c>
-      <c r="K31">
-        <v>27801.11</v>
+      <c r="G31" t="s">
+        <v>92</v>
+      </c>
+      <c r="L31">
+        <v>48857.39550000001</v>
       </c>
       <c r="M31" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N31" t="s">
-        <v>122</v>
-      </c>
-      <c r="P31">
-        <v>1500000</v>
+        <v>124</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -2140,33 +2151,71 @@
         <v>64</v>
       </c>
       <c r="D32">
-        <v>1882</v>
-      </c>
-      <c r="E32" s="1">
-        <v>46199</v>
+        <v>1465</v>
+      </c>
+      <c r="E32" s="2">
+        <v>46104</v>
       </c>
       <c r="F32" t="s">
-        <v>90</v>
-      </c>
-      <c r="H32" s="1">
-        <v>46233</v>
+        <v>80</v>
+      </c>
+      <c r="H32" s="2">
+        <v>46106</v>
       </c>
       <c r="I32">
-        <v>58868.35</v>
+        <v>27801.11</v>
       </c>
       <c r="J32" t="s">
         <v>119</v>
       </c>
       <c r="K32">
+        <v>27801.11</v>
+      </c>
+      <c r="M32" t="s">
+        <v>122</v>
+      </c>
+      <c r="N32" t="s">
+        <v>123</v>
+      </c>
+      <c r="P32">
+        <v>1500000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16">
+      <c r="A33">
+        <v>3</v>
+      </c>
+      <c r="B33" t="s">
+        <v>65</v>
+      </c>
+      <c r="D33">
+        <v>1882</v>
+      </c>
+      <c r="E33" s="2">
+        <v>46199</v>
+      </c>
+      <c r="F33" t="s">
+        <v>91</v>
+      </c>
+      <c r="H33" s="2">
+        <v>46233</v>
+      </c>
+      <c r="I33">
         <v>58868.35</v>
       </c>
-      <c r="M32" t="s">
-        <v>121</v>
-      </c>
-      <c r="N32" t="s">
-        <v>124</v>
-      </c>
-      <c r="P32">
+      <c r="J33" t="s">
+        <v>120</v>
+      </c>
+      <c r="K33">
+        <v>58868.35</v>
+      </c>
+      <c r="M33" t="s">
+        <v>122</v>
+      </c>
+      <c r="N33" t="s">
+        <v>125</v>
+      </c>
+      <c r="P33">
         <v>2364771.07</v>
       </c>
     </row>
@@ -2181,25 +2230,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
-        <v>125</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="C1" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="E1" t="s">
+      <c r="D1" s="1" t="s">
         <v>128</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B2">
         <v>52250.04</v>
@@ -2210,7 +2259,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B3">
         <v>881914.1800000001</v>
@@ -2221,7 +2270,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B4">
         <v>750000</v>
@@ -2232,7 +2281,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B5">
         <v>949835.78</v>
@@ -2243,7 +2292,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B6">
         <v>524584.95</v>
@@ -2254,7 +2303,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B7">
         <v>211614.23</v>
@@ -2265,7 +2314,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B8">
         <v>2391157.41</v>
@@ -2276,7 +2325,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B9">
         <v>618154.38</v>
@@ -2287,7 +2336,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B10">
         <v>1600334.09</v>
@@ -2298,7 +2347,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B11">
         <v>2364771.07</v>
@@ -2309,7 +2358,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B12">
         <v>968237.39</v>
@@ -2320,7 +2369,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B13">
         <v>1011677.95</v>
@@ -2331,7 +2380,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B14">
         <v>1580293.02</v>
@@ -2342,7 +2391,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -2353,7 +2402,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B16">
         <v>63746.85</v>
@@ -2364,7 +2413,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B17">
         <v>947931.1</v>
@@ -2375,7 +2424,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B18">
         <v>259790.57</v>
@@ -2386,7 +2435,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B19">
         <v>170479.3</v>
@@ -2397,7 +2446,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B20">
         <v>1500000</v>
@@ -2408,7 +2457,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B21">
         <v>1000001.64</v>
@@ -2419,7 +2468,7 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B22">
         <v>68405.66</v>
@@ -2430,7 +2479,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B23">
         <v>1157673.06</v>
@@ -2441,7 +2490,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B24">
         <v>34065.36</v>
@@ -2452,7 +2501,7 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B25">
         <v>843261.89</v>
@@ -2463,7 +2512,7 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -2474,7 +2523,7 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -2485,7 +2534,7 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B28">
         <v>0</v>
@@ -2496,7 +2545,7 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -2507,7 +2556,7 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B30">
         <v>0</v>
@@ -2518,7 +2567,7 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B31">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (06/08/2026 21:44)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="152">
   <si>
     <t>numero_contrato</t>
   </si>
@@ -473,6 +473,9 @@
   </si>
   <si>
     <t>2026NE000944</t>
+  </si>
+  <si>
+    <t>2026NE900959</t>
   </si>
 </sst>
 </file>
@@ -482,16 +485,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -507,7 +502,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -515,30 +510,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -838,37 +815,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -918,58 +895,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -986,13 +963,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>69</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1027,13 +1004,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>70</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1068,13 +1045,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>71</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1109,13 +1086,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>72</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1150,13 +1127,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>73</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1194,13 +1171,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>74</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1235,13 +1212,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>75</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1276,13 +1253,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>76</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1314,13 +1291,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>77</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1355,13 +1332,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>78</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1396,13 +1373,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>79</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1434,13 +1411,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>80</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1472,13 +1449,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>81</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1513,13 +1490,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>82</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1554,13 +1531,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>83</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1595,13 +1572,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>83</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1636,13 +1613,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>83</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1677,13 +1654,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>84</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1718,13 +1695,13 @@
       <c r="D20">
         <v>402</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>45791</v>
       </c>
       <c r="F20" t="s">
         <v>85</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>45834</v>
       </c>
       <c r="I20">
@@ -1759,13 +1736,13 @@
       <c r="D21">
         <v>447</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45814</v>
       </c>
       <c r="F21" t="s">
         <v>86</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45955</v>
       </c>
       <c r="I21">
@@ -1803,13 +1780,13 @@
       <c r="D22">
         <v>529</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45853</v>
       </c>
       <c r="F22" t="s">
         <v>87</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45939</v>
       </c>
       <c r="I22">
@@ -1847,13 +1824,13 @@
       <c r="D23">
         <v>691</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45910</v>
       </c>
       <c r="F23" t="s">
         <v>87</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45941</v>
       </c>
       <c r="I23">
@@ -1891,13 +1868,13 @@
       <c r="D24">
         <v>677</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45904</v>
       </c>
       <c r="F24" t="s">
         <v>72</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45935</v>
       </c>
       <c r="I24">
@@ -1932,13 +1909,13 @@
       <c r="D25">
         <v>278</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>46008</v>
       </c>
       <c r="F25" t="s">
         <v>88</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46066</v>
       </c>
       <c r="I25">
@@ -1973,13 +1950,13 @@
       <c r="D26">
         <v>748</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45930</v>
       </c>
       <c r="F26" t="s">
         <v>89</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2014,13 +1991,13 @@
       <c r="D27">
         <v>822</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45968</v>
       </c>
       <c r="F27" t="s">
         <v>90</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2055,13 +2032,13 @@
       <c r="D28">
         <v>360</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>46043</v>
       </c>
       <c r="F28" t="s">
         <v>80</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46075</v>
       </c>
       <c r="I28">
@@ -2153,13 +2130,13 @@
       <c r="D32">
         <v>1465</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>46104</v>
       </c>
       <c r="F32" t="s">
         <v>80</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46106</v>
       </c>
       <c r="I32">
@@ -2191,13 +2168,13 @@
       <c r="D33">
         <v>1882</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46199</v>
       </c>
       <c r="F33" t="s">
         <v>91</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46233</v>
       </c>
       <c r="I33">
@@ -2226,23 +2203,23 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>127</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>128</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>129</v>
       </c>
     </row>
@@ -2574,6 +2551,17 @@
       </c>
       <c r="C31">
         <v>173846.38</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>151</v>
+      </c>
+      <c r="B32">
+        <v>0</v>
+      </c>
+      <c r="C32">
+        <v>236343.68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização manual: pagamentos (06/08/2026, 2ª checagem)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="152">
   <si>
     <t>numero_contrato</t>
   </si>
@@ -473,6 +473,9 @@
   </si>
   <si>
     <t>2026NE000944</t>
+  </si>
+  <si>
+    <t>2026NE900959</t>
   </si>
 </sst>
 </file>
@@ -2226,7 +2229,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2576,6 +2579,17 @@
         <v>173846.38</v>
       </c>
     </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>151</v>
+      </c>
+      <c r="B32">
+        <v>0</v>
+      </c>
+      <c r="C32">
+        <v>236343.68</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualização manual: pagamentos e empenhos (11/08/2026)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -475,7 +475,7 @@
     <t>2026NE000944</t>
   </si>
   <si>
-    <t>2026NE900959</t>
+    <t>2026NE001015</t>
   </si>
 </sst>
 </file>
@@ -485,8 +485,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -502,7 +510,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -510,12 +518,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -815,37 +841,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -895,58 +921,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -963,13 +989,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>69</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1004,13 +1030,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>70</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1045,13 +1071,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>71</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1086,13 +1112,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>72</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1127,13 +1153,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>73</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1171,13 +1197,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>74</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1212,13 +1238,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>75</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1253,13 +1279,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>76</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1291,13 +1317,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>77</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1332,13 +1358,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>78</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1373,13 +1399,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>79</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1411,13 +1437,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>80</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1449,13 +1475,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>81</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1490,13 +1516,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>82</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1531,13 +1557,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>83</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1572,13 +1598,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>83</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1613,13 +1639,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>83</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1654,13 +1680,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>84</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1695,13 +1721,13 @@
       <c r="D20">
         <v>402</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>45791</v>
       </c>
       <c r="F20" t="s">
         <v>85</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>45834</v>
       </c>
       <c r="I20">
@@ -1736,13 +1762,13 @@
       <c r="D21">
         <v>447</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45814</v>
       </c>
       <c r="F21" t="s">
         <v>86</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45955</v>
       </c>
       <c r="I21">
@@ -1780,13 +1806,13 @@
       <c r="D22">
         <v>529</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45853</v>
       </c>
       <c r="F22" t="s">
         <v>87</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45939</v>
       </c>
       <c r="I22">
@@ -1824,13 +1850,13 @@
       <c r="D23">
         <v>691</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45910</v>
       </c>
       <c r="F23" t="s">
         <v>87</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45941</v>
       </c>
       <c r="I23">
@@ -1868,13 +1894,13 @@
       <c r="D24">
         <v>677</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45904</v>
       </c>
       <c r="F24" t="s">
         <v>72</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45935</v>
       </c>
       <c r="I24">
@@ -1909,13 +1935,13 @@
       <c r="D25">
         <v>278</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>46008</v>
       </c>
       <c r="F25" t="s">
         <v>88</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46066</v>
       </c>
       <c r="I25">
@@ -1950,13 +1976,13 @@
       <c r="D26">
         <v>748</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45930</v>
       </c>
       <c r="F26" t="s">
         <v>89</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -1991,13 +2017,13 @@
       <c r="D27">
         <v>822</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45968</v>
       </c>
       <c r="F27" t="s">
         <v>90</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2032,13 +2058,13 @@
       <c r="D28">
         <v>360</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>46043</v>
       </c>
       <c r="F28" t="s">
         <v>80</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46075</v>
       </c>
       <c r="I28">
@@ -2130,13 +2156,13 @@
       <c r="D32">
         <v>1465</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E32" s="2">
         <v>46104</v>
       </c>
       <c r="F32" t="s">
         <v>80</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46106</v>
       </c>
       <c r="I32">
@@ -2168,13 +2194,13 @@
       <c r="D33">
         <v>1882</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46199</v>
       </c>
       <c r="F33" t="s">
         <v>91</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46233</v>
       </c>
       <c r="I33">
@@ -2207,19 +2233,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>129</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (14/08/2026 18:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -485,16 +485,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -510,7 +502,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -518,30 +510,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -841,37 +815,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -921,58 +895,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -989,13 +963,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>69</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1030,13 +1004,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>70</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1071,13 +1045,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>71</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1112,13 +1086,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>72</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1153,13 +1127,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>73</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1197,13 +1171,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>74</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1238,13 +1212,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>75</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1279,13 +1253,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>76</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1317,13 +1291,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>77</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1358,13 +1332,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>78</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1399,13 +1373,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>79</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1437,13 +1411,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>80</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1475,13 +1449,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>81</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1516,13 +1490,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>82</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1557,13 +1531,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>83</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1598,13 +1572,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>83</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1639,13 +1613,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>83</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1680,13 +1654,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>84</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1721,13 +1695,13 @@
       <c r="D20">
         <v>402</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>45791</v>
       </c>
       <c r="F20" t="s">
         <v>85</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>45834</v>
       </c>
       <c r="I20">
@@ -1762,13 +1736,13 @@
       <c r="D21">
         <v>447</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45814</v>
       </c>
       <c r="F21" t="s">
         <v>86</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45955</v>
       </c>
       <c r="I21">
@@ -1806,13 +1780,13 @@
       <c r="D22">
         <v>529</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45853</v>
       </c>
       <c r="F22" t="s">
         <v>87</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45939</v>
       </c>
       <c r="I22">
@@ -1850,13 +1824,13 @@
       <c r="D23">
         <v>691</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45910</v>
       </c>
       <c r="F23" t="s">
         <v>87</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45941</v>
       </c>
       <c r="I23">
@@ -1894,13 +1868,13 @@
       <c r="D24">
         <v>677</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45904</v>
       </c>
       <c r="F24" t="s">
         <v>72</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45935</v>
       </c>
       <c r="I24">
@@ -1935,13 +1909,13 @@
       <c r="D25">
         <v>278</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>46008</v>
       </c>
       <c r="F25" t="s">
         <v>88</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46066</v>
       </c>
       <c r="I25">
@@ -1976,13 +1950,13 @@
       <c r="D26">
         <v>748</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45930</v>
       </c>
       <c r="F26" t="s">
         <v>89</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2017,13 +1991,13 @@
       <c r="D27">
         <v>822</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45968</v>
       </c>
       <c r="F27" t="s">
         <v>90</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2058,13 +2032,13 @@
       <c r="D28">
         <v>360</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>46043</v>
       </c>
       <c r="F28" t="s">
         <v>80</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46075</v>
       </c>
       <c r="I28">
@@ -2156,13 +2130,13 @@
       <c r="D32">
         <v>1465</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>46104</v>
       </c>
       <c r="F32" t="s">
         <v>80</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46106</v>
       </c>
       <c r="I32">
@@ -2194,13 +2168,13 @@
       <c r="D33">
         <v>1882</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46199</v>
       </c>
       <c r="F33" t="s">
         <v>91</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46233</v>
       </c>
       <c r="I33">
@@ -2233,19 +2207,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>127</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>128</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>129</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza Disponibilidade Diária (17/08) e Pagamentos/Empenhos
Disponibilidade: relatório de 17/08/2026, 31 relatórios/899 aeronaves-linha
no total, sem inconsistências (rodado em processo isolado, sem o bug de
common.py cruzado entre áreas).

Pagamentos: 32 lançamentos, mesmas inconsistências conhecidas de
formatação e o mesmo gap não resolvido do empenho 2025NE000005.

Inclui também 2026-07_vee_one.csv (gerado num teste anterior desta sessão,
ficou pendente de commit).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -485,8 +485,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -502,7 +510,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -510,12 +518,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -815,37 +841,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -895,58 +921,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -963,13 +989,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>69</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1004,13 +1030,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>70</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1045,13 +1071,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>71</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1086,13 +1112,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>72</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1127,13 +1153,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>73</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1171,13 +1197,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>74</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1212,13 +1238,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>75</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1253,13 +1279,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>76</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1291,13 +1317,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>77</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1332,13 +1358,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>78</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1373,13 +1399,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>79</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1411,13 +1437,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>80</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1449,13 +1475,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>81</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1490,13 +1516,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>82</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1531,13 +1557,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>83</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1572,13 +1598,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>83</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1613,13 +1639,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>83</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1654,13 +1680,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>84</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1695,13 +1721,13 @@
       <c r="D20">
         <v>402</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>45791</v>
       </c>
       <c r="F20" t="s">
         <v>85</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>45834</v>
       </c>
       <c r="I20">
@@ -1736,13 +1762,13 @@
       <c r="D21">
         <v>447</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45814</v>
       </c>
       <c r="F21" t="s">
         <v>86</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45955</v>
       </c>
       <c r="I21">
@@ -1780,13 +1806,13 @@
       <c r="D22">
         <v>529</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45853</v>
       </c>
       <c r="F22" t="s">
         <v>87</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45939</v>
       </c>
       <c r="I22">
@@ -1824,13 +1850,13 @@
       <c r="D23">
         <v>691</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45910</v>
       </c>
       <c r="F23" t="s">
         <v>87</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45941</v>
       </c>
       <c r="I23">
@@ -1868,13 +1894,13 @@
       <c r="D24">
         <v>677</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45904</v>
       </c>
       <c r="F24" t="s">
         <v>72</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45935</v>
       </c>
       <c r="I24">
@@ -1909,13 +1935,13 @@
       <c r="D25">
         <v>278</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>46008</v>
       </c>
       <c r="F25" t="s">
         <v>88</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46066</v>
       </c>
       <c r="I25">
@@ -1950,13 +1976,13 @@
       <c r="D26">
         <v>748</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45930</v>
       </c>
       <c r="F26" t="s">
         <v>89</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -1991,13 +2017,13 @@
       <c r="D27">
         <v>822</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45968</v>
       </c>
       <c r="F27" t="s">
         <v>90</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2032,13 +2058,13 @@
       <c r="D28">
         <v>360</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>46043</v>
       </c>
       <c r="F28" t="s">
         <v>80</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46075</v>
       </c>
       <c r="I28">
@@ -2130,13 +2156,13 @@
       <c r="D32">
         <v>1465</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E32" s="2">
         <v>46104</v>
       </c>
       <c r="F32" t="s">
         <v>80</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46106</v>
       </c>
       <c r="I32">
@@ -2168,13 +2194,13 @@
       <c r="D33">
         <v>1882</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46199</v>
       </c>
       <c r="F33" t="s">
         <v>91</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46233</v>
       </c>
       <c r="I33">
@@ -2207,19 +2233,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>129</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (17/08/2026 12:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -485,16 +485,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -510,7 +502,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -518,30 +510,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -841,37 +815,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -921,58 +895,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -989,13 +963,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>69</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1030,13 +1004,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>70</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1071,13 +1045,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>71</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1112,13 +1086,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>72</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1153,13 +1127,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>73</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1197,13 +1171,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>74</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1238,13 +1212,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>75</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1279,13 +1253,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>76</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1317,13 +1291,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>77</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1358,13 +1332,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>78</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1399,13 +1373,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>79</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1437,13 +1411,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>80</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1475,13 +1449,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>81</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1516,13 +1490,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>82</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1557,13 +1531,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>83</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1598,13 +1572,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>83</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1639,13 +1613,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>83</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1680,13 +1654,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>84</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1721,13 +1695,13 @@
       <c r="D20">
         <v>402</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>45791</v>
       </c>
       <c r="F20" t="s">
         <v>85</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>45834</v>
       </c>
       <c r="I20">
@@ -1762,13 +1736,13 @@
       <c r="D21">
         <v>447</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45814</v>
       </c>
       <c r="F21" t="s">
         <v>86</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45955</v>
       </c>
       <c r="I21">
@@ -1806,13 +1780,13 @@
       <c r="D22">
         <v>529</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45853</v>
       </c>
       <c r="F22" t="s">
         <v>87</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45939</v>
       </c>
       <c r="I22">
@@ -1850,13 +1824,13 @@
       <c r="D23">
         <v>691</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45910</v>
       </c>
       <c r="F23" t="s">
         <v>87</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45941</v>
       </c>
       <c r="I23">
@@ -1894,13 +1868,13 @@
       <c r="D24">
         <v>677</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45904</v>
       </c>
       <c r="F24" t="s">
         <v>72</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45935</v>
       </c>
       <c r="I24">
@@ -1935,13 +1909,13 @@
       <c r="D25">
         <v>278</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>46008</v>
       </c>
       <c r="F25" t="s">
         <v>88</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46066</v>
       </c>
       <c r="I25">
@@ -1976,13 +1950,13 @@
       <c r="D26">
         <v>748</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45930</v>
       </c>
       <c r="F26" t="s">
         <v>89</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2017,13 +1991,13 @@
       <c r="D27">
         <v>822</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45968</v>
       </c>
       <c r="F27" t="s">
         <v>90</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2058,13 +2032,13 @@
       <c r="D28">
         <v>360</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>46043</v>
       </c>
       <c r="F28" t="s">
         <v>80</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46075</v>
       </c>
       <c r="I28">
@@ -2156,13 +2130,13 @@
       <c r="D32">
         <v>1465</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>46104</v>
       </c>
       <c r="F32" t="s">
         <v>80</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46106</v>
       </c>
       <c r="I32">
@@ -2194,13 +2168,13 @@
       <c r="D33">
         <v>1882</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46199</v>
       </c>
       <c r="F33" t="s">
         <v>91</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46233</v>
       </c>
       <c r="I33">
@@ -2233,19 +2207,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>127</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>128</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>129</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (18/08/2026 12:31)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -485,8 +485,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -502,7 +510,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -510,12 +518,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -815,37 +841,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -895,58 +921,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -963,13 +989,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>69</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1004,13 +1030,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>70</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1045,13 +1071,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>71</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1086,13 +1112,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>72</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1127,13 +1153,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>73</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1171,13 +1197,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>74</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1212,13 +1238,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>75</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1253,13 +1279,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>76</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1291,13 +1317,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>77</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1332,13 +1358,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>78</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1373,13 +1399,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>79</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1411,13 +1437,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>80</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1449,13 +1475,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>81</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1490,13 +1516,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>82</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1531,13 +1557,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>83</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1572,13 +1598,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>83</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1613,13 +1639,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>83</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1654,13 +1680,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>84</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1695,13 +1721,13 @@
       <c r="D20">
         <v>402</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>45791</v>
       </c>
       <c r="F20" t="s">
         <v>85</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>45834</v>
       </c>
       <c r="I20">
@@ -1736,13 +1762,13 @@
       <c r="D21">
         <v>447</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45814</v>
       </c>
       <c r="F21" t="s">
         <v>86</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45955</v>
       </c>
       <c r="I21">
@@ -1780,13 +1806,13 @@
       <c r="D22">
         <v>529</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45853</v>
       </c>
       <c r="F22" t="s">
         <v>87</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45939</v>
       </c>
       <c r="I22">
@@ -1824,13 +1850,13 @@
       <c r="D23">
         <v>691</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45910</v>
       </c>
       <c r="F23" t="s">
         <v>87</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45941</v>
       </c>
       <c r="I23">
@@ -1868,13 +1894,13 @@
       <c r="D24">
         <v>677</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45904</v>
       </c>
       <c r="F24" t="s">
         <v>72</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45935</v>
       </c>
       <c r="I24">
@@ -1909,13 +1935,13 @@
       <c r="D25">
         <v>278</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>46008</v>
       </c>
       <c r="F25" t="s">
         <v>88</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>46066</v>
       </c>
       <c r="I25">
@@ -1950,13 +1976,13 @@
       <c r="D26">
         <v>748</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>45930</v>
       </c>
       <c r="F26" t="s">
         <v>89</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -1991,13 +2017,13 @@
       <c r="D27">
         <v>822</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45968</v>
       </c>
       <c r="F27" t="s">
         <v>90</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2032,13 +2058,13 @@
       <c r="D28">
         <v>360</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>46043</v>
       </c>
       <c r="F28" t="s">
         <v>80</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>46075</v>
       </c>
       <c r="I28">
@@ -2130,13 +2156,13 @@
       <c r="D32">
         <v>1465</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E32" s="2">
         <v>46104</v>
       </c>
       <c r="F32" t="s">
         <v>80</v>
       </c>
-      <c r="H32" s="1">
+      <c r="H32" s="2">
         <v>46106</v>
       </c>
       <c r="I32">
@@ -2168,13 +2194,13 @@
       <c r="D33">
         <v>1882</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46199</v>
       </c>
       <c r="F33" t="s">
         <v>91</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46233</v>
       </c>
       <c r="I33">
@@ -2207,19 +2233,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>129</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (18/08/2026 12:39)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -485,16 +485,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -510,7 +502,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -518,30 +510,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -841,37 +815,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -921,58 +895,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -989,13 +963,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>69</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1030,13 +1004,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>70</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1071,13 +1045,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>71</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1112,13 +1086,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>72</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1153,13 +1127,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>73</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1197,13 +1171,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>74</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1238,13 +1212,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>75</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1279,13 +1253,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>76</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1317,13 +1291,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>77</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1358,13 +1332,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>78</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1399,13 +1373,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>79</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1437,13 +1411,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>80</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1475,13 +1449,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>81</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1516,13 +1490,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>82</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1557,13 +1531,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>83</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1598,13 +1572,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>83</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1639,13 +1613,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>83</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1680,13 +1654,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>84</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1721,13 +1695,13 @@
       <c r="D20">
         <v>402</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>45791</v>
       </c>
       <c r="F20" t="s">
         <v>85</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>45834</v>
       </c>
       <c r="I20">
@@ -1762,13 +1736,13 @@
       <c r="D21">
         <v>447</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45814</v>
       </c>
       <c r="F21" t="s">
         <v>86</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45955</v>
       </c>
       <c r="I21">
@@ -1806,13 +1780,13 @@
       <c r="D22">
         <v>529</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45853</v>
       </c>
       <c r="F22" t="s">
         <v>87</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45939</v>
       </c>
       <c r="I22">
@@ -1850,13 +1824,13 @@
       <c r="D23">
         <v>691</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45910</v>
       </c>
       <c r="F23" t="s">
         <v>87</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45941</v>
       </c>
       <c r="I23">
@@ -1894,13 +1868,13 @@
       <c r="D24">
         <v>677</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45904</v>
       </c>
       <c r="F24" t="s">
         <v>72</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45935</v>
       </c>
       <c r="I24">
@@ -1935,13 +1909,13 @@
       <c r="D25">
         <v>278</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>46008</v>
       </c>
       <c r="F25" t="s">
         <v>88</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>46066</v>
       </c>
       <c r="I25">
@@ -1976,13 +1950,13 @@
       <c r="D26">
         <v>748</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>45930</v>
       </c>
       <c r="F26" t="s">
         <v>89</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>45935</v>
       </c>
       <c r="I26">
@@ -2017,13 +1991,13 @@
       <c r="D27">
         <v>822</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45968</v>
       </c>
       <c r="F27" t="s">
         <v>90</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2058,13 +2032,13 @@
       <c r="D28">
         <v>360</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>46043</v>
       </c>
       <c r="F28" t="s">
         <v>80</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>46075</v>
       </c>
       <c r="I28">
@@ -2156,13 +2130,13 @@
       <c r="D32">
         <v>1465</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="1">
         <v>46104</v>
       </c>
       <c r="F32" t="s">
         <v>80</v>
       </c>
-      <c r="H32" s="2">
+      <c r="H32" s="1">
         <v>46106</v>
       </c>
       <c r="I32">
@@ -2194,13 +2168,13 @@
       <c r="D33">
         <v>1882</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46199</v>
       </c>
       <c r="F33" t="s">
         <v>91</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46233</v>
       </c>
       <c r="I33">
@@ -2233,19 +2207,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>127</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>128</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>129</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (19/08/2026 10:51)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="153">
   <si>
     <t>numero_contrato</t>
   </si>
@@ -172,6 +172,9 @@
   </si>
   <si>
     <t>JUNHO/26</t>
+  </si>
+  <si>
+    <t>JULHO/26</t>
   </si>
   <si>
     <t>Módulo II – Parcial Orçamento 10 (FAB 2728)</t>
@@ -891,7 +894,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R33"/>
+  <dimension ref="A1:R34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
@@ -958,7 +961,7 @@
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D2">
         <v>594</v>
@@ -967,7 +970,7 @@
         <v>45740</v>
       </c>
       <c r="F2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H2" s="1">
         <v>45778</v>
@@ -976,16 +979,16 @@
         <v>748504.24</v>
       </c>
       <c r="J2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="K2">
         <v>748504.24</v>
       </c>
       <c r="M2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P2">
         <v>881914.1800000001</v>
@@ -999,7 +1002,7 @@
         <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D3">
         <v>620</v>
@@ -1008,7 +1011,7 @@
         <v>45775</v>
       </c>
       <c r="F3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H3" s="1">
         <v>45806</v>
@@ -1017,16 +1020,16 @@
         <v>1110378.24</v>
       </c>
       <c r="J3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="K3">
         <v>1110378.24</v>
       </c>
       <c r="M3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P3">
         <v>2634000</v>
@@ -1040,7 +1043,7 @@
         <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D4">
         <v>634</v>
@@ -1049,7 +1052,7 @@
         <v>45799</v>
       </c>
       <c r="F4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H4" s="1">
         <v>45844</v>
@@ -1058,16 +1061,16 @@
         <v>974557.12</v>
       </c>
       <c r="J4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K4">
         <v>974557.12</v>
       </c>
       <c r="M4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P4">
         <v>1686034.96</v>
@@ -1081,7 +1084,7 @@
         <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D5">
         <v>660</v>
@@ -1090,7 +1093,7 @@
         <v>45856</v>
       </c>
       <c r="F5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H5" s="1">
         <v>45891</v>
@@ -1099,16 +1102,16 @@
         <v>1402001.34</v>
       </c>
       <c r="J5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K5">
         <v>1402001.34</v>
       </c>
       <c r="M5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P5">
         <v>1600334.09</v>
@@ -1122,7 +1125,7 @@
         <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D6">
         <v>661</v>
@@ -1131,7 +1134,7 @@
         <v>45856</v>
       </c>
       <c r="F6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H6" s="1">
         <v>45891</v>
@@ -1140,16 +1143,16 @@
         <v>1223702.3</v>
       </c>
       <c r="J6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K6">
         <v>1223702.3</v>
       </c>
       <c r="M6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="O6">
         <v>0.02</v>
@@ -1166,7 +1169,7 @@
         <v>39</v>
       </c>
       <c r="C7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D7">
         <v>688</v>
@@ -1175,7 +1178,7 @@
         <v>45901</v>
       </c>
       <c r="F7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H7" s="1">
         <v>45938</v>
@@ -1184,16 +1187,16 @@
         <v>1011677.95</v>
       </c>
       <c r="J7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K7">
         <v>1011677.95</v>
       </c>
       <c r="M7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P7">
         <v>2568571.48</v>
@@ -1207,7 +1210,7 @@
         <v>40</v>
       </c>
       <c r="C8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D8">
         <v>696</v>
@@ -1216,7 +1219,7 @@
         <v>45923</v>
       </c>
       <c r="F8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H8" s="1">
         <v>45938</v>
@@ -1225,16 +1228,16 @@
         <v>896744.0600000001</v>
       </c>
       <c r="J8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K8">
         <v>896744.0600000001</v>
       </c>
       <c r="M8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N8" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P8">
         <v>968237.39</v>
@@ -1248,7 +1251,7 @@
         <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D9">
         <v>704</v>
@@ -1257,7 +1260,7 @@
         <v>45957</v>
       </c>
       <c r="F9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H9" s="1">
         <v>46003</v>
@@ -1266,16 +1269,16 @@
         <v>919329.0600000001</v>
       </c>
       <c r="J9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K9">
         <v>919329.0600000001</v>
       </c>
       <c r="M9" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P9">
         <v>1947932.74</v>
@@ -1295,7 +1298,7 @@
         <v>45972</v>
       </c>
       <c r="F10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H10" s="1">
         <v>46016</v>
@@ -1304,16 +1307,16 @@
         <v>1157009.26</v>
       </c>
       <c r="J10" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K10">
         <v>1157009.26</v>
       </c>
       <c r="M10" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P10">
         <v>3105605.8</v>
@@ -1327,7 +1330,7 @@
         <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D11">
         <v>728</v>
@@ -1336,7 +1339,7 @@
         <v>46008</v>
       </c>
       <c r="F11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H11" s="1">
         <v>46040</v>
@@ -1345,16 +1348,16 @@
         <v>1214597.952</v>
       </c>
       <c r="J11" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K11">
         <v>1214597.952</v>
       </c>
       <c r="M11" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N11" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P11">
         <v>2096487.74</v>
@@ -1368,7 +1371,7 @@
         <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D12">
         <v>278</v>
@@ -1377,7 +1380,7 @@
         <v>46042</v>
       </c>
       <c r="F12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H12" s="1">
         <v>46074</v>
@@ -1386,16 +1389,16 @@
         <v>967082.09</v>
       </c>
       <c r="J12" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K12">
         <v>967082.09</v>
       </c>
       <c r="M12" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N12" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P12">
         <v>3522444.13</v>
@@ -1415,7 +1418,7 @@
         <v>46078</v>
       </c>
       <c r="F13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H13" s="1">
         <v>46106</v>
@@ -1424,16 +1427,16 @@
         <v>719561.08</v>
       </c>
       <c r="J13" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K13">
         <v>719561.08</v>
       </c>
       <c r="M13" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P13">
         <v>1500000</v>
@@ -1453,7 +1456,7 @@
         <v>46094</v>
       </c>
       <c r="F14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H14" s="1">
         <v>46128</v>
@@ -1462,16 +1465,16 @@
         <v>885881.08</v>
       </c>
       <c r="J14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K14">
         <v>885881.08</v>
       </c>
       <c r="M14" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N14" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="O14">
         <v>34065.36</v>
@@ -1494,7 +1497,7 @@
         <v>46128</v>
       </c>
       <c r="F15" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H15" s="1">
         <v>46164</v>
@@ -1503,16 +1506,16 @@
         <v>1350542.52</v>
       </c>
       <c r="J15" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K15">
         <v>1350542.52</v>
       </c>
       <c r="M15" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N15" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="O15">
         <v>0.01</v>
@@ -1535,7 +1538,7 @@
         <v>46156</v>
       </c>
       <c r="F16" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H16" s="1">
         <v>46191</v>
@@ -1544,16 +1547,16 @@
         <v>1108954.435833333</v>
       </c>
       <c r="J16" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K16">
         <v>1108954.435833333</v>
       </c>
       <c r="M16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N16" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="O16">
         <v>0.01</v>
@@ -1576,7 +1579,7 @@
         <v>46149</v>
       </c>
       <c r="F17" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H17" s="1">
         <v>46185</v>
@@ -1585,16 +1588,16 @@
         <v>218206.1</v>
       </c>
       <c r="J17" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K17">
         <v>218206.1</v>
       </c>
       <c r="M17" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N17" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="O17">
         <v>0.01</v>
@@ -1617,7 +1620,7 @@
         <v>46156</v>
       </c>
       <c r="F18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H18" s="1">
         <v>46191</v>
@@ -1626,16 +1629,16 @@
         <v>1549250.84</v>
       </c>
       <c r="J18" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K18">
         <v>1549250.84</v>
       </c>
       <c r="M18" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N18" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="O18">
         <v>0.01</v>
@@ -1658,7 +1661,7 @@
         <v>46230</v>
       </c>
       <c r="F19" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H19" s="1">
         <v>46262</v>
@@ -1667,16 +1670,16 @@
         <v>1340865.98</v>
       </c>
       <c r="J19" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="K19">
         <v>1340865.98</v>
       </c>
       <c r="M19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N19" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="O19">
         <v>927618.61</v>
@@ -1687,40 +1690,19 @@
     </row>
     <row r="20" spans="1:16">
       <c r="A20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B20" t="s">
         <v>52</v>
       </c>
-      <c r="D20">
-        <v>402</v>
-      </c>
-      <c r="E20" s="1">
-        <v>45791</v>
-      </c>
-      <c r="F20" t="s">
-        <v>85</v>
-      </c>
-      <c r="H20" s="1">
-        <v>45834</v>
-      </c>
-      <c r="I20">
-        <v>188246.17</v>
-      </c>
-      <c r="J20" t="s">
-        <v>110</v>
-      </c>
-      <c r="K20">
-        <v>188246.17</v>
+      <c r="L20">
+        <v>1629834.48</v>
       </c>
       <c r="M20" t="s">
         <v>122</v>
       </c>
       <c r="N20" t="s">
-        <v>123</v>
-      </c>
-      <c r="P20">
-        <v>211614.23</v>
+        <v>125</v>
       </c>
     </row>
     <row r="21" spans="1:16">
@@ -1730,41 +1712,35 @@
       <c r="B21" t="s">
         <v>53</v>
       </c>
-      <c r="C21">
-        <v>46</v>
-      </c>
       <c r="D21">
-        <v>447</v>
+        <v>402</v>
       </c>
       <c r="E21" s="1">
-        <v>45814</v>
+        <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>86</v>
       </c>
       <c r="H21" s="1">
-        <v>45955</v>
+        <v>45834</v>
       </c>
       <c r="I21">
-        <v>112720.77</v>
+        <v>188246.17</v>
       </c>
       <c r="J21" t="s">
         <v>111</v>
       </c>
       <c r="K21">
-        <v>112720.77</v>
+        <v>188246.17</v>
       </c>
       <c r="M21" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N21" t="s">
-        <v>123</v>
-      </c>
-      <c r="O21">
-        <v>0.01</v>
+        <v>124</v>
       </c>
       <c r="P21">
-        <v>3359394.8</v>
+        <v>211614.23</v>
       </c>
     </row>
     <row r="22" spans="1:16">
@@ -1774,41 +1750,41 @@
       <c r="B22" t="s">
         <v>54</v>
       </c>
-      <c r="C22" t="s">
-        <v>67</v>
+      <c r="C22">
+        <v>46</v>
       </c>
       <c r="D22">
-        <v>529</v>
+        <v>447</v>
       </c>
       <c r="E22" s="1">
-        <v>45853</v>
+        <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>87</v>
       </c>
       <c r="H22" s="1">
-        <v>45939</v>
+        <v>45955</v>
       </c>
       <c r="I22">
-        <v>378307.61</v>
+        <v>112720.77</v>
       </c>
       <c r="J22" t="s">
         <v>112</v>
       </c>
       <c r="K22">
-        <v>378307.61</v>
+        <v>112720.77</v>
       </c>
       <c r="M22" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="O22">
         <v>0.01</v>
       </c>
       <c r="P22">
-        <v>2391157.41</v>
+        <v>3359394.8</v>
       </c>
     </row>
     <row r="23" spans="1:16">
@@ -1819,34 +1795,34 @@
         <v>55</v>
       </c>
       <c r="C23" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D23">
-        <v>691</v>
+        <v>529</v>
       </c>
       <c r="E23" s="1">
-        <v>45910</v>
+        <v>45853</v>
       </c>
       <c r="F23" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H23" s="1">
-        <v>45941</v>
+        <v>45939</v>
       </c>
       <c r="I23">
-        <v>3315.047100000025</v>
+        <v>378307.61</v>
       </c>
       <c r="J23" t="s">
         <v>113</v>
       </c>
       <c r="K23">
-        <v>3315.04710000003</v>
+        <v>378307.61</v>
       </c>
       <c r="M23" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N23" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="O23">
         <v>0.01</v>
@@ -1862,38 +1838,41 @@
       <c r="B24" t="s">
         <v>56</v>
       </c>
-      <c r="C24">
-        <v>135</v>
+      <c r="C24" t="s">
+        <v>68</v>
       </c>
       <c r="D24">
-        <v>677</v>
+        <v>691</v>
       </c>
       <c r="E24" s="1">
-        <v>45904</v>
+        <v>45910</v>
       </c>
       <c r="F24" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="H24" s="1">
-        <v>45935</v>
+        <v>45941</v>
       </c>
       <c r="I24">
-        <v>198332.75</v>
+        <v>3315.047100000025</v>
       </c>
       <c r="J24" t="s">
         <v>114</v>
       </c>
       <c r="K24">
-        <v>198332.75</v>
+        <v>3315.04710000003</v>
       </c>
       <c r="M24" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N24" t="s">
-        <v>123</v>
+        <v>124</v>
+      </c>
+      <c r="O24">
+        <v>0.01</v>
       </c>
       <c r="P24">
-        <v>1600334.09</v>
+        <v>2391157.41</v>
       </c>
     </row>
     <row r="25" spans="1:16">
@@ -1904,37 +1883,37 @@
         <v>57</v>
       </c>
       <c r="C25">
-        <v>40</v>
+        <v>135</v>
       </c>
       <c r="D25">
-        <v>278</v>
+        <v>677</v>
       </c>
       <c r="E25" s="1">
-        <v>46008</v>
+        <v>45904</v>
       </c>
       <c r="F25" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="H25" s="1">
-        <v>46066</v>
+        <v>45935</v>
       </c>
       <c r="I25">
-        <v>1528.62</v>
+        <v>198332.75</v>
       </c>
       <c r="J25" t="s">
         <v>115</v>
       </c>
       <c r="K25">
-        <v>1528.62</v>
+        <v>198332.75</v>
       </c>
       <c r="M25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N25" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P25">
-        <v>1157673.06</v>
+        <v>1600334.09</v>
       </c>
     </row>
     <row r="26" spans="1:16">
@@ -1944,38 +1923,38 @@
       <c r="B26" t="s">
         <v>58</v>
       </c>
-      <c r="C26" t="s">
-        <v>68</v>
+      <c r="C26">
+        <v>40</v>
       </c>
       <c r="D26">
-        <v>748</v>
+        <v>278</v>
       </c>
       <c r="E26" s="1">
-        <v>45930</v>
+        <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>89</v>
       </c>
       <c r="H26" s="1">
-        <v>45935</v>
+        <v>46066</v>
       </c>
       <c r="I26">
-        <v>38718.58</v>
+        <v>1528.62</v>
       </c>
       <c r="J26" t="s">
         <v>116</v>
       </c>
       <c r="K26">
-        <v>38718.58</v>
+        <v>1528.62</v>
       </c>
       <c r="M26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P26">
-        <v>63746.85</v>
+        <v>1157673.06</v>
       </c>
     </row>
     <row r="27" spans="1:16">
@@ -1985,14 +1964,14 @@
       <c r="B27" t="s">
         <v>59</v>
       </c>
-      <c r="C27">
-        <v>154</v>
+      <c r="C27" t="s">
+        <v>69</v>
       </c>
       <c r="D27">
-        <v>822</v>
+        <v>748</v>
       </c>
       <c r="E27" s="1">
-        <v>45968</v>
+        <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>90</v>
@@ -2001,22 +1980,22 @@
         <v>45935</v>
       </c>
       <c r="I27">
-        <v>133124.11</v>
+        <v>38718.58</v>
       </c>
       <c r="J27" t="s">
         <v>117</v>
       </c>
       <c r="K27">
-        <v>133124.11</v>
+        <v>38718.58</v>
       </c>
       <c r="M27" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N27" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P27">
-        <v>1000001.64</v>
+        <v>63746.85</v>
       </c>
     </row>
     <row r="28" spans="1:16">
@@ -2027,37 +2006,37 @@
         <v>60</v>
       </c>
       <c r="C28">
-        <v>252</v>
+        <v>154</v>
       </c>
       <c r="D28">
-        <v>360</v>
+        <v>822</v>
       </c>
       <c r="E28" s="1">
-        <v>46043</v>
+        <v>45968</v>
       </c>
       <c r="F28" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="H28" s="1">
-        <v>46075</v>
+        <v>45935</v>
       </c>
       <c r="I28">
-        <v>11372.9</v>
+        <v>133124.11</v>
       </c>
       <c r="J28" t="s">
         <v>118</v>
       </c>
       <c r="K28">
-        <v>11372.9</v>
+        <v>133124.11</v>
       </c>
       <c r="M28" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N28" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="P28">
-        <v>1500000</v>
+        <v>1000001.64</v>
       </c>
     </row>
     <row r="29" spans="1:16">
@@ -2067,17 +2046,38 @@
       <c r="B29" t="s">
         <v>61</v>
       </c>
-      <c r="G29" t="s">
-        <v>92</v>
-      </c>
-      <c r="L29">
-        <v>15854.78</v>
+      <c r="C29">
+        <v>252</v>
+      </c>
+      <c r="D29">
+        <v>360</v>
+      </c>
+      <c r="E29" s="1">
+        <v>46043</v>
+      </c>
+      <c r="F29" t="s">
+        <v>81</v>
+      </c>
+      <c r="H29" s="1">
+        <v>46075</v>
+      </c>
+      <c r="I29">
+        <v>11372.9</v>
+      </c>
+      <c r="J29" t="s">
+        <v>119</v>
+      </c>
+      <c r="K29">
+        <v>11372.9</v>
       </c>
       <c r="M29" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N29" t="s">
         <v>124</v>
+      </c>
+      <c r="P29">
+        <v>1500000</v>
       </c>
     </row>
     <row r="30" spans="1:16">
@@ -2088,16 +2088,16 @@
         <v>62</v>
       </c>
       <c r="G30" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="L30">
-        <v>42229.72325</v>
+        <v>15854.78</v>
       </c>
       <c r="M30" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N30" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -2108,54 +2108,36 @@
         <v>63</v>
       </c>
       <c r="G31" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="L31">
-        <v>48857.39550000001</v>
+        <v>42229.72325</v>
       </c>
       <c r="M31" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N31" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="32" spans="1:16">
       <c r="A32">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B32" t="s">
         <v>64</v>
       </c>
-      <c r="D32">
-        <v>1465</v>
-      </c>
-      <c r="E32" s="1">
-        <v>46104</v>
-      </c>
-      <c r="F32" t="s">
-        <v>80</v>
-      </c>
-      <c r="H32" s="1">
-        <v>46106</v>
-      </c>
-      <c r="I32">
-        <v>27801.11</v>
-      </c>
-      <c r="J32" t="s">
-        <v>119</v>
-      </c>
-      <c r="K32">
-        <v>27801.11</v>
+      <c r="G32" t="s">
+        <v>93</v>
+      </c>
+      <c r="L32">
+        <v>48857.39550000001</v>
       </c>
       <c r="M32" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N32" t="s">
-        <v>123</v>
-      </c>
-      <c r="P32">
-        <v>1500000</v>
+        <v>125</v>
       </c>
     </row>
     <row r="33" spans="1:16">
@@ -2166,33 +2148,71 @@
         <v>65</v>
       </c>
       <c r="D33">
-        <v>1882</v>
+        <v>1465</v>
       </c>
       <c r="E33" s="1">
-        <v>46199</v>
+        <v>46104</v>
       </c>
       <c r="F33" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="H33" s="1">
-        <v>46233</v>
+        <v>46106</v>
       </c>
       <c r="I33">
-        <v>58868.35</v>
+        <v>27801.11</v>
       </c>
       <c r="J33" t="s">
         <v>120</v>
       </c>
       <c r="K33">
+        <v>27801.11</v>
+      </c>
+      <c r="M33" t="s">
+        <v>123</v>
+      </c>
+      <c r="N33" t="s">
+        <v>124</v>
+      </c>
+      <c r="P33">
+        <v>1500000</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16">
+      <c r="A34">
+        <v>3</v>
+      </c>
+      <c r="B34" t="s">
+        <v>66</v>
+      </c>
+      <c r="D34">
+        <v>1882</v>
+      </c>
+      <c r="E34" s="1">
+        <v>46199</v>
+      </c>
+      <c r="F34" t="s">
+        <v>92</v>
+      </c>
+      <c r="H34" s="1">
+        <v>46233</v>
+      </c>
+      <c r="I34">
         <v>58868.35</v>
       </c>
-      <c r="M33" t="s">
-        <v>122</v>
-      </c>
-      <c r="N33" t="s">
-        <v>125</v>
-      </c>
-      <c r="P33">
+      <c r="J34" t="s">
+        <v>121</v>
+      </c>
+      <c r="K34">
+        <v>58868.35</v>
+      </c>
+      <c r="M34" t="s">
+        <v>123</v>
+      </c>
+      <c r="N34" t="s">
+        <v>126</v>
+      </c>
+      <c r="P34">
         <v>2364771.07</v>
       </c>
     </row>
@@ -2208,24 +2228,24 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B1" t="s">
         <v>7</v>
       </c>
       <c r="C1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B2">
         <v>52250.04</v>
@@ -2236,7 +2256,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B3">
         <v>881914.1800000001</v>
@@ -2247,7 +2267,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B4">
         <v>750000</v>
@@ -2258,7 +2278,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B5">
         <v>949835.78</v>
@@ -2269,7 +2289,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B6">
         <v>524584.95</v>
@@ -2280,7 +2300,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B7">
         <v>211614.23</v>
@@ -2291,7 +2311,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B8">
         <v>2391157.41</v>
@@ -2302,7 +2322,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B9">
         <v>618154.38</v>
@@ -2313,7 +2333,7 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B10">
         <v>1600334.09</v>
@@ -2324,7 +2344,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B11">
         <v>2364771.07</v>
@@ -2335,7 +2355,7 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B12">
         <v>968237.39</v>
@@ -2346,7 +2366,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B13">
         <v>1011677.95</v>
@@ -2357,7 +2377,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B14">
         <v>1580293.02</v>
@@ -2368,7 +2388,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -2379,7 +2399,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B16">
         <v>63746.85</v>
@@ -2390,7 +2410,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B17">
         <v>947931.1</v>
@@ -2401,7 +2421,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B18">
         <v>259790.57</v>
@@ -2412,7 +2432,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B19">
         <v>170479.3</v>
@@ -2423,7 +2443,7 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B20">
         <v>1500000</v>
@@ -2434,7 +2454,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B21">
         <v>1000001.64</v>
@@ -2445,7 +2465,7 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B22">
         <v>68405.66</v>
@@ -2456,7 +2476,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B23">
         <v>1157673.06</v>
@@ -2467,7 +2487,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B24">
         <v>34065.36</v>
@@ -2478,7 +2498,7 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B25">
         <v>843261.89</v>
@@ -2489,7 +2509,7 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -2500,7 +2520,7 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -2511,7 +2531,7 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B28">
         <v>0</v>
@@ -2522,7 +2542,7 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -2533,7 +2553,7 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B30">
         <v>0</v>
@@ -2544,7 +2564,7 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B31">
         <v>0</v>
@@ -2555,7 +2575,7 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B32">
         <v>0</v>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (19/08/2026 13:06)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -488,8 +488,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -505,7 +513,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -513,12 +521,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -818,37 +844,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -898,58 +924,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -966,13 +992,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1007,13 +1033,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1048,13 +1074,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1089,13 +1115,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1130,13 +1156,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1174,13 +1200,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1215,13 +1241,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1256,13 +1282,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1294,13 +1320,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1335,13 +1361,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1376,13 +1402,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1414,13 +1440,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1452,13 +1478,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1493,13 +1519,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1534,13 +1560,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1575,13 +1601,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1616,13 +1642,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1657,13 +1683,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1715,13 +1741,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>86</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1756,13 +1782,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>87</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1800,13 +1826,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>88</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1844,13 +1870,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>88</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1888,13 +1914,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1929,13 +1955,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>89</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -1970,13 +1996,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>90</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2011,13 +2037,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>91</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2052,13 +2078,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2150,13 +2176,13 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46106</v>
       </c>
       <c r="I33">
@@ -2188,13 +2214,13 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
         <v>92</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46233</v>
       </c>
       <c r="I34">
@@ -2227,19 +2253,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>130</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (21/08/2026 09:06)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -488,8 +488,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -505,7 +513,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -513,12 +521,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -818,37 +844,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -898,58 +924,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -966,13 +992,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1007,13 +1033,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1048,13 +1074,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1089,13 +1115,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1130,13 +1156,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1174,13 +1200,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1215,13 +1241,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1256,13 +1282,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1294,13 +1320,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1335,13 +1361,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1376,13 +1402,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1414,13 +1440,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1452,13 +1478,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1493,13 +1519,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1534,13 +1560,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1575,13 +1601,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1616,13 +1642,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1657,13 +1683,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1715,13 +1741,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>86</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1756,13 +1782,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>87</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1800,13 +1826,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>88</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1844,13 +1870,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>88</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1888,13 +1914,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1929,13 +1955,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>89</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -1970,13 +1996,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>90</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2011,13 +2037,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>91</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2052,13 +2078,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2150,13 +2176,13 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46106</v>
       </c>
       <c r="I33">
@@ -2188,13 +2214,13 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
         <v>92</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46233</v>
       </c>
       <c r="I34">
@@ -2227,19 +2253,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>130</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (21/08/2026 10:51)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -488,16 +488,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -513,7 +505,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -521,30 +513,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -844,37 +818,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -924,58 +898,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -992,13 +966,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1033,13 +1007,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1074,13 +1048,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1115,13 +1089,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1156,13 +1130,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1200,13 +1174,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1241,13 +1215,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1282,13 +1256,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1320,13 +1294,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1361,13 +1335,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1402,13 +1376,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1440,13 +1414,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1478,13 +1452,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1519,13 +1493,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1560,13 +1534,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1601,13 +1575,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1642,13 +1616,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1683,13 +1657,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1741,13 +1715,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>86</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1782,13 +1756,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>87</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1826,13 +1800,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>88</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1870,13 +1844,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>88</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1914,13 +1888,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1955,13 +1929,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>89</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -1996,13 +1970,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>90</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2037,13 +2011,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>91</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2078,13 +2052,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2176,13 +2150,13 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46106</v>
       </c>
       <c r="I33">
@@ -2214,13 +2188,13 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
         <v>92</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46233</v>
       </c>
       <c r="I34">
@@ -2253,19 +2227,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>127</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>128</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>129</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>130</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (24/08/2026 10:51)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="153">
   <si>
     <t>numero_contrato</t>
   </si>
@@ -280,6 +280,9 @@
     <t>2025NE001065, 2026NE000330</t>
   </si>
   <si>
+    <t>2026NE000388</t>
+  </si>
+  <si>
     <t>2025NE000559</t>
   </si>
   <si>
@@ -397,12 +400,12 @@
     <t>Pago</t>
   </si>
   <si>
+    <t>Faturado, aguardando pagamento</t>
+  </si>
+  <si>
     <t>Pendente</t>
   </si>
   <si>
-    <t>Faturado, aguardando pagamento</t>
-  </si>
-  <si>
     <t>numero_empenho</t>
   </si>
   <si>
@@ -458,9 +461,6 @@
   </si>
   <si>
     <t>2026NE000330</t>
-  </si>
-  <si>
-    <t>2026NE000388</t>
   </si>
   <si>
     <t>2026NE000748</t>
@@ -488,8 +488,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -505,7 +513,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -513,12 +521,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -818,37 +844,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -898,58 +924,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -966,29 +992,29 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
         <v>748504.24</v>
       </c>
       <c r="J2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="K2">
         <v>748504.24</v>
       </c>
       <c r="M2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P2">
         <v>881914.1800000001</v>
@@ -1007,29 +1033,29 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
         <v>1110378.24</v>
       </c>
       <c r="J3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K3">
         <v>1110378.24</v>
       </c>
       <c r="M3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P3">
         <v>2634000</v>
@@ -1048,29 +1074,29 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
         <v>974557.12</v>
       </c>
       <c r="J4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K4">
         <v>974557.12</v>
       </c>
       <c r="M4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P4">
         <v>1686034.96</v>
@@ -1089,29 +1115,29 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
         <v>1402001.34</v>
       </c>
       <c r="J5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="K5">
         <v>1402001.34</v>
       </c>
       <c r="M5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P5">
         <v>1600334.09</v>
@@ -1130,29 +1156,29 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
         <v>1223702.3</v>
       </c>
       <c r="J6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K6">
         <v>1223702.3</v>
       </c>
       <c r="M6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O6">
         <v>0.02</v>
@@ -1174,29 +1200,29 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
         <v>1011677.95</v>
       </c>
       <c r="J7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K7">
         <v>1011677.95</v>
       </c>
       <c r="M7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P7">
         <v>2568571.48</v>
@@ -1215,29 +1241,29 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
         <v>896744.0600000001</v>
       </c>
       <c r="J8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="K8">
         <v>896744.0600000001</v>
       </c>
       <c r="M8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P8">
         <v>968237.39</v>
@@ -1256,29 +1282,29 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
         <v>919329.0600000001</v>
       </c>
       <c r="J9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="K9">
         <v>919329.0600000001</v>
       </c>
       <c r="M9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P9">
         <v>1947932.74</v>
@@ -1294,29 +1320,29 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
         <v>1157009.26</v>
       </c>
       <c r="J10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="K10">
         <v>1157009.26</v>
       </c>
       <c r="M10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P10">
         <v>3105605.8</v>
@@ -1335,29 +1361,29 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
         <v>1214597.952</v>
       </c>
       <c r="J11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K11">
         <v>1214597.952</v>
       </c>
       <c r="M11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N11" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P11">
         <v>2096487.74</v>
@@ -1376,29 +1402,29 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
         <v>967082.09</v>
       </c>
       <c r="J12" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="K12">
         <v>967082.09</v>
       </c>
       <c r="M12" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N12" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P12">
         <v>3522444.13</v>
@@ -1414,29 +1440,29 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
         <v>719561.08</v>
       </c>
       <c r="J13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K13">
         <v>719561.08</v>
       </c>
       <c r="M13" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N13" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P13">
         <v>1500000</v>
@@ -1452,29 +1478,29 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
         <v>885881.08</v>
       </c>
       <c r="J14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K14">
         <v>885881.08</v>
       </c>
       <c r="M14" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N14" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O14">
         <v>34065.36</v>
@@ -1493,29 +1519,29 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
         <v>1350542.52</v>
       </c>
       <c r="J15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="K15">
         <v>1350542.52</v>
       </c>
       <c r="M15" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N15" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O15">
         <v>0.01</v>
@@ -1534,29 +1560,29 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
         <v>1108954.435833333</v>
       </c>
       <c r="J16" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K16">
         <v>1108954.435833333</v>
       </c>
       <c r="M16" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N16" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O16">
         <v>0.01</v>
@@ -1575,29 +1601,29 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
         <v>218206.1</v>
       </c>
       <c r="J17" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="K17">
         <v>218206.1</v>
       </c>
       <c r="M17" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N17" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O17">
         <v>0.01</v>
@@ -1616,29 +1642,29 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
         <v>1549250.84</v>
       </c>
       <c r="J18" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="K18">
         <v>1549250.84</v>
       </c>
       <c r="M18" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N18" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O18">
         <v>0.01</v>
@@ -1657,29 +1683,29 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
         <v>1340865.98</v>
       </c>
       <c r="J19" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K19">
         <v>1340865.98</v>
       </c>
       <c r="M19" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N19" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O19">
         <v>927618.61</v>
@@ -1695,14 +1721,32 @@
       <c r="B20" t="s">
         <v>52</v>
       </c>
-      <c r="L20">
+      <c r="D20">
+        <v>49</v>
+      </c>
+      <c r="E20" s="2">
+        <v>46252</v>
+      </c>
+      <c r="F20" t="s">
+        <v>86</v>
+      </c>
+      <c r="H20" s="2">
+        <v>46284</v>
+      </c>
+      <c r="K20">
         <v>1629834.48</v>
       </c>
       <c r="M20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="N20" t="s">
-        <v>125</v>
+        <v>126</v>
+      </c>
+      <c r="O20">
+        <v>282458.04</v>
+      </c>
+      <c r="P20">
+        <v>1629834.48</v>
       </c>
     </row>
     <row r="21" spans="1:16">
@@ -1715,29 +1759,29 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
-        <v>86</v>
-      </c>
-      <c r="H21" s="1">
+        <v>87</v>
+      </c>
+      <c r="H21" s="2">
         <v>45834</v>
       </c>
       <c r="I21">
         <v>188246.17</v>
       </c>
       <c r="J21" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="K21">
         <v>188246.17</v>
       </c>
       <c r="M21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N21" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P21">
         <v>211614.23</v>
@@ -1756,29 +1800,29 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
-        <v>87</v>
-      </c>
-      <c r="H22" s="1">
+        <v>88</v>
+      </c>
+      <c r="H22" s="2">
         <v>45955</v>
       </c>
       <c r="I22">
         <v>112720.77</v>
       </c>
       <c r="J22" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K22">
         <v>112720.77</v>
       </c>
       <c r="M22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N22" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O22">
         <v>0.01</v>
@@ -1800,29 +1844,29 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
-        <v>88</v>
-      </c>
-      <c r="H23" s="1">
+        <v>89</v>
+      </c>
+      <c r="H23" s="2">
         <v>45939</v>
       </c>
       <c r="I23">
         <v>378307.61</v>
       </c>
       <c r="J23" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K23">
         <v>378307.61</v>
       </c>
       <c r="M23" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N23" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O23">
         <v>0.01</v>
@@ -1844,29 +1888,29 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
-        <v>88</v>
-      </c>
-      <c r="H24" s="1">
+        <v>89</v>
+      </c>
+      <c r="H24" s="2">
         <v>45941</v>
       </c>
       <c r="I24">
         <v>3315.047100000025</v>
       </c>
       <c r="J24" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K24">
         <v>3315.04710000003</v>
       </c>
       <c r="M24" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N24" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O24">
         <v>0.01</v>
@@ -1888,29 +1932,29 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45935</v>
       </c>
       <c r="I25">
         <v>198332.75</v>
       </c>
       <c r="J25" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K25">
         <v>198332.75</v>
       </c>
       <c r="M25" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N25" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P25">
         <v>1600334.09</v>
@@ -1929,29 +1973,29 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
-        <v>89</v>
-      </c>
-      <c r="H26" s="1">
+        <v>90</v>
+      </c>
+      <c r="H26" s="2">
         <v>46066</v>
       </c>
       <c r="I26">
         <v>1528.62</v>
       </c>
       <c r="J26" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K26">
         <v>1528.62</v>
       </c>
       <c r="M26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N26" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P26">
         <v>1157673.06</v>
@@ -1970,29 +2014,29 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
-        <v>90</v>
-      </c>
-      <c r="H27" s="1">
+        <v>91</v>
+      </c>
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
         <v>38718.58</v>
       </c>
       <c r="J27" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K27">
         <v>38718.58</v>
       </c>
       <c r="M27" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P27">
         <v>63746.85</v>
@@ -2011,29 +2055,29 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
-        <v>91</v>
-      </c>
-      <c r="H28" s="1">
+        <v>92</v>
+      </c>
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
         <v>133124.11</v>
       </c>
       <c r="J28" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K28">
         <v>133124.11</v>
       </c>
       <c r="M28" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N28" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P28">
         <v>1000001.64</v>
@@ -2052,29 +2096,29 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46075</v>
       </c>
       <c r="I29">
         <v>11372.9</v>
       </c>
       <c r="J29" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K29">
         <v>11372.9</v>
       </c>
       <c r="M29" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N29" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P29">
         <v>1500000</v>
@@ -2088,16 +2132,16 @@
         <v>62</v>
       </c>
       <c r="G30" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L30">
         <v>15854.78</v>
       </c>
       <c r="M30" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N30" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="31" spans="1:16">
@@ -2108,16 +2152,16 @@
         <v>63</v>
       </c>
       <c r="G31" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L31">
         <v>42229.72325</v>
       </c>
       <c r="M31" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N31" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="32" spans="1:16">
@@ -2128,16 +2172,16 @@
         <v>64</v>
       </c>
       <c r="G32" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L32">
         <v>48857.39550000001</v>
       </c>
       <c r="M32" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N32" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="33" spans="1:16">
@@ -2150,29 +2194,29 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46106</v>
       </c>
       <c r="I33">
         <v>27801.11</v>
       </c>
       <c r="J33" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K33">
         <v>27801.11</v>
       </c>
       <c r="M33" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N33" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P33">
         <v>1500000</v>
@@ -2188,26 +2232,26 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
-        <v>92</v>
-      </c>
-      <c r="H34" s="1">
+        <v>93</v>
+      </c>
+      <c r="H34" s="2">
         <v>46233</v>
       </c>
       <c r="I34">
         <v>58868.35</v>
       </c>
       <c r="J34" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K34">
         <v>58868.35</v>
       </c>
       <c r="M34" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N34" t="s">
         <v>126</v>
@@ -2227,25 +2271,25 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
-        <v>127</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
-        <v>128</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="C1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="E1" t="s">
+      <c r="D1" s="1" t="s">
         <v>130</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B2">
         <v>52250.04</v>
@@ -2256,7 +2300,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B3">
         <v>881914.1800000001</v>
@@ -2267,7 +2311,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B4">
         <v>750000</v>
@@ -2278,7 +2322,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B5">
         <v>949835.78</v>
@@ -2289,7 +2333,7 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B6">
         <v>524584.95</v>
@@ -2300,7 +2344,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B7">
         <v>211614.23</v>
@@ -2311,7 +2355,7 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B8">
         <v>2391157.41</v>
@@ -2322,7 +2366,7 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B9">
         <v>618154.38</v>
@@ -2344,7 +2388,7 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B11">
         <v>2364771.07</v>
@@ -2366,7 +2410,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B13">
         <v>1011677.95</v>
@@ -2377,7 +2421,7 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B14">
         <v>1580293.02</v>
@@ -2388,7 +2432,7 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -2399,7 +2443,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B16">
         <v>63746.85</v>
@@ -2410,7 +2454,7 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B17">
         <v>947931.1</v>
@@ -2421,7 +2465,7 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B18">
         <v>259790.57</v>
@@ -2432,7 +2476,7 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B19">
         <v>170479.3</v>
@@ -2454,7 +2498,7 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B21">
         <v>1000001.64</v>
@@ -2465,7 +2509,7 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B22">
         <v>68405.66</v>
@@ -2476,7 +2520,7 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B23">
         <v>1157673.06</v>
@@ -2487,7 +2531,7 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B24">
         <v>34065.36</v>
@@ -2498,7 +2542,7 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B25">
         <v>843261.89</v>
@@ -2509,13 +2553,13 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>146</v>
+        <v>86</v>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>1629834.48</v>
       </c>
       <c r="C26">
-        <v>1912292.52</v>
+        <v>282458.04</v>
       </c>
     </row>
     <row r="27" spans="1:3">

</xml_diff>

<commit_message>
Corrige bug real: extrair_empenhos() pulava o 1º empenho da aba EMPENHOS
Achado pelo Wallace ao pedir pra olhar a inconsistência recorrente
'Empenho 2025NE000005 não encontrado na aba EMPENHOS' (aparecia em toda
atualização de Pagamentos desde julho, sempre pra referência JUN/25).

Causa: extrair_empenhos() lia a aba a partir da linha 4 (min_row=4),
assumindo que as 3 primeiras linhas eram cabeçalho/vazias. Na prática, a
linha 1 é vazia, a linha 2 só tem uma data solta na coluna A (parece um
'última atualização' mal posicionado na planilha original), mas a linha 3
já é o primeiro empenho de verdade (2025NE000005) — sempre pulado.

Corrigido min_row=4 -> min_row=3. Resultado: 32 empenhos reconhecidos (era
31), inconsistência 'não encontrado' para esse empenho desaparece (9 -> 8
inconsistências nessa extração).
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="154">
   <si>
     <t>numero_contrato</t>
   </si>
@@ -416,6 +416,9 @@
   </si>
   <si>
     <t>justificativa</t>
+  </si>
+  <si>
+    <t>2025NE000005</t>
   </si>
   <si>
     <t>2025NE000367</t>
@@ -1184,7 +1187,7 @@
         <v>0.02</v>
       </c>
       <c r="P6">
-        <v>3533896.74</v>
+        <v>3534896.74</v>
       </c>
     </row>
     <row r="7" spans="1:18">
@@ -2267,7 +2270,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2292,7 +2295,7 @@
         <v>132</v>
       </c>
       <c r="B2">
-        <v>52250.04</v>
+        <v>1000</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -2303,7 +2306,7 @@
         <v>133</v>
       </c>
       <c r="B3">
-        <v>881914.1800000001</v>
+        <v>52250.04</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -2314,7 +2317,7 @@
         <v>134</v>
       </c>
       <c r="B4">
-        <v>750000</v>
+        <v>881914.1800000001</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -2325,7 +2328,7 @@
         <v>135</v>
       </c>
       <c r="B5">
-        <v>949835.78</v>
+        <v>750000</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -2336,7 +2339,7 @@
         <v>136</v>
       </c>
       <c r="B6">
-        <v>524584.95</v>
+        <v>949835.78</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -2344,10 +2347,10 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>87</v>
+        <v>137</v>
       </c>
       <c r="B7">
-        <v>211614.23</v>
+        <v>524584.95</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -2355,21 +2358,21 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B8">
-        <v>2391157.41</v>
+        <v>211614.23</v>
       </c>
       <c r="C8">
-        <v>0.01</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>137</v>
+        <v>89</v>
       </c>
       <c r="B9">
-        <v>618154.38</v>
+        <v>2391157.41</v>
       </c>
       <c r="C9">
         <v>0.01</v>
@@ -2377,21 +2380,21 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>138</v>
       </c>
       <c r="B10">
-        <v>1600334.09</v>
+        <v>618154.38</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="B11">
-        <v>2364771.07</v>
+        <v>1600334.09</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -2399,10 +2402,10 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>76</v>
+        <v>93</v>
       </c>
       <c r="B12">
-        <v>968237.39</v>
+        <v>2364771.07</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -2410,10 +2413,10 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>138</v>
+        <v>76</v>
       </c>
       <c r="B13">
-        <v>1011677.95</v>
+        <v>968237.39</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -2424,7 +2427,7 @@
         <v>139</v>
       </c>
       <c r="B14">
-        <v>1580293.02</v>
+        <v>1011677.95</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -2435,29 +2438,29 @@
         <v>140</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>1580293.02</v>
       </c>
       <c r="C15">
-        <v>34065.36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>141</v>
       </c>
       <c r="B16">
-        <v>63746.85</v>
+        <v>0</v>
       </c>
       <c r="C16">
-        <v>0</v>
+        <v>34065.36</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>141</v>
+        <v>91</v>
       </c>
       <c r="B17">
-        <v>947931.1</v>
+        <v>63746.85</v>
       </c>
       <c r="C17">
         <v>0</v>
@@ -2468,7 +2471,7 @@
         <v>142</v>
       </c>
       <c r="B18">
-        <v>259790.57</v>
+        <v>947931.1</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -2479,7 +2482,7 @@
         <v>143</v>
       </c>
       <c r="B19">
-        <v>170479.3</v>
+        <v>259790.57</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -2487,10 +2490,10 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>81</v>
+        <v>144</v>
       </c>
       <c r="B20">
-        <v>1500000</v>
+        <v>170479.3</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -2498,10 +2501,10 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="B21">
-        <v>1000001.64</v>
+        <v>1500000</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -2509,10 +2512,10 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>144</v>
+        <v>92</v>
       </c>
       <c r="B22">
-        <v>68405.66</v>
+        <v>1000001.64</v>
       </c>
       <c r="C22">
         <v>0</v>
@@ -2520,10 +2523,10 @@
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>90</v>
+        <v>145</v>
       </c>
       <c r="B23">
-        <v>1157673.06</v>
+        <v>68405.66</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -2531,10 +2534,10 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>145</v>
+        <v>90</v>
       </c>
       <c r="B24">
-        <v>34065.36</v>
+        <v>1157673.06</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -2545,32 +2548,32 @@
         <v>146</v>
       </c>
       <c r="B25">
-        <v>843261.89</v>
+        <v>34065.36</v>
       </c>
       <c r="C25">
-        <v>927618.61</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>86</v>
+        <v>147</v>
       </c>
       <c r="B26">
-        <v>1629834.48</v>
+        <v>843261.89</v>
       </c>
       <c r="C26">
-        <v>282458.04</v>
+        <v>927618.61</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>147</v>
+        <v>86</v>
       </c>
       <c r="B27">
-        <v>0</v>
+        <v>1629834.48</v>
       </c>
       <c r="C27">
-        <v>1496713.48</v>
+        <v>282458.04</v>
       </c>
     </row>
     <row r="28" spans="1:3">
@@ -2581,7 +2584,7 @@
         <v>0</v>
       </c>
       <c r="C28">
-        <v>624166.14</v>
+        <v>1496713.48</v>
       </c>
     </row>
     <row r="29" spans="1:3">
@@ -2592,7 +2595,7 @@
         <v>0</v>
       </c>
       <c r="C29">
-        <v>18462.36</v>
+        <v>624166.14</v>
       </c>
     </row>
     <row r="30" spans="1:3">
@@ -2603,7 +2606,7 @@
         <v>0</v>
       </c>
       <c r="C30">
-        <v>1530656.62</v>
+        <v>18462.36</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -2614,7 +2617,7 @@
         <v>0</v>
       </c>
       <c r="C31">
-        <v>173846.38</v>
+        <v>1530656.62</v>
       </c>
     </row>
     <row r="32" spans="1:3">
@@ -2625,6 +2628,17 @@
         <v>0</v>
       </c>
       <c r="C32">
+        <v>173846.38</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" t="s">
+        <v>153</v>
+      </c>
+      <c r="B33">
+        <v>0</v>
+      </c>
+      <c r="C33">
         <v>236343.68</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (24/08/2026 18:37)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -491,16 +491,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -516,7 +508,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -524,30 +516,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -847,37 +821,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -927,58 +901,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -995,13 +969,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1036,13 +1010,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1077,13 +1051,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1118,13 +1092,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1159,13 +1133,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1203,13 +1177,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1244,13 +1218,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1285,13 +1259,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1323,13 +1297,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1364,13 +1338,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1405,13 +1379,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1443,13 +1417,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1481,13 +1455,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1522,13 +1496,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1563,13 +1537,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1604,13 +1578,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1645,13 +1619,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1686,13 +1660,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1727,13 +1701,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>86</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1762,13 +1736,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>87</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1803,13 +1777,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>88</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1847,13 +1821,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>89</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1891,13 +1865,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>89</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1935,13 +1909,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1976,13 +1950,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>90</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -2017,13 +1991,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>91</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2058,13 +2032,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>92</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2099,13 +2073,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2197,13 +2171,13 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46106</v>
       </c>
       <c r="I33">
@@ -2235,13 +2209,13 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
         <v>93</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46233</v>
       </c>
       <c r="I34">
@@ -2274,19 +2248,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>128</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>129</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>130</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>131</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (25/08/2026 08:30)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -491,8 +491,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -508,7 +516,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -516,12 +524,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -821,37 +847,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -901,58 +927,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -969,13 +995,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1010,13 +1036,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1051,13 +1077,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1092,13 +1118,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1133,13 +1159,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1177,13 +1203,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1218,13 +1244,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1259,13 +1285,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1297,13 +1323,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1338,13 +1364,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1379,13 +1405,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1417,13 +1443,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1455,13 +1481,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1496,13 +1522,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1537,13 +1563,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1578,13 +1604,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1619,13 +1645,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1660,13 +1686,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1701,13 +1727,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>86</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1736,13 +1762,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>87</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1777,13 +1803,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>88</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1821,13 +1847,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>89</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1865,13 +1891,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>89</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1909,13 +1935,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1950,13 +1976,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>90</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -1991,13 +2017,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>91</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2032,13 +2058,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>92</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2073,13 +2099,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2171,13 +2197,13 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46106</v>
       </c>
       <c r="I33">
@@ -2209,13 +2235,13 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
         <v>93</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46233</v>
       </c>
       <c r="I34">
@@ -2248,19 +2274,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>131</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (01/09/2026 11:15)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -491,8 +491,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -508,7 +516,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -516,12 +524,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -821,37 +847,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -901,58 +927,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -969,13 +995,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1010,13 +1036,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1051,13 +1077,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1092,13 +1118,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1133,13 +1159,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1177,13 +1203,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1218,13 +1244,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1259,13 +1285,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1297,13 +1323,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1338,13 +1364,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1379,13 +1405,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1417,13 +1443,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1455,13 +1481,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1496,13 +1522,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1537,13 +1563,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1578,13 +1604,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1619,13 +1645,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1660,13 +1686,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1701,13 +1727,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>86</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1736,13 +1762,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>87</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1777,13 +1803,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>88</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1821,13 +1847,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>89</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1865,13 +1891,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>89</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1909,13 +1935,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1950,13 +1976,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>90</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -1991,13 +2017,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>91</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2032,13 +2058,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>92</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2073,13 +2099,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2171,13 +2197,13 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46106</v>
       </c>
       <c r="I33">
@@ -2209,13 +2235,13 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
         <v>93</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46233</v>
       </c>
       <c r="I34">
@@ -2248,19 +2274,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>131</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (01/09/2026 12:27)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -491,16 +491,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -516,7 +508,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -524,30 +516,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -847,37 +821,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -927,58 +901,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -995,13 +969,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1036,13 +1010,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1077,13 +1051,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1118,13 +1092,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1159,13 +1133,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1203,13 +1177,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1244,13 +1218,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1285,13 +1259,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1323,13 +1297,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1364,13 +1338,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1405,13 +1379,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1443,13 +1417,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1481,13 +1455,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1522,13 +1496,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1563,13 +1537,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1604,13 +1578,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1645,13 +1619,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1686,13 +1660,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1727,13 +1701,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>86</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1762,13 +1736,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>87</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1803,13 +1777,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>88</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1847,13 +1821,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>89</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1891,13 +1865,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>89</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1935,13 +1909,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1976,13 +1950,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>90</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -2017,13 +1991,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>91</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2058,13 +2032,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>92</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2099,13 +2073,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2197,13 +2171,13 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46106</v>
       </c>
       <c r="I33">
@@ -2235,13 +2209,13 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
         <v>93</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46233</v>
       </c>
       <c r="I34">
@@ -2274,19 +2248,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>128</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>129</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>130</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>131</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (02/09/2026 09:38)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -491,8 +491,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -508,7 +516,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -516,12 +524,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -821,37 +847,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -901,58 +927,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -969,13 +995,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1010,13 +1036,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1051,13 +1077,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1092,13 +1118,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1133,13 +1159,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1177,13 +1203,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1218,13 +1244,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1259,13 +1285,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1297,13 +1323,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1338,13 +1364,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1379,13 +1405,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1417,13 +1443,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1455,13 +1481,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1496,13 +1522,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1537,13 +1563,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1578,13 +1604,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1619,13 +1645,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1660,13 +1686,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1701,13 +1727,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>86</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1736,13 +1762,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>87</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1777,13 +1803,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>88</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1821,13 +1847,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>89</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1865,13 +1891,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>89</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1909,13 +1935,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1950,13 +1976,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>90</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -1991,13 +2017,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>91</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2032,13 +2058,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>92</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2073,13 +2099,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2171,13 +2197,13 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46106</v>
       </c>
       <c r="I33">
@@ -2209,13 +2235,13 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
         <v>93</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46233</v>
       </c>
       <c r="I34">
@@ -2248,19 +2274,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>131</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (02/09/2026 12:04)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -491,16 +491,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -516,7 +508,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -524,30 +516,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -847,37 +821,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -927,58 +901,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -995,13 +969,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1036,13 +1010,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1077,13 +1051,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1118,13 +1092,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1159,13 +1133,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1203,13 +1177,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1244,13 +1218,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1285,13 +1259,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1323,13 +1297,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1364,13 +1338,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1405,13 +1379,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1443,13 +1417,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1481,13 +1455,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1522,13 +1496,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1563,13 +1537,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1604,13 +1578,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1645,13 +1619,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1686,13 +1660,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1727,13 +1701,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>86</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1762,13 +1736,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>87</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1803,13 +1777,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>88</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1847,13 +1821,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>89</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1891,13 +1865,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>89</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1935,13 +1909,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1976,13 +1950,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>90</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -2017,13 +1991,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>91</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2058,13 +2032,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>92</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2099,13 +2073,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2197,13 +2171,13 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46106</v>
       </c>
       <c r="I33">
@@ -2235,13 +2209,13 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
         <v>93</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46233</v>
       </c>
       <c r="I34">
@@ -2274,19 +2248,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>128</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>129</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>130</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>131</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (04/09/2026 11:55)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -491,16 +491,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -516,7 +508,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -524,30 +516,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -847,37 +821,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -927,58 +901,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -995,13 +969,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1036,13 +1010,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1077,13 +1051,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1118,13 +1092,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1159,13 +1133,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1203,13 +1177,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1244,13 +1218,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1285,13 +1259,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1323,13 +1297,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1364,13 +1338,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1405,13 +1379,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1443,13 +1417,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1481,13 +1455,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1522,13 +1496,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1563,13 +1537,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1604,13 +1578,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1645,13 +1619,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1686,13 +1660,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1727,13 +1701,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>86</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1762,13 +1736,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>87</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1803,13 +1777,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>88</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1847,13 +1821,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>89</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1891,13 +1865,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>89</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1935,13 +1909,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1976,13 +1950,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>90</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -2017,13 +1991,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>91</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2058,13 +2032,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>92</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2099,13 +2073,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2197,13 +2171,13 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46106</v>
       </c>
       <c r="I33">
@@ -2235,13 +2209,13 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
         <v>93</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46233</v>
       </c>
       <c r="I34">
@@ -2274,19 +2248,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>128</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>129</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>130</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>131</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (08/09/2026 08:22)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -491,8 +491,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -508,7 +516,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -516,12 +524,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -821,37 +847,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -901,58 +927,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -969,13 +995,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="2">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2" s="2">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1010,13 +1036,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="2">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3" s="2">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1051,13 +1077,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="2">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4" s="2">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1092,13 +1118,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="2">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="1">
+      <c r="H5" s="2">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1133,13 +1159,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="2">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="1">
+      <c r="H6" s="2">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1177,13 +1203,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="2">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="1">
+      <c r="H7" s="2">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1218,13 +1244,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="2">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="1">
+      <c r="H8" s="2">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1259,13 +1285,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="2">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="1">
+      <c r="H9" s="2">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1297,13 +1323,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="2">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="1">
+      <c r="H10" s="2">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1338,13 +1364,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="2">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="1">
+      <c r="H11" s="2">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1379,13 +1405,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="2">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="1">
+      <c r="H12" s="2">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1417,13 +1443,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="2">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="1">
+      <c r="H13" s="2">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1455,13 +1481,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="1">
+      <c r="H14" s="2">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1496,13 +1522,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="2">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="1">
+      <c r="H15" s="2">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1537,13 +1563,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="2">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="1">
+      <c r="H16" s="2">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1578,13 +1604,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="2">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="1">
+      <c r="H17" s="2">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1619,13 +1645,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="2">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="1">
+      <c r="H18" s="2">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1660,13 +1686,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="2">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="1">
+      <c r="H19" s="2">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1701,13 +1727,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="2">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>86</v>
       </c>
-      <c r="H20" s="1">
+      <c r="H20" s="2">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1736,13 +1762,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="2">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>87</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="2">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1777,13 +1803,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="2">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>88</v>
       </c>
-      <c r="H22" s="1">
+      <c r="H22" s="2">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1821,13 +1847,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="2">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>89</v>
       </c>
-      <c r="H23" s="1">
+      <c r="H23" s="2">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1865,13 +1891,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="2">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>89</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="2">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1909,13 +1935,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="2">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="2">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1950,13 +1976,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="2">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>90</v>
       </c>
-      <c r="H26" s="1">
+      <c r="H26" s="2">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -1991,13 +2017,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27" s="2">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>91</v>
       </c>
-      <c r="H27" s="1">
+      <c r="H27" s="2">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2032,13 +2058,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="2">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>92</v>
       </c>
-      <c r="H28" s="1">
+      <c r="H28" s="2">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2073,13 +2099,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="2">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="2">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2171,13 +2197,13 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33" s="2">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="1">
+      <c r="H33" s="2">
         <v>46106</v>
       </c>
       <c r="I33">
@@ -2209,13 +2235,13 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="2">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
         <v>93</v>
       </c>
-      <c r="H34" s="1">
+      <c r="H34" s="2">
         <v>46233</v>
       </c>
       <c r="I34">
@@ -2248,19 +2274,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>131</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: pagamentos (08/09/2026 12:03)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_pagamentos_tratada.xlsx
@@ -491,16 +491,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -516,7 +508,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -524,30 +516,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -847,37 +821,37 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -927,58 +901,58 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>21</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>26</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>27</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>28</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>29</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>31</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -995,13 +969,13 @@
       <c r="D2">
         <v>594</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>45740</v>
       </c>
       <c r="F2" t="s">
         <v>70</v>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="1">
         <v>45778</v>
       </c>
       <c r="I2">
@@ -1036,13 +1010,13 @@
       <c r="D3">
         <v>620</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>45775</v>
       </c>
       <c r="F3" t="s">
         <v>71</v>
       </c>
-      <c r="H3" s="2">
+      <c r="H3" s="1">
         <v>45806</v>
       </c>
       <c r="I3">
@@ -1077,13 +1051,13 @@
       <c r="D4">
         <v>634</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>45799</v>
       </c>
       <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="1">
         <v>45844</v>
       </c>
       <c r="I4">
@@ -1118,13 +1092,13 @@
       <c r="D5">
         <v>660</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>45856</v>
       </c>
       <c r="F5" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="1">
         <v>45891</v>
       </c>
       <c r="I5">
@@ -1159,13 +1133,13 @@
       <c r="D6">
         <v>661</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>45856</v>
       </c>
       <c r="F6" t="s">
         <v>74</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="1">
         <v>45891</v>
       </c>
       <c r="I6">
@@ -1203,13 +1177,13 @@
       <c r="D7">
         <v>688</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <v>45901</v>
       </c>
       <c r="F7" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="1">
         <v>45938</v>
       </c>
       <c r="I7">
@@ -1244,13 +1218,13 @@
       <c r="D8">
         <v>696</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>45923</v>
       </c>
       <c r="F8" t="s">
         <v>76</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="1">
         <v>45938</v>
       </c>
       <c r="I8">
@@ -1285,13 +1259,13 @@
       <c r="D9">
         <v>704</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>45957</v>
       </c>
       <c r="F9" t="s">
         <v>77</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="1">
         <v>46003</v>
       </c>
       <c r="I9">
@@ -1323,13 +1297,13 @@
       <c r="D10">
         <v>705</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>45972</v>
       </c>
       <c r="F10" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="1">
         <v>46016</v>
       </c>
       <c r="I10">
@@ -1364,13 +1338,13 @@
       <c r="D11">
         <v>728</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>46008</v>
       </c>
       <c r="F11" t="s">
         <v>79</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="1">
         <v>46040</v>
       </c>
       <c r="I11">
@@ -1405,13 +1379,13 @@
       <c r="D12">
         <v>278</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <v>46042</v>
       </c>
       <c r="F12" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="1">
         <v>46074</v>
       </c>
       <c r="I12">
@@ -1443,13 +1417,13 @@
       <c r="D13">
         <v>10</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <v>46078</v>
       </c>
       <c r="F13" t="s">
         <v>81</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="1">
         <v>46106</v>
       </c>
       <c r="I13">
@@ -1481,13 +1455,13 @@
       <c r="D14">
         <v>15</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <v>46094</v>
       </c>
       <c r="F14" t="s">
         <v>82</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="1">
         <v>46128</v>
       </c>
       <c r="I14">
@@ -1522,13 +1496,13 @@
       <c r="D15">
         <v>28</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <v>46128</v>
       </c>
       <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="1">
         <v>46164</v>
       </c>
       <c r="I15">
@@ -1563,13 +1537,13 @@
       <c r="D16">
         <v>33</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <v>46156</v>
       </c>
       <c r="F16" t="s">
         <v>84</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="1">
         <v>46191</v>
       </c>
       <c r="I16">
@@ -1604,13 +1578,13 @@
       <c r="D17">
         <v>29</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <v>46149</v>
       </c>
       <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="1">
         <v>46185</v>
       </c>
       <c r="I17">
@@ -1645,13 +1619,13 @@
       <c r="D18">
         <v>40</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <v>46156</v>
       </c>
       <c r="F18" t="s">
         <v>84</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="1">
         <v>46191</v>
       </c>
       <c r="I18">
@@ -1686,13 +1660,13 @@
       <c r="D19">
         <v>48</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <v>46230</v>
       </c>
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="1">
         <v>46262</v>
       </c>
       <c r="I19">
@@ -1727,13 +1701,13 @@
       <c r="D20">
         <v>49</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <v>46252</v>
       </c>
       <c r="F20" t="s">
         <v>86</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="1">
         <v>46284</v>
       </c>
       <c r="K20">
@@ -1762,13 +1736,13 @@
       <c r="D21">
         <v>402</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <v>45791</v>
       </c>
       <c r="F21" t="s">
         <v>87</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="1">
         <v>45834</v>
       </c>
       <c r="I21">
@@ -1803,13 +1777,13 @@
       <c r="D22">
         <v>447</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <v>45814</v>
       </c>
       <c r="F22" t="s">
         <v>88</v>
       </c>
-      <c r="H22" s="2">
+      <c r="H22" s="1">
         <v>45955</v>
       </c>
       <c r="I22">
@@ -1847,13 +1821,13 @@
       <c r="D23">
         <v>529</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <v>45853</v>
       </c>
       <c r="F23" t="s">
         <v>89</v>
       </c>
-      <c r="H23" s="2">
+      <c r="H23" s="1">
         <v>45939</v>
       </c>
       <c r="I23">
@@ -1891,13 +1865,13 @@
       <c r="D24">
         <v>691</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <v>45910</v>
       </c>
       <c r="F24" t="s">
         <v>89</v>
       </c>
-      <c r="H24" s="2">
+      <c r="H24" s="1">
         <v>45941</v>
       </c>
       <c r="I24">
@@ -1935,13 +1909,13 @@
       <c r="D25">
         <v>677</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="1">
         <v>45904</v>
       </c>
       <c r="F25" t="s">
         <v>73</v>
       </c>
-      <c r="H25" s="2">
+      <c r="H25" s="1">
         <v>45935</v>
       </c>
       <c r="I25">
@@ -1976,13 +1950,13 @@
       <c r="D26">
         <v>278</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26" s="1">
         <v>46008</v>
       </c>
       <c r="F26" t="s">
         <v>90</v>
       </c>
-      <c r="H26" s="2">
+      <c r="H26" s="1">
         <v>46066</v>
       </c>
       <c r="I26">
@@ -2017,13 +1991,13 @@
       <c r="D27">
         <v>748</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="1">
         <v>45930</v>
       </c>
       <c r="F27" t="s">
         <v>91</v>
       </c>
-      <c r="H27" s="2">
+      <c r="H27" s="1">
         <v>45935</v>
       </c>
       <c r="I27">
@@ -2058,13 +2032,13 @@
       <c r="D28">
         <v>822</v>
       </c>
-      <c r="E28" s="2">
+      <c r="E28" s="1">
         <v>45968</v>
       </c>
       <c r="F28" t="s">
         <v>92</v>
       </c>
-      <c r="H28" s="2">
+      <c r="H28" s="1">
         <v>45935</v>
       </c>
       <c r="I28">
@@ -2099,13 +2073,13 @@
       <c r="D29">
         <v>360</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="1">
         <v>46043</v>
       </c>
       <c r="F29" t="s">
         <v>81</v>
       </c>
-      <c r="H29" s="2">
+      <c r="H29" s="1">
         <v>46075</v>
       </c>
       <c r="I29">
@@ -2197,13 +2171,13 @@
       <c r="D33">
         <v>1465</v>
       </c>
-      <c r="E33" s="2">
+      <c r="E33" s="1">
         <v>46104</v>
       </c>
       <c r="F33" t="s">
         <v>81</v>
       </c>
-      <c r="H33" s="2">
+      <c r="H33" s="1">
         <v>46106</v>
       </c>
       <c r="I33">
@@ -2235,13 +2209,13 @@
       <c r="D34">
         <v>1882</v>
       </c>
-      <c r="E34" s="2">
+      <c r="E34" s="1">
         <v>46199</v>
       </c>
       <c r="F34" t="s">
         <v>93</v>
       </c>
-      <c r="H34" s="2">
+      <c r="H34" s="1">
         <v>46233</v>
       </c>
       <c r="I34">
@@ -2274,19 +2248,19 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>128</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>129</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>130</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>131</v>
       </c>
     </row>

</xml_diff>